<commit_message>
skill v0p4(optimized by AI) and rtm(gen in plan mode)
</commit_message>
<xml_diff>
--- a/RTM_AI_gen.xlsx
+++ b/RTM_AI_gen.xlsx
@@ -1548,7 +1548,7 @@
       </c>
       <c r="E6" s="31" t="inlineStr">
         <is>
-          <t>CHK_004</t>
+          <t>CHK_004, CHK_005</t>
         </is>
       </c>
       <c r="F6" s="31" t="inlineStr">
@@ -1582,7 +1582,7 @@
       </c>
       <c r="E7" s="31" t="inlineStr">
         <is>
-          <t>CHK_005</t>
+          <t>CHK_004</t>
         </is>
       </c>
       <c r="F7" s="31" t="inlineStr">
@@ -1616,7 +1616,7 @@
       </c>
       <c r="E8" s="31" t="inlineStr">
         <is>
-          <t>CHK_006</t>
+          <t>CHK_005, CHK_006</t>
         </is>
       </c>
       <c r="F8" s="31" t="inlineStr">
@@ -1650,7 +1650,7 @@
       </c>
       <c r="E9" s="31" t="inlineStr">
         <is>
-          <t>CHK_007</t>
+          <t>CHK_005</t>
         </is>
       </c>
       <c r="F9" s="31" t="inlineStr">
@@ -1684,7 +1684,7 @@
       </c>
       <c r="E10" s="31" t="inlineStr">
         <is>
-          <t>CHK_008</t>
+          <t>CHK_006</t>
         </is>
       </c>
       <c r="F10" s="31" t="inlineStr">
@@ -1718,7 +1718,7 @@
       </c>
       <c r="E11" s="31" t="inlineStr">
         <is>
-          <t>CHK_009</t>
+          <t>CHK_007</t>
         </is>
       </c>
       <c r="F11" s="31" t="inlineStr">
@@ -1752,7 +1752,7 @@
       </c>
       <c r="E12" s="31" t="inlineStr">
         <is>
-          <t>CHK_010</t>
+          <t>CHK_008</t>
         </is>
       </c>
       <c r="F12" s="31" t="inlineStr">
@@ -1786,7 +1786,7 @@
       </c>
       <c r="E13" s="31" t="inlineStr">
         <is>
-          <t>CHK_011</t>
+          <t>CHK_009</t>
         </is>
       </c>
       <c r="F13" s="31" t="inlineStr">
@@ -1820,7 +1820,7 @@
       </c>
       <c r="E14" s="31" t="inlineStr">
         <is>
-          <t>CHK_012</t>
+          <t>CHK_010</t>
         </is>
       </c>
       <c r="F14" s="31" t="inlineStr">
@@ -1854,7 +1854,7 @@
       </c>
       <c r="E15" s="31" t="inlineStr">
         <is>
-          <t>CHK_013</t>
+          <t>CHK_011</t>
         </is>
       </c>
       <c r="F15" s="31" t="inlineStr">
@@ -1888,7 +1888,7 @@
       </c>
       <c r="E16" s="31" t="inlineStr">
         <is>
-          <t>CHK_014</t>
+          <t>CHK_012</t>
         </is>
       </c>
       <c r="F16" s="31" t="inlineStr">
@@ -1922,7 +1922,7 @@
       </c>
       <c r="E17" s="31" t="inlineStr">
         <is>
-          <t>CHK_015</t>
+          <t>CHK_013</t>
         </is>
       </c>
       <c r="F17" s="31" t="inlineStr">
@@ -1956,7 +1956,7 @@
       </c>
       <c r="E18" s="31" t="inlineStr">
         <is>
-          <t>CHK_016</t>
+          <t>CHK_014</t>
         </is>
       </c>
       <c r="F18" s="31" t="inlineStr">
@@ -1973,9 +1973,6 @@
       <c r="E19" s="31" t="n"/>
       <c r="F19" s="31" t="n"/>
     </row>
-    <row r="20"/>
-    <row r="21"/>
-    <row r="22"/>
     <row r="23">
       <c r="A23" s="23" t="inlineStr">
         <is>
@@ -2144,8 +2141,9 @@
       </c>
       <c r="C3" s="6" t="inlineStr">
         <is>
-          <t>1. 检查频率值是否正确：连续采集时钟上升沿和下降沿并计算实际频率/周期，判断是否处于目标频率的允许误差范围内（±1%）；
-2. 检查时钟稳定性：通过连续采样周期，对比相邻两个周期的频率偏差是否在3%内。</t>
+          <t xml:space="preserve">1.检查频率值是否正确：连续采集时钟上升沿和下降沿并计算实际频率/周期，判断是否处于目标频率的允许误差范围内（±1%）；
+2.检查时钟稳定性：通过连续采样周期，对比相邻两个周期的频率偏差是否在3%内。
+</t>
         </is>
       </c>
       <c r="D3" s="4" t="n"/>
@@ -2163,13 +2161,11 @@
       </c>
       <c r="C4" s="17" t="inlineStr">
         <is>
-          <t>在rst_ni释放后，检查以下复位状态：
-1. 状态机状态：确认fsm_state == IDLE；
-2. CTRL寄存器默认值：CTRL.EN=0，CTRL.LANE_MODE=2'b00（1-bit模式），CTRL.SOFT_RST=0；
-3. STATUS寄存器：STATUS[7:0]=0x00，所有sticky位清零；
-4. LAST_ERR寄存器：LAST_ERR[7:0]=0x00；
-5. 协议上下文：rx_shift_reg=0，tx_shift_reg=0，opcode_reg=0，addr_reg=0，wdata_reg=0；
-6. 错误状态寄存器清零。</t>
+          <t>1. 检查复位后状态机状态：内部fsm_state信号 == IDLE(0x00)；
+2. 检查CTRL寄存器默认值：通过RD_CSR(addr=0x04)读取，期望bit[0]=0(EN=0), bit[2:1]=00(LANE_MODE=1-bit)；
+3. 检查STATUS寄存器：RD_CSR(addr=0x08)返回0x00；
+4. 检查LAST_ERR寄存器：RD_CSR(addr=0x0C)返回0x00；
+5. 检查AHB接口：htrans_o==2'b00, hwrite_o==0, haddr_o==0。</t>
         </is>
       </c>
       <c r="D4" s="4" t="n"/>
@@ -2182,17 +2178,16 @@
       </c>
       <c r="B5" s="31" t="inlineStr">
         <is>
-          <t>csr_access_check</t>
+          <t>csr_rw_check</t>
         </is>
       </c>
       <c r="C5" s="6" t="inlineStr">
         <is>
-          <t>检查CSR读写正确性：
-1. VERSION寄存器：RD_CSR读取地址0x00，验证返回值符合预期版本号（如0x0001_0001）；
-2. CTRL寄存器：WR_CSR写地址0x04，配置EN/LANE_MODE/SOFT_RST字段，RD_CSR读回验证写入值正确；
-3. STATUS寄存器：RD_CSR读取地址0x08，验证BUSY/RESP_VALID/CMD_ERR/BUS_ERR/FRAME_ERR/IN_TEST_MODE/OUT_EN字段反映正确状态；
-4. LAST_ERR寄存器：RD_CSR读取地址0x0C，验证最近错误码记录正确；
-5. 非法CSR地址（非0x00/0x04/0x08/0x0C）访问返回STS_BAD_REG(0x02)。</t>
+          <t>1. 检查VERSION寄存器(addr=0x00)只读：WR_CSR写入0xFF后RD_CSR读回原值；
+2. 检查CTRL寄存器(addr=0x04)读写：WR_CSR(0x04, 0x03)后RD_CSR读回0x03；
+3. 检查STATUS寄存器(addr=0x08)只读；
+4. 检查LAST_ERR寄存器(addr=0x0C)只读；
+5. 检查非法地址：RD_CSR(0x10)返回status_code=0x02。</t>
         </is>
       </c>
       <c r="D5" s="4" t="n"/>
@@ -2205,16 +2200,15 @@
       </c>
       <c r="B6" s="31" t="inlineStr">
         <is>
-          <t>test_mode_check</t>
+          <t>lane_mode_check</t>
         </is>
       </c>
       <c r="C6" s="6" t="inlineStr">
         <is>
-          <t>检查测试模式工作条件：
-1. test_mode_i=1且CTRL.EN=1时，模块允许执行功能命令（WR_CSR/RD_CSR/AHB_WR32/AHB_RD32）；
-2. test_mode_i=0时发送命令，返回STS_NOT_IN_TEST(0x05)；
-3. CTRL.EN=0时发送命令，返回STS_DISABLED(0x04)；
-4. 半双工请求/响应模式：请求阶段pdo_oe_o=0，响应阶段pdo_oe_o=1。</t>
+          <t>1. 检查1-bit模式：WR_CSR(0x04, 0x01)配置LANE_MODE=00，发送WR_CSR命令，监控pdi_i[0]/pdo_o[0]有效，pdi_i[3:1]忽略；
+2. 检查4-bit模式：WR_CSR(0x04, 0x03)配置LANE_MODE=01，发送命令，监控pdi_i[3:0]/pdo_o[3:0]全部有效；
+3. 检查非法值：WR_CSR(0x04, 0x05)尝试配置LANE_MODE=10，读回验证是否生效；
+4. 检查事务期间不可切换：事务执行中修改LANE_MODE，验证当前事务按原模式完成。</t>
         </is>
       </c>
       <c r="D6" s="4" t="n"/>
@@ -2227,16 +2221,15 @@
       </c>
       <c r="B7" s="12" t="inlineStr">
         <is>
-          <t>lane_mode_check</t>
+          <t>protocol_timing_check</t>
         </is>
       </c>
       <c r="C7" s="6" t="inlineStr">
         <is>
-          <t>检查lane模式配置正确性：
-1. LANE_MODE=00时，仅使用pdi_i[0]/pdo_o[0]传输，pdi_i[3:1]/pdo_o[3:1]忽略或驱动为0；
-2. LANE_MODE=01时，使用pdi_i[3:0]/pdo_o[3:0]传输，按高nibble优先发送；
-3. LANE_MODE=10/11时，返回配置错误或保持原模式不变；
-4. 事务执行期间不允许动态切换LANE_MODE生效。</t>
+          <t>1. 检查turnaround周期：请求阶段结束(pcs_n_i保持低)后，监控pdo_oe_o从0变为1恰好经过1个clk_i周期；
+2. 检查pdo_oe_o时序：响应阶段pdo_oe_o=1，其他阶段pdo_oe_o=0；
+3. 检查MSB first：发送opcode=0x10(WR_CSR)，监控pdi_i接收顺序为bit[7]-&gt;bit[0]；
+4. 检查帧边界：pcs_n_i从1-&gt;0开启事务，0-&gt;1结束事务。</t>
         </is>
       </c>
       <c r="D7" s="14" t="n"/>
@@ -2249,17 +2242,16 @@
       </c>
       <c r="B8" s="12" t="inlineStr">
         <is>
-          <t>data_interface_check</t>
+          <t>opcode_decode_check</t>
         </is>
       </c>
       <c r="C8" s="6" t="inlineStr">
         <is>
-          <t>检查数据接口时序正确性：
-1. pcs_n_i帧边界：pcs_n_i=1表示空闲，pcs_n_i=0表示帧开始；
-2. 请求阶段：主机驱动pdi_i，模块采样；
-3. 响应阶段：模块驱动pdo_o，pdo_oe_o=1；
-4. turnaround周期：请求与响应之间固定1个clk_i周期，此时pdo_oe_o=0；
-5. MSB-first传输：协议字段按最高位先发送。</t>
+          <t>1. 检查opcode=0x10译码：发送帧{0x10, 0x04, 0x00000003}，验证识别为WR_CSR，帧长=48bit(1-bit模式48拍，4-bit模式12拍)；
+2. 检查opcode=0x11译码：发送帧{0x11, 0x00}，验证识别为RD_CSR，帧长=16bit；
+3. 检查opcode=0x20译码：发送帧{0x20, 0x00001000, 0xDEADBEEF}，验证识别为AHB_WR32，帧长=72bit；
+4. 检查opcode=0x21译码：发送帧{0x21, 0x00001000}，验证识别为AHB_RD32，帧长=40bit；
+5. 检查非法opcode：发送opcode=0x00，响应status_code=0x01。</t>
         </is>
       </c>
       <c r="D8" s="14" t="n"/>
@@ -2272,17 +2264,14 @@
       </c>
       <c r="B9" s="12" t="inlineStr">
         <is>
-          <t>protocol_format_check</t>
+          <t>ctrl_config_check</t>
         </is>
       </c>
       <c r="C9" s="6" t="inlineStr">
         <is>
-          <t>检查协议帧格式正确性：
-1. WR_CSR(0x10)：opcode(8bit) + addr(8bit) + wdata(32bit) = 48bit请求，status(8bit)响应；
-2. RD_CSR(0x11)：opcode(8bit) + addr(8bit) = 16bit请求，status(8bit) + rdata(32bit) = 40bit响应；
-3. AHB_WR32(0x20)：opcode(8bit) + addr(32bit) + wdata(32bit) = 72bit请求，status(8bit)响应；
-4. AHB_RD32(0x21)：opcode(8bit) + addr(32bit) = 40bit请求，status(8bit) + rdata(32bit) = 40bit响应；
-5. 帧长度与opcode不匹配时返回STS_FRAME_ERR(0x06)。</t>
+          <t>1. 检查EN使能：WR_CSR(0x04, 0x01)配置EN=1，发送AHB_RD32命令验证可执行；WR_CSR(0x04, 0x00)配置EN=0，发送命令验证返回status_code=0x04；
+2. 检查SOFT_RST：WR_CSR(0x04, 0x08)写SOFT_RST=1，检查协议上下文清零，LANE_MODE恢复00；
+3. 检查SOFT_RST自清零：WR_CSR(0x04, 0x08)后RD_CSR(0x04)读回bit[3]=0。</t>
         </is>
       </c>
       <c r="D9" s="14" t="n"/>
@@ -2295,17 +2284,16 @@
       </c>
       <c r="B10" s="12" t="inlineStr">
         <is>
-          <t>opcode_decode_check</t>
+          <t>status_err_check</t>
         </is>
       </c>
       <c r="C10" s="6" t="inlineStr">
         <is>
-          <t>检查opcode译码正确性：
-1. opcode=0x10：WR_CSR命令，期望帧长48bit（1-bit模式）或12拍（4-bit模式）；
-2. opcode=0x11：RD_CSR命令，期望帧长16bit（1-bit模式）或4拍（4-bit模式）；
-3. opcode=0x20：AHB_WR32命令，期望帧长72bit（1-bit模式）或18拍（4-bit模式）；
-4. opcode=0x21：AHB_RD32命令，期望帧长40bit（1-bit模式）或10拍（4-bit模式）；
-5. 非法opcode（非0x10/0x11/0x20/0x21）：返回STS_BAD_OPCODE(0x01)，不发起CSR/AHB访问。</t>
+          <t>1. 检查STATUS[0]BUSY：发送命令期间RD_CSR(0x08)返回bit[0]=1，命令完成后bit[0]=0；
+2. 检查STATUS[2]CMD_ERR：发送非法opcode后STATUS bit[2]=1；
+3. 检查STATUS[3]BUS_ERR：触发hresp_i=1后STATUS bit[3]=1；
+4. 检查STATUS[4]FRAME_ERR：提前拉高pcs_n_i后STATUS bit[4]=1；
+5. 检查LAST_ERR：触发错误后RD_CSR(0x0C)返回对应错误码。</t>
         </is>
       </c>
       <c r="D10" s="14" t="n"/>
@@ -2318,16 +2306,19 @@
       </c>
       <c r="B11" s="12" t="inlineStr">
         <is>
-          <t>ctrl_config_check</t>
+          <t>error_detection_check</t>
         </is>
       </c>
       <c r="C11" s="6" t="inlineStr">
         <is>
-          <t>检查CTRL寄存器配置生效：
-1. EN字段：EN=1时模块使能，EN=0时模块禁用，命令返回STS_DISABLED(0x04)；
-2. LANE_MODE字段：配置00/01生效，配置10/11返回错误或忽略；
-3. SOFT_RST字段：写1触发软复位，协议上下文清零，LANE_MODE恢复默认1-bit模式；
-4. 配置后立即生效（下一拍）。</t>
+          <t>1. 检查BAD_OPCODE(0x01)：发送opcode=0x00，响应status_code==0x01，不发起AHB访问；
+2. 检查BAD_REG(0x02)：RD_CSR(0x10)，status_code==0x02；
+3. 检查ALIGN_ERR(0x03)：AHB_WR32(addr=0x00000003)，status_code==0x03，htrans_o保持IDLE；
+4. 检查DISABLED(0x04)：WR_CSR(0x04, 0x00)后发送命令，status_code==0x04；
+5. 检查NOT_IN_TEST(0x05)：test_mode_i=0时发送命令，status_code==0x05；
+6. 检查FRAME_ERR(0x06)：请求阶段提前拉高pcs_n_i，status_code==0x06；
+7. 检查AHB_ERR(0x07)：配置AHB slave返回hresp_i=1，status_code==0x07；
+8. 检查TIMEOUT(0x08)：配置hready_i=0持续&gt;1024周期，status_code==0x08。</t>
         </is>
       </c>
       <c r="D11" s="14" t="n"/>
@@ -2340,19 +2331,15 @@
       </c>
       <c r="B12" s="12" t="inlineStr">
         <is>
-          <t>status_polling_check</t>
+          <t>low_power_check</t>
         </is>
       </c>
       <c r="C12" s="6" t="inlineStr">
         <is>
-          <t>检查状态轮询机制：
-1. STATUS[0] BUSY：事务执行期间为1，空闲时为0；
-2. STATUS[1] RESP_VALID：响应有效时为1，读STATUS后清零或保持；
-3. STATUS[2] CMD_ERR：命令错误时置1（sticky）；
-4. STATUS[3] BUS_ERR：总线错误时置1（sticky）；
-5. STATUS[4] FRAME_ERR：帧错误时置1（sticky）；
-6. LAST_ERR[7:0]：记录最近一次错误码（0x01~0x08）；
-7. 无独立中断输出信号。</t>
+          <t>1. 检查空闲态移位寄存器：pcs_n_i=1时，监控内部rx_shift_reg和tx_shift_reg信号不翻转；
+2. 检查超时计数器：监控timeout_counter仅在AHB_WAIT状态计数；
+3. 检查AHB空闲输出：test_mode_i=0时，htrans_o==2'b00, hwrite_o==0；
+4. 检查关键寄存器翻转：仅在RX/TX/WAIT_AHB状态翻转相关寄存器。</t>
         </is>
       </c>
       <c r="D12" s="14" t="n"/>
@@ -2365,20 +2352,14 @@
       </c>
       <c r="B13" s="12" t="inlineStr">
         <is>
-          <t>error_detection_check</t>
+          <t>throughput_check</t>
         </is>
       </c>
       <c r="C13" s="6" t="inlineStr">
         <is>
-          <t>检查错误检测与返回：
-1. BAD_OPCODE(0x01)：opcode非0x10/0x11/0x20/0x21，返回status=0x01，STATUS.CMD_ERR=1，LAST_ERR=0x01；
-2. BAD_REG(0x02)：CSR地址非0x00/0x04/0x08/0x0C，返回status=0x02，STATUS.CMD_ERR=1，LAST_ERR=0x02；
-3. ALIGN_ERR(0x03)：AHB地址非4Byte对齐，返回status=0x03，STATUS.CMD_ERR=1，LAST_ERR=0x03；
-4. DISABLED(0x04)：CTRL.EN=0时发送命令，返回status=0x04，STATUS.CMD_ERR=1，LAST_ERR=0x04；
-5. NOT_IN_TEST(0x05)：test_mode_i=0时发送命令，返回status=0x05，STATUS.CMD_ERR=1，LAST_ERR=0x05；
-6. FRAME_ERR(0x06)：pcs_n_i提前拉高或帧长度不匹配，返回status=0x06，STATUS.FRAME_ERR=1，LAST_ERR=0x06；
-7. AHB_ERR(0x07)：hresp_i=1，返回status=0x07，STATUS.BUS_ERR=1，LAST_ERR=0x07；
-8. TIMEOUT(0x08)：hready_i等待超时，返回status=0x08，STATUS.BUS_ERR=1，LAST_ERR=0x08。</t>
+          <t>1. 检查端到端延时：4-bit模式发送AHB_RD32，从pcs_n_i拉低到pdo_o输出第一个status bit，周期数约23~24个clk_i；
+2. 检查吞吐率：连续发送100次AHB_RD32，计算吞吐率，4-bit模式目标&gt;40MB/s；
+3. 检查AHB访问粒度：hsize_o==3'b010(WORD)，haddr_o[1:0]==2'b00。</t>
         </is>
       </c>
       <c r="D13" s="14" t="n"/>
@@ -2391,17 +2372,16 @@
       </c>
       <c r="B14" s="12" t="inlineStr">
         <is>
-          <t>low_power_check</t>
+          <t>dfx_observability_check</t>
         </is>
       </c>
       <c r="C14" s="6" t="inlineStr">
         <is>
-          <t>检查低功耗设计实现：
-1. pcs_n_i=1时，接收移位寄存器（rx_shift_reg）不更新；
-2. 非发送阶段（pdo_oe_o=0），发送移位寄存器（tx_shift_reg）不翻转；
-3. timeout_counter仅在AHB等待态（wait_ahb状态）工作；
-4. test_mode_i=0时，AHB输出保持IDLE（htrans_o=2'b00）；
-5. 仅在RX/TX/WAIT_AHB相关状态翻转关键寄存器。</t>
+          <t>1. 检查状态机状态可观测：仿真中可访问内部fsm_state信号；
+2. 检查opcode可观测：可访问当前执行的opcode_reg信号；
+3. 检查地址/数据可观测：可访问addr_reg, wdata_reg, rdata_reg信号；
+4. 检查rx/tx计数可观测：可访问rx_cnt, tx_cnt信号；
+5. 检查status_code可观测：可访问status_code信号。</t>
         </is>
       </c>
       <c r="D14" s="14" t="n"/>
@@ -2414,18 +2394,14 @@
       </c>
       <c r="B15" s="12" t="inlineStr">
         <is>
-          <t>performance_check</t>
+          <t>csr_memory_map_check</t>
         </is>
       </c>
       <c r="C15" s="6" t="inlineStr">
         <is>
-          <t>检查性能指标达成：
-1. 工作频率：clk_i稳定工作于100MHz（±1%）；
-2. 1-bit模式链路线速：理论12.5MB/s（100MHz/8）；
-3. 4-bit模式链路线速：理论50MB/s（100MHz/2）；
-4. AHB_RD32端到端延时：4-bit模式下约23~24 cycles；
-5. AHB_WR32端到端延时：4-bit模式下约23 cycles；
-6. AHB访问约束：hsize_o=3'b010（WORD），地址4Byte对齐。</t>
+          <t>1. 检查CSR访问路径：通过协议命令WR_CSR/RD_CSR访问CSR，不通过AHB地址空间；
+2. 检查AHB Master地址空间：AHB_WR32/AHB_RD32命令时haddr_o输出32-bit地址，支持完整地址空间；
+3. 检查访问粒度：CSR和AHB访问均为32-bit word粒度。</t>
         </is>
       </c>
       <c r="D15" s="14" t="n"/>
@@ -2438,71 +2414,32 @@
       </c>
       <c r="B16" s="12" t="inlineStr">
         <is>
-          <t>dfx_observability_check</t>
+          <t>ahb_interface_check</t>
         </is>
       </c>
       <c r="C16" s="6" t="inlineStr">
         <is>
-          <t>检查DFX调试可观测性：
-1. 状态机状态（fsm_state）可观测；
-2. opcode寄存器（opcode_reg）可观测；
-3. 地址寄存器（addr_reg）可观测；
-4. 写数据寄存器（wdata_reg）可观测；
-5. 读数据寄存器（rdata_reg）可观测；
-6. 状态码（status_code）可观测；
-7. rx/tx计数器可观测；
-8. 外部接口信号（pcs_n_i/pdi_i/pdo_o/pdo_oe_o）可观测。</t>
+          <t>1. 检查htrans_o：发送AHB_WR32命令，监控htrans_o仅输出2'b00(IDLE)或2'b10(NONSEQ)；
+2. 检查hsize_o：AHB命令期间hsize_o==3'b010(WORD)；
+3. 检查hburst_o：hburst_o==3'b000(SINGLE)；
+4. 检查写时序：AHB_WR32时，第1周期haddr_o/hwrite_o=1/htrans_o=NONSEQ输出，第2周期hwdata_o输出数据；
+5. 检查读时序：AHB_RD32时，第1周期haddr_o/hwrite_o=0/htrans_o=NONSEQ输出，第2周期采样hrdata_i；
+6. 检查hresp_i=1处理：配置slave返回hresp_i=1，验证事务正确终止；
+7. 检查hready_i=0处理：配置hready_i=0，验证等待状态处理。</t>
         </is>
       </c>
       <c r="D16" s="14" t="n"/>
     </row>
     <row r="17">
-      <c r="A17" s="12" t="inlineStr">
-        <is>
-          <t>CHK_015</t>
-        </is>
-      </c>
-      <c r="B17" s="12" t="inlineStr">
-        <is>
-          <t>memory_map_check</t>
-        </is>
-      </c>
-      <c r="C17" s="6" t="inlineStr">
-        <is>
-          <t>检查Memory map访问约束：
-1. 模块自身CSR（VERSION/CTRL/STATUS/LAST_ERR）不进入SoC AHB memory map，仅通过协议命令访问；
-2. AHB Master访问采用32bit地址空间（haddr_o[31:0]）；
-3. AHB Master访问粒度为word（4Byte）；
-4. 目标地址范围由SoC顶层约束。</t>
-        </is>
-      </c>
+      <c r="A17" s="12" t="n"/>
+      <c r="B17" s="12" t="n"/>
+      <c r="C17" s="6" t="n"/>
       <c r="D17" s="14" t="n"/>
     </row>
     <row r="18">
-      <c r="A18" s="12" t="inlineStr">
-        <is>
-          <t>CHK_016</t>
-        </is>
-      </c>
-      <c r="B18" s="12" t="inlineStr">
-        <is>
-          <t>ahb_interface_check</t>
-        </is>
-      </c>
-      <c r="C18" s="6" t="inlineStr">
-        <is>
-          <t>检查AHB-Lite Master接口正确性：
-1. htrans_o：仅输出IDLE(2'b00)或NONSEQ(2'b10)，不输出SEQ(2'b11)；
-2. hsize_o：固定为WORD(3'b010)；
-3. hburst_o：固定为SINGLE(3'b000)；
-4. hwrite_o：写命令为1，读命令为0；
-5. haddr_o：地址4Byte对齐；
-6. hwdata_o：在地址相下一拍输出写数据；
-7. hrdata_i：正确采样读返回数据；
-8. hready_i：等待周期处理，支持多周期等待；
-9. hresp_i：错误响应检测，返回STS_AHB_ERR(0x07)。</t>
-        </is>
-      </c>
+      <c r="A18" s="12" t="n"/>
+      <c r="B18" s="12" t="n"/>
+      <c r="C18" s="6" t="n"/>
       <c r="D18" s="14" t="n"/>
     </row>
     <row r="19">
@@ -2541,9 +2478,6 @@
       <c r="C24" s="6" t="n"/>
       <c r="D24" s="4" t="n"/>
     </row>
-    <row r="25"/>
-    <row r="26"/>
-    <row r="27"/>
     <row r="28">
       <c r="A28" s="23" t="inlineStr">
         <is>
@@ -2661,26 +2595,21 @@
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>clk_freq_test</t>
+          <t>xxx</t>
         </is>
       </c>
       <c r="C3" s="3" t="inlineStr">
         <is>
-          <t>配置条件：
-1. 时钟配置：clk_i频率设置为100MHz，test_mode_i=1
-2. 模块使能：通过WR_CSR设置CTRL.EN=1
-3. LANE_MODE：分别配置为00（1-bit）和01（4-bit）两种模式
+          <t xml:space="preserve">配置条件：
+//对配置寄存器或接口控制信号进行描述
 输入激励：
-1. 发送AHB_RD32命令，读取SoC内部测试地址
-2. 发送AHB_WR32命令，写入SoC内部测试地址
-3. 交替执行读/写命令，覆盖两种lane模式
-4. 持续运行1000个事务以上
+1/对接口激励进行描述
 期望结果：
-1. 所有命令在100MHz频率下正确执行
-2. 协议采样、状态机控制和AHB-Lite主接口同域工作正常
-3. 无时序违例，无setup/hold violation
+// 描述逻辑处理期望的结果，以及check点
 coverage check点：
-直接用例覆盖，不收功能覆盖率。</t>
+//如果通过随机测试，功能模型建模来确认对测试点的覆盖，需要描述功能模型的功能。如果通过直接用例来覆盖测试点，则不需要收集功
+能覆盖率，该部分内容不用描述。
+</t>
         </is>
       </c>
       <c r="D3" s="4" t="n"/>
@@ -2693,28 +2622,28 @@
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>reset_test</t>
+          <t>test_reset_behavior</t>
         </is>
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
           <t>配置条件：
 1. 初始状态：rst_ni=0，模块处于复位状态
-2. 时钟正常：clk_i=100MHz
+2. test_mode_i=1，clk_i=100MHz
 输入激励：
-1. 释放rst_ni（拉高），等待1个时钟周期
-2. 通过RD_CSR读取CTRL寄存器，验证EN=0、LANE_MODE=00、SOFT_RST=0
-3. 通过RD_CSR读取STATUS寄存器，验证所有位为0
-4. 通过RD_CSR读取LAST_ERR寄存器，验证ERR_CODE=0x00
-5. 检查状态机状态fsm_state == IDLE
-6. 检查协议上下文（rx_shift_reg、tx_shift_reg、opcode_reg等）为初始值
+1. 拉高rst_ni释放复位，等待2个clk_i周期确保复位同步释放
+2. 通过RD_CSR命令(opcode=0x11, addr=0x04)读取CTRL寄存器，验证返回值
+3. 通过RD_CSR命令(opcode=0x11, addr=0x08)读取STATUS寄存器
+4. 通过RD_CSR命令(opcode=0x11, addr=0x0C)读取LAST_ERR寄存器
+5. 监控AHB接口信号：htrans_o, hwrite_o
 期望结果：
-1. 状态机处于IDLE状态
-2. CTRL.EN=0，CTRL.LANE_MODE=00（1-bit默认值）
-3. STATUS/LAST_ERR寄存器清零
-4. 协议上下文和错误状态已清空
+1. CTRL寄存器返回值bit[0]=0(EN=0), bit[2:1]=00(LANE_MODE=1-bit), bit[3]=0(SOFT_RST=0)
+2. STATUS寄存器返回0x00
+3. LAST_ERR寄存器返回0x00
+4. AHB接口：htrans_o=2'b00(IDLE), hwrite_o=0
+5. 内部状态机fsm_state=IDLE(0x00)
 coverage check点：
-直接用例覆盖，不收功能覆盖率。</t>
+直接用例覆盖，不收功能覆盖率</t>
         </is>
       </c>
       <c r="D4" s="4" t="n"/>
@@ -2727,30 +2656,30 @@
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>csr_access_test</t>
+          <t>test_csr_access</t>
         </is>
       </c>
       <c r="C5" s="3" t="inlineStr">
         <is>
           <t>配置条件：
-1. 模块使能：test_mode_i=1，CTRL.EN=1
-2. 配置LANE_MODE=00或01
+1. test_mode_i=1
+2. 通过WR_CSR命令(opcode=0x10, addr=0x04, wdata=0x00000001)设置CTRL.EN=1
+3. 配置LANE_MODE=00(1-bit模式)
 输入激励：
-1. RD_CSR读取VERSION寄存器（地址0x00），验证版本号
-2. WR_CSR写入CTRL寄存器（地址0x04），配置EN=1、LANE_MODE=01
-3. RD_CSR读回CTRL寄存器，验证写入值正确
-4. WR_CSR写入CTRL寄存器，配置SOFT_RST=1，触发软复位
-5. RD_CSR读取STATUS寄存器（地址0x08），检查BUSY/RESP_VALID/CMD_ERR等字段
-6. RD_CSR读取LAST_ERR寄存器（地址0x0C），检查最近错误码
-7. 尝试访问非法CSR地址（如0x10），验证返回STS_BAD_REG(0x02)
+1. 发送RD_CSR命令(opcode=0x11, addr=0x00)读取VERSION寄存器，记录返回的version值
+2. 发送WR_CSR命令(opcode=0x10, addr=0x04, wdata=0x00000003)，配置EN=1, LANE_MODE=01
+3. 发送RD_CSR命令(opcode=0x11, addr=0x04)读取CTRL寄存器，验证写入值
+4. 发送RD_CSR命令(opcode=0x11, addr=0x08)读取STATUS寄存器
+5. 发送RD_CSR命令(opcode=0x11, addr=0x0C)读取LAST_ERR寄存器
+6. 发送RD_CSR命令(opcode=0x11, addr=0x10)尝试访问非法CSR地址
 期望结果：
-1. CSR读写正确，VERSION返回预期值
-2. CTRL配置生效，LANE_MODE切换成功
-3. SOFT_RST触发软复位，上下文清零
-4. STATUS/LAST_ERR反映正确状态
-5. 非法地址访问返回错误码0x02
+1. VERSION寄存器返回预设版本号(如0x00000100)
+2. CTRL写入0x03后读回0x03
+3. STATUS返回当前状态
+4. 非法地址0x10的访问返回status_code=0x02(BAD_REG)
+5. VERSION/STATUS/LAST_ERR寄存器只读属性正确：写入后读回值不变
 coverage check点：
-直接用例覆盖，不收功能覆盖率。</t>
+对CSR地址(0x00/0x04/0x08/0x0C/非法地址)和读/写属性收集功能覆盖率</t>
         </is>
       </c>
       <c r="D5" s="4" t="n"/>
@@ -2763,27 +2692,28 @@
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>test_mode_test</t>
+          <t>test_work_mode_ate</t>
         </is>
       </c>
       <c r="C6" s="3" t="inlineStr">
         <is>
           <t>配置条件：
-1. 初始状态：test_mode_i=0，CTRL.EN=0
+1. test_mode_i=1
+2. 通过WR_CSR(opcode=0x10, addr=0x04, wdata=0x00000001)设置CTRL.EN=1
+3. 配置LANE_MODE=01(4-bit模式，wdata=0x00000003)
 输入激励：
-1. test_mode_i=0时，发送WR_CSR命令，验证返回STS_NOT_IN_TEST(0x05)
-2. test_mode_i=1，CTRL.EN=0时，发送AHB_RD32命令，验证返回STS_DISABLED(0x04)
-3. test_mode_i=1，CTRL.EN=1时，发送WR_CSR命令验证正常执行
-4. 发送AHB_WR32命令，验证半双工模式：请求阶段pdo_oe_o=0，响应阶段pdo_oe_o=1
-5. 发送AHB_RD32命令，验证请求/响应分离正确
+1. 发送WR_CSR命令(opcode=0x10, addr=0x04, wdata=0x00000003)，配置EN=1, LANE_MODE=01
+2. 发送AHB_WR32命令(opcode=0x20, addr=0x00001000, wdata=0xDEADBEEF)
+3. 发送AHB_RD32命令(opcode=0x21, addr=0x00001000)，验证读回0xDEADBEEF
+4. 监控协议时序：pcs_n_i, pdi_i, pdo_o, pdo_oe_o
 期望结果：
-1. test_mode_i=0时命令返回错误码0x05
-2. CTRL.EN=0时命令返回错误码0x04
-3. 使能状态下命令正常执行
-4. 半双工请求/响应模式工作正常
-5. CSR访问与AHB-Lite单次读写正常
+1. WR_CSR命令成功，status_code=0x00
+2. AHB_WR32命令成功，haddr_o=0x00001000, hwdata_o=0xDEADBEEF
+3. AHB_RD32命令成功，hrdata_i返回0xDEADBEEF
+4. 半双工协议正确：请求阶段-&gt;turnaround(1周期)-&gt;响应阶段
+5. pdo_oe_o在响应阶段=1，其他阶段=0
 coverage check点：
-直接用例覆盖，不收功能覆盖率。</t>
+对命令类型(WR_CSR/RD_CSR/AHB_WR32/AHB_RD32)和LANE_MODE(00/01)组合收集功能覆盖率</t>
         </is>
       </c>
       <c r="D6" s="4" t="n"/>
@@ -2796,26 +2726,29 @@
       </c>
       <c r="B7" s="16" t="inlineStr">
         <is>
-          <t>lane_mode_test</t>
+          <t>test_lane_mode</t>
         </is>
       </c>
       <c r="C7" s="3" t="inlineStr">
         <is>
           <t>配置条件：
-1. 模块使能：test_mode_i=1，CTRL.EN=1
+1. test_mode_i=1, CTRL.EN=1(通过WR_CSR: opcode=0x10, addr=0x04, wdata=0x00000001)
+2. clk_i=100MHz
 输入激励：
-1. 配置LANE_MODE=00，发送WR_CSR命令，验证仅pdi_i[0]/pdo_o[0]有效
-2. 配置LANE_MODE=01，发送AHB_RD32命令，验证pdi_i[3:0]/pdo_o[3:0]按高nibble优先发送
-3. 配置LANE_MODE=10，验证返回错误或忽略配置
-4. 配置LANE_MODE=11，验证返回错误或忽略配置
-5. 事务执行期间尝试切换LANE_MODE，验证原模式保持至事务结束
+1. 配置LANE_MODE=00：发送WR_CSR(opcode=0x10, addr=0x04, wdata=0x00000001)
+2. 发送RD_CSR命令(opcode=0x11, addr=0x00)，监控pdi_i[0]/pdo_o[0]有效，pdi_i[3:1]忽略
+3. 配置LANE_MODE=01：发送WR_CSR(opcode=0x10, addr=0x04, wdata=0x00000003)
+4. 发送相同RD_CSR命令，监控pdi_i[3:0]/pdo_o[3:0]全部有效，高nibble优先发送
+5. 尝试配置LANE_MODE=10：发送WR_CSR(opcode=0x10, addr=0x04, wdata=0x00000005)
+6. 发送RD_CSR(opcode=0x11, addr=0x04)读取CTRL，验证LANE_MODE是否生效
+7. 在事务执行期间修改LANE_MODE，验证当前事务不受影响
 期望结果：
-1. 1-bit模式正常工作，仅bit0传输数据
-2. 4-bit模式正常工作，高nibble优先发送
-3. 非法LANE_MODE配置返回错误或保持原值
-4. 事务期间模式切换不生效
+1. LANE_MODE=00(1-bit)时：数据仅通过pdi_i[0]/pdo_o[0]传输，帧长按1-bit计算(如RD_CSR=16拍)
+2. LANE_MODE=01(4-bit)时：数据通过pdi_i[3:0]/pdo_o[3:0]传输，高nibble优先，帧长按4-bit计算(如RD_CSR=4拍)
+3. LANE_MODE=10写入后读回仍为原值或返回错误
+4. 事务执行期间修改LANE_MODE不影响当前事务
 coverage check点：
-直接用例覆盖，不收功能覆盖率。</t>
+对LANE_MODE配置值(00/01/10/11)收集功能覆盖率</t>
         </is>
       </c>
       <c r="D7" s="14" t="n"/>
@@ -2828,28 +2761,27 @@
       </c>
       <c r="B8" s="16" t="inlineStr">
         <is>
-          <t>data_interface_test</t>
+          <t>test_data_interface</t>
         </is>
       </c>
       <c r="C8" s="3" t="inlineStr">
         <is>
           <t>配置条件：
-1. 模块使能：test_mode_i=1，CTRL.EN=1
-2. 配置1-bit和4-bit lane模式
+1. test_mode_i=1
+2. 通过WR_CSR(opcode=0x10, addr=0x04, wdata=0x00000001)设置CTRL.EN=1, LANE_MODE=00
+3. 配置LANE_MODE=01：WR_CSR(opcode=0x10, addr=0x04, wdata=0x00000003)
 输入激励：
-1. 在1-bit模式下发送WR_CSR命令，监控pdi_i[0]/pdo_o[0]数据传输
-2. 在4-bit模式下发送AHB_WR32命令，监控pdi_i[3:0]/pdo_o[3:0]数据传输
-3. 验证pcs_n_i帧边界：拉低开始帧，拉高结束帧
-4. 验证MSB-first传输顺序
-5. 验证turnaround周期（1个clk_i）
+1. 在1-bit模式下(LANE_MODE=00)：发送WR_CSR(opcode=0x10, addr=0x04, wdata=0x00000003)，监控pdi_i[0]和pdo_o[0]信号波形，忽略pdi_i[3:1]
+2. 在4-bit模式下(LANE_MODE=01)：发送相同WR_CSR命令，监控pdi_i[3:0]和pdo_o[3:0]信号波形
+3. 验证MSB first传输顺序：发送opcode=0x10(二进制0001_0000)，监控pdi_i接收顺序为bit[7]-&gt;bit[6]-&gt;...-&gt;bit[0]
+4. 验证帧边界：监控pcs_n_i从1-&gt;0开启事务，命令完成后0-&gt;1结束事务
 期望结果：
-1. 1-bit模式数据按bit0顺序传输
-2. 4-bit模式数据按高nibble优先传输
-3. pcs_n_i帧边界清晰正确
-4. MSB-first顺序正确
-5. turnaround固定1周期
+1. 1-bit模式：pdi_i[0]/pdo_o[0]传输数据，pdi_i[3:1]被忽略，帧长=48拍(opcode+addr+wdata各按1-bit传输)
+2. 4-bit模式：pdi_i[3:0]/pdo_o[3:0]全部有效，高nibble先发送，帧长=12拍
+3. MSB first正确：opcode 0x10发送顺序为0001_0000(MSB first)
+4. 帧边界正确：pcs_n_i低有效期间为事务周期
 coverage check点：
-直接用例覆盖，不收功能覆盖率。</t>
+直接用例覆盖，不收功能覆盖率</t>
         </is>
       </c>
       <c r="D8" s="14" t="n"/>
@@ -2862,31 +2794,31 @@
       </c>
       <c r="B9" s="16" t="inlineStr">
         <is>
-          <t>protocol_format_test</t>
+          <t>test_turnaround</t>
         </is>
       </c>
       <c r="C9" s="3" t="inlineStr">
         <is>
           <t>配置条件：
-1. 模块使能：test_mode_i=1，CTRL.EN=1
-2. 配置不同lane模式
+1. test_mode_i=1, CTRL.EN=1
+2. 配置LANE_MODE=01(4-bit模式)
 输入激励：
-1. 发送WR_CSR(0x10)命令：opcode(8bit)+addr(8bit)+wdata(32bit)，验证请求阶段
-2. 验证turnaround周期（1个clk_i），pdo_oe_o=0
-3. 检查响应阶段pdo_oe_o=1，输出使能正确
-4. 发送RD_CSR(0x11)命令：opcode(8bit)+addr(8bit)，验证响应包含status+rdata
-5. 发送AHB_WR32(0x20)命令：opcode(8bit)+addr(32bit)+wdata(32bit)
-6. 发送AHB_RD32(0x21)命令：opcode(8bit)+addr(32bit)
-7. 提前拉高pcs_n_i验证FRAME_ERR错误
+1. 发送WR_CSR命令(opcode=0x10, addr=0x04, wdata=0x00000003)
+2. 监控请求阶段结束时刻(最后一个数据接收完成)
+3. 监控turnaround周期：记录pdo_oe_o从0变为1的时间间隔
+4. 监控响应阶段pdo_oe_o状态
+5. 发送四种命令验证帧格式：
+   - WR_CSR: opcode=0x10, addr=0x04, wdata=0x00000001
+   - RD_CSR: opcode=0x11, addr=0x00
+   - AHB_WR32: opcode=0x20, addr=0x00001000, wdata=0x12345678
+   - AHB_RD32: opcode=0x21, addr=0x00001000
 期望结果：
-1. WR_CSR请求48bit，响应8bit
-2. RD_CSR请求16bit，响应40bit
-3. AHB_WR32请求72bit，响应8bit
-4. AHB_RD32请求40bit，响应40bit
-5. turnaround固定1周期，协议字段MSB first传输
-6. 提前结束帧返回FRAME_ERR(0x06)
+1. 请求阶段结束后，pdo_oe_o保持0恰好1个clk_i周期
+2. turnaround后pdo_oe_o=1，进入响应阶段
+3. 响应阶段pdo_oe_o=1，输出status+rdata
+4. 四种命令帧格式正确处理，响应格式：写命令返回8-bit status，读命令返回8-bit status+32-bit rdata
 coverage check点：
-直接用例覆盖，不收功能覆盖率。</t>
+对四种命令类型(0x10/0x11/0x20/0x21)收集功能覆盖率</t>
         </is>
       </c>
       <c r="D9" s="14" t="n"/>
@@ -2899,29 +2831,32 @@
       </c>
       <c r="B10" s="16" t="inlineStr">
         <is>
-          <t>opcode_decode_test</t>
+          <t>test_opcode_decode</t>
         </is>
       </c>
       <c r="C10" s="3" t="inlineStr">
         <is>
           <t>配置条件：
-1. 模块使能：test_mode_i=1，CTRL.EN=1
-2. AHB总线空闲
+1. test_mode_i=1
+2. 通过WR_CSR(opcode=0x10, addr=0x04, wdata=0x00000001)设置CTRL.EN=1
+3. AHB总线空闲
 输入激励：
-1. 发送opcode=0x10执行WR_CSR命令，验证帧长判定正确
-2. 发送opcode=0x11执行RD_CSR命令，验证帧长判定正确
-3. 发送opcode=0x20执行AHB_WR32命令，验证帧长判定正确
-4. 发送opcode=0x21执行AHB_RD32命令，验证帧长判定正确
-5. 发送非法opcode=0x00，验证返回STS_BAD_OPCODE(0x01)
-6. 发送非法opcode=0xFF，验证返回STS_BAD_OPCODE(0x01)
-7. 发送其他非法opcode（如0x12、0x22等），验证错误处理
+1. 发送opcode=0x10的WR_CSR命令，帧格式{0x10, 0x04, 0x00000003}，监控帧长=12拍(4-bit模式)
+2. 发送opcode=0x11的RD_CSR命令，帧格式{0x11, 0x00}，监控帧长=4拍
+3. 发送opcode=0x20的AHB_WR32命令，帧格式{0x20, 0x00001000, 0xDEADBEEF}，监控帧长=18拍
+4. 发送opcode=0x21的AHB_RD32命令，帧格式{0x21, 0x00001000}，监控帧长=10拍
+5. 发送非法opcode=0x00，监控响应status_code
+6. 发送非法opcode=0xFF，监控响应status_code
 期望结果：
-1. 四种opcode正确译码并执行对应命令
-2. 前端正确确定期望帧长
-3. 非法opcode返回STS_BAD_OPCODE(0x01)
-4. 非法opcode不发起CSR/AHB访问
+1. opcode=0x10正确译码为WR_CSR，期望帧长=48bit(4-bit模式12拍)
+2. opcode=0x11正确译码为RD_CSR，期望帧长=16bit(4-bit模式4拍)
+3. opcode=0x20正确译码为AHB_WR32，期望帧长=72bit(4-bit模式18拍)
+4. opcode=0x21正确译码为AHB_RD32，期望帧长=40bit(4-bit模式10拍)
+5. opcode=0x00返回status_code=0x01(BAD_OPCODE)
+6. opcode=0xFF返回status_code=0x01(BAD_OPCODE)
+7. 非法opcode不发起AHB访问
 coverage check点：
-直接用例覆盖，不收功能覆盖率。</t>
+对opcode值(0x10/0x11/0x20/0x21/非法值)收集功能覆盖率</t>
         </is>
       </c>
       <c r="D10" s="14" t="n"/>
@@ -2934,29 +2869,32 @@
       </c>
       <c r="B11" s="16" t="inlineStr">
         <is>
-          <t>ctrl_config_test</t>
+          <t>test_ctrl_config</t>
         </is>
       </c>
       <c r="C11" s="3" t="inlineStr">
         <is>
           <t>配置条件：
-1. 模块初始状态：test_mode_i=1
+1. test_mode_i=1
 输入激励：
-1. 写CTRL.EN=1使能模块，发送命令验证可执行
-2. 写CTRL.EN=0禁用模块，发送命令验证返回STS_DISABLED(0x04)
-3. 配置LANE_MODE=00验证1-bit模式生效
-4. 配置LANE_MODE=01验证4-bit模式生效
-5. 配置LANE_MODE=10/11验证错误处理
-6. 写CTRL.SOFT_RST=1触发软复位
-7. 验证软复位后协议上下文清零，LANE_MODE恢复默认
+1. 写CTRL.EN=1：发送WR_CSR(opcode=0x10, addr=0x04, wdata=0x00000001)
+2. 发送AHB_RD32命令(opcode=0x21, addr=0x00001000)验证功能命令可执行
+3. 写CTRL.EN=0：发送WR_CSR(opcode=0x10, addr=0x04, wdata=0x00000000)
+4. 发送AHB_RD32命令，验证返回status_code=0x04(DISABLED)
+5. 写CTRL.LANE_MODE=01：发送WR_CSR(opcode=0x10, addr=0x04, wdata=0x00000003)
+6. 发送RD_CSR(opcode=0x11, addr=0x04)读取CTRL，验证LANE_MODE=01
+7. 写CTRL.SOFT_RST=1：发送WR_CSR(opcode=0x10, addr=0x04, wdata=0x00000008)
+8. 发送RD_CSR(opcode=0x11, addr=0x04)读取CTRL，验证SOFT_RST=0(自清零)且LANE_MODE恢复00
+9. 检查协议上下文是否清零
 期望结果：
-1. EN=1时命令正常执行，EN=0时返回错误
-2. LANE_MODE=00/01配置生效
-3. LANE_MODE=10/11返回错误或忽略
-4. SOFT_RST触发软复位，上下文清零
-5. 软复位后LANE_MODE恢复1-bit模式
+1. CTRL.EN=1时功能命令成功执行，status_code=0x00
+2. CTRL.EN=0时返回status_code=0x04(DISABLED)
+3. CTRL.LANE_MODE配置生效，读回值与写入一致
+4. CTRL.SOFT_RST=1后读回bit[3]=0(自清零)
+5. 软复位后LANE_MODE恢复00(1-bit默认值)
+6. 协议上下文(rx_shift_reg, tx_shift_reg等)清零
 coverage check点：
-直接用例覆盖，不收功能覆盖率。</t>
+对CTRL字段组合(EN=0/1, LANE_MODE=00/01/10/11, SOFT_RST=0/1)收集功能覆盖率</t>
         </is>
       </c>
       <c r="D11" s="14" t="n"/>
@@ -2969,28 +2907,31 @@
       </c>
       <c r="B12" s="16" t="inlineStr">
         <is>
-          <t>status_polling_test</t>
+          <t>test_status_query</t>
         </is>
       </c>
       <c r="C12" s="3" t="inlineStr">
         <is>
           <t>配置条件：
-1. 模块使能：test_mode_i=1，CTRL.EN=1
-2. 执行各类命令触发不同状态
+1. test_mode_i=1
+2. 通过WR_CSR(opcode=0x10, addr=0x04, wdata=0x00000001)设置CTRL.EN=1
 输入激励：
-1. 触发各类错误条件：非法opcode、帧错误、AHB错误等
-2. 通过RD_CSR读取STATUS寄存器，检查sticky位：CMD_ERR/BUS_ERR/FRAME_ERR
-3. 读取LAST_ERR寄存器获取最近错误码
-4. 验证BUSY位在事务执行期间为1，空闲时为0
-5. 验证RESP_VALID位在响应有效时为1
-6. 验证无独立中断输出信号
+1. 发送非法opcode=0x00，触发BAD_OPCODE错误
+2. 发送RD_CSR(opcode=0x11, addr=0x08)读取STATUS寄存器，检查bit[2]=1(CMD_ERR)
+3. 发送RD_CSR(opcode=0x11, addr=0x0C)读取LAST_ERR寄存器，验证返回0x01(BAD_OPCODE)
+4. 配置AHB slave返回hresp_i=1，发送AHB_RD32命令触发AHB_ERR
+5. 读取STATUS检查bit[3]=1(BUS_ERR)，读取LAST_ERR返回0x07
+6. 发送命令过程中提前拉高pcs_n_i，触发FRAME_ERR
+7. 读取STATUS检查bit[4]=1(FRAME_ERR)，读取LAST_ERR返回0x06
+8. 验证无独立中断输出信号
 期望结果：
-1. STATUS寄存器正确反映当前状态
-2. sticky错误位保持，需手动清除
-3. LAST_ERR记录最近错误码
-4. 无中断输出，通过轮询获取状态
+1. 触发错误后STATUS相应错误位置位且sticky
+2. LAST_ERR记录最近一次错误码
+3. 多次错误后LAST_ERR只记录最近一次
+4. MVP版本无中断输出信号
+5. 通过轮询STATUS/LAST_ERR可获取错误状态
 coverage check点：
-直接用例覆盖，不收功能覆盖率。</t>
+直接用例覆盖，不收功能覆盖率</t>
         </is>
       </c>
       <c r="D12" s="14" t="n"/>
@@ -3003,30 +2944,36 @@
       </c>
       <c r="B13" s="16" t="inlineStr">
         <is>
-          <t>error_detection_test</t>
+          <t>test_error_handling</t>
         </is>
       </c>
       <c r="C13" s="3" t="inlineStr">
         <is>
           <t>配置条件：
-1. 模块使能：test_mode_i=1，CTRL.EN=1
-2. AHB总线正常
+1. test_mode_i=1
+2. 通过WR_CSR(opcode=0x10, addr=0x04, wdata=0x00000001)设置CTRL.EN=1
+3. AHB总线正常工作
 输入激励：
-1. 发送非法opcode(0x00/0xFF)验证BAD_OPCODE错误(0x01)
-2. 访问非法CSR地址(0x10)验证BAD_REG错误(0x02)
-3. 发送非4Byte对齐地址(如0x0000_0001)验证ALIGN_ERR错误(0x03)
-4. CTRL.EN=0时发送命令验证DISABLED错误(0x04)
-5. test_mode_i=0时发送命令验证NOT_IN_TEST错误(0x05)
-6. 提前拉高pcs_n_i验证FRAME_ERR错误(0x06)
-7. 触发hresp_i=1验证AHB_ERR错误(0x07)
-8. 模拟AHB超时（hready_i长时间为0）验证TIMEOUT错误(0x08)
+1. 发送opcode=0x00验证BAD_OPCODE(0x01)：发送帧{0x00}，监控响应status_code==0x01，htrans_o保持IDLE
+2. 发送RD_CSR(addr=0x10)验证BAD_REG(0x02)：发送帧{0x11, 0x10}，status_code==0x02
+3. 发送AHB_WR32(addr=0x00000003)验证ALIGN_ERR(0x03)：发送帧{0x20, 0x00000003, 0xDEADBEEF}，status_code==0x03，htrans_o保持IDLE
+4. 配置CTRL.EN=0：WR_CSR(opcode=0x10, addr=0x04, wdata=0x00000000)，发送命令验证DISABLED(0x04)
+5. 配置test_mode_i=0，发送命令验证NOT_IN_TEST(0x05)
+6. 发送命令过程中提前拉高pcs_n_i验证FRAME_ERR(0x06)
+7. 配置AHB slave返回hresp_i=1验证AHB_ERR(0x07)
+8. 配置AHB slave持续hready_i=0超过1024周期验证TIMEOUT(0x08)
 期望结果：
-1. 各类错误正确检测并返回对应状态码
-2. 在发起AHB访问前完成前置错误收敛
-3. LAST_ERR更新正确
-4. STATUS寄存器对应错误位置位
+1. BAD_OPCODE：status_code=0x01，不发起AHB访问，htrans_o=IDLE
+2. BAD_REG：status_code=0x02，不发起AHB访问
+3. ALIGN_ERR：status_code=0x03，不发起AHB访问，htrans_o=IDLE
+4. DISABLED：status_code=0x04
+5. NOT_IN_TEST：status_code=0x05
+6. FRAME_ERR：status_code=0x06
+7. AHB_ERR：status_code=0x07，STATUS[3]=1
+8. TIMEOUT：status_code=0x08，STATUS[3]=1
+9. 所有前置错误(BAD_OPCODE/BAD_REG/ALIGN_ERR/DISABLED/NOT_IN_TEST/FRAME_ERR)在发起AHB访问前完成检测
 coverage check点：
-直接用例覆盖，不收功能覆盖率。</t>
+对错误类型(0x01~0x08)收集功能覆盖率</t>
         </is>
       </c>
       <c r="D13" s="14" t="n"/>
@@ -3039,28 +2986,25 @@
       </c>
       <c r="B14" s="16" t="inlineStr">
         <is>
-          <t>low_power_test</t>
+          <t>test_low_power</t>
         </is>
       </c>
       <c r="C14" s="3" t="inlineStr">
         <is>
           <t>配置条件：
-1. 模块处于空闲态（test_mode_i=0或无有效任务）
+1. test_mode_i=0或无有效任务(pcs_n_i=1)
 输入激励：
-1. 保持pcs_n_i=1，监控rx_shift_reg是否不更新
-2. 监控非发送阶段tx_shift_reg是否不翻转
-3. 模拟AHB等待态，验证timeout_counter仅在此状态工作
-4. test_mode_i=0时验证AHB输出保持IDLE（htrans_o=2'b00）
-5. 切换到工作态验证关键寄存器翻转
-6. 对比空闲态和工作态的信号翻转率
+1. 保持pcs_n_i=1(空闲态)，监控内部rx_shift_reg和tx_shift_reg信号，验证不翻转
+2. 发送AHB_RD32命令，配置hready_i=0模拟AHB等待态，监控timeout_counter信号计数
+3. 配置test_mode_i=0，监控AHB接口：htrans_o==2'b00(IDLE), hwrite_o==0
+4. 切换到工作态(pcs_n_i=0, test_mode_i=1, CTRL.EN=1)，发送命令，监控关键寄存器翻转
 期望结果：
-1. 空闲态无效翻转最小化
-2. rx_shift_reg在pcs_n_i=1时不更新
-3. tx_shift_reg在非发送阶段不翻转
-4. timeout_counter仅在AHB等待态工作
-5. 低功耗设计目标满足
+1. 空闲态(pcs_n_i=1)：rx_shift_reg和tx_shift_reg不翻转
+2. timeout_counter仅在AHB_WAIT状态(等待hready_i=1)计数，其他状态=0
+3. test_mode_i=0时：htrans_o=2'b00, hwrite_o=0
+4. 工作态：关键寄存器(opcode_reg, addr_reg等)在RX/TX/WAIT_AHB状态正确翻转
 coverage check点：
-直接用例覆盖，不收功能覆盖率。</t>
+直接用例覆盖，不收功能覆盖率</t>
         </is>
       </c>
       <c r="D14" s="14" t="n"/>
@@ -3073,30 +3017,30 @@
       </c>
       <c r="B15" s="16" t="inlineStr">
         <is>
-          <t>performance_test</t>
+          <t>test_performance</t>
         </is>
       </c>
       <c r="C15" s="3" t="inlineStr">
         <is>
           <t>配置条件：
-1. 时钟配置：clk_i=100MHz
-2. AHB总线响应正常（hready_i=1，hresp_i=0）
+1. clk_i=100MHz
+2. test_mode_i=1, CTRL.EN=1, LANE_MODE=01(4-bit模式)
+3. AHB总线响应正常(hready_i=1, hresp_i=0)
 输入激励：
-1. 在1-bit模式下连续执行AHB_RD32/AHB_WR32命令，计算端到端延时和吞吐率
-2. 在4-bit模式下执行相同测试
-3. 验证原始链路线速：1-bit模式理论12.5MB/s，4-bit模式理论50MB/s
-4. 验证AHB接口32bit字访问约束
-5. 验证地址4Byte对齐要求
-6. 测量AHB_RD32端到端延时（预期约23~24 cycles）
-7. 测量AHB_WR32端到端延时（预期约23 cycles）
+1. 在4-bit模式下发送AHB_RD32命令(opcode=0x21, addr=0x00001000)
+2. 记录时间戳：T1=pcs_n_i拉低时刻，T2=pdo_o输出第一个status bit时刻
+3. 计算端到端延时：T2-T1(周期数)
+4. 在4-bit模式下连续发送100次AHB_RD32/AHB_WR32命令
+5. 记录总传输数据量和总时间，计算吞吐率
+6. 发送AHB命令时监控haddr_o[1:0]，验证4字节对齐
 期望结果：
-1. 目标频率100MHz稳定工作
-2. 延时符合预期（约23~24 cycles）
-3. 吞吐率达标
-4. AHB访问约束满足
-5. 无时序违例
+1. 端到端延时：4-bit模式AHB_RD32约23~24个clk_i周期
+2. 吞吐率：4-bit模式约50MB/s(理论值，实际应&gt;40MB/s)
+3. AHB访问粒度：hsize_o=3'b010(WORD)
+4. 地址对齐：haddr_o[1:0]=2'b00
+5. 频率稳定性：100MHz稳定工作，无时序违例
 coverage check点：
-直接用例覆盖，不收功能覆盖率。</t>
+直接用例覆盖，不收功能覆盖率</t>
         </is>
       </c>
       <c r="D15" s="14" t="n"/>
@@ -3109,31 +3053,39 @@
       </c>
       <c r="B16" s="16" t="inlineStr">
         <is>
-          <t>dfx_observability_test</t>
+          <t>test_dfx_observability</t>
         </is>
       </c>
       <c r="C16" s="3" t="inlineStr">
         <is>
           <t>配置条件：
-1. 仿真环境，模块使能
-2. 波形记录使能
+1. 仿真环境
+2. test_mode_i=1
+3. 通过WR_CSR(opcode=0x10, addr=0x04, wdata=0x00000001)设置CTRL.EN=1
 输入激励：
-1. 执行多种命令序列：WR_CSR、RD_CSR、AHB_WR32、AHB_RD32
-2. 采集状态机状态（fsm_state）
-3. 采集opcode寄存器（opcode_reg）
-4. 采集地址寄存器（addr_reg）
-5. 采集写数据寄存器（wdata_reg）
-6. 采集读数据寄存器（rdata_reg）
-7. 采集状态码（status_code）
-8. 采集rx/tx计数器
-9. 采集外部接口信号（pcs_n_i/pdi_i/pdo_o/pdo_oe_o）
+1. 执行WR_CSR命令(opcode=0x10, addr=0x04, wdata=0x00000003)
+2. 执行RD_CSR命令(opcode=0x11, addr=0x00)
+3. 执行AHB_WR32命令(opcode=0x20, addr=0x00001000, wdata=0xDEADBEEF)
+4. 执行AHB_RD32命令(opcode=0x21, addr=0x00001000)
+5. 采集调试可观测点：
+   - fsm_state(状态机状态)
+   - opcode_reg(当前opcode)
+   - addr_reg(地址寄存器)
+   - wdata_reg(写数据寄存器)
+   - rdata_reg(读数据寄存器)
+   - status_code(响应状态码)
+   - rx_cnt/tx_cnt(接收/发送计数)
+   - pdo_oe_o(输出使能)
 期望结果：
-1. 所有调试可观测点可采集
-2. 状态机状态变化可追踪
-3. 数据流可观测
-4. 便于联调、波形定位和故障复现
+1. fsm_state可观测：IDLE-&gt;RX-&gt;DECODE-&gt;WAIT_AHB-&gt;TX-&gt;IDLE状态转换可追踪
+2. opcode_reg可观测：正确记录0x10/0x11/0x20/0x21
+3. addr_reg可观测：正确记录地址值
+4. wdata_reg/rdata_reg可观测：正确记录数据值
+5. status_code可观测：记录响应状态码0x00(成功)或错误码
+6. rx_cnt/tx_cnt可观测：正确计数传输bit数
+7. 所有调试信号可通过仿真波形或调试接口访问
 coverage check点：
-直接用例覆盖，不收功能覆盖率。</t>
+直接用例覆盖，不收功能覆盖率</t>
         </is>
       </c>
       <c r="D16" s="14" t="n"/>
@@ -3146,27 +3098,31 @@
       </c>
       <c r="B17" s="16" t="inlineStr">
         <is>
-          <t>memory_map_test</t>
+          <t>test_memory_map</t>
         </is>
       </c>
       <c r="C17" s="3" t="inlineStr">
         <is>
           <t>配置条件：
-1. 模块使能：test_mode_i=1，CTRL.EN=1
+1. test_mode_i=1
+2. 通过WR_CSR(opcode=0x10, addr=0x04, wdata=0x00000001)设置CTRL.EN=1
 输入激励：
-1. 通过WR_CSR/RD_CSR访问模块内部CSR寄存器（VERSION/CTRL/STATUS/LAST_ERR）
-2. 发送AHB_WR32命令访问SoC内部memory-mapped地址（如0x2000_0000）
-3. 发送AHB_RD32命令访问SoC内部memory-mapped地址
-4. 验证模块自身CSR不进入SoC AHB memory map
-5. 验证AHB Master访问采用32bit地址空间
-6. 验证word访问粒度
+1. 通过WR_CSR(opcode=0x10, addr=0x00, wdata=0xFFFFFFFF)尝试写VERSION寄存器，验证只读属性
+2. 通过RD_CSR(opcode=0x11, addr=0x00)读取VERSION寄存器
+3. 通过WR_CSR(opcode=0x10, addr=0x04, wdata=0x00000003)写CTRL寄存器
+4. 通过RD_CSR(opcode=0x11, addr=0x04)读取CTRL寄存器
+5. 发送AHB_WR32命令(opcode=0x20, addr=0x00001000, wdata=0x12345678)访问SoC内部memory-mapped地址
+6. 发送AHB_RD32命令(opcode=0x21, addr=0x00001000)读回验证
+7. 监控AHB地址空间范围：haddr_o输出32-bit地址
 期望结果：
-1. CSR通过协议命令访问正常
-2. AHB Master访问SoC地址正确
-3. 模块CSR不映射到SoC AHB空间
-4. AHB访问约束满足
+1. CSR通过WR_CSR/RD_CSR协议命令正确访问
+2. VERSION寄存器只读，写入后读回原值
+3. CTRL寄存器读写正确
+4. AHB_WR32/AHB_RD32正确访问SoC memory-mapped地址，haddr_o=0x00001000
+5. 模块自身CSR(addr=0x00/0x04/0x08/0x0C)不进入SoC AHB memory map
+6. AHB Master访问采用32-bit地址空间，word访问粒度
 coverage check点：
-直接用例覆盖，不收功能覆盖率。</t>
+对CSR地址(0x00~0x0C)和AHB地址空间收集功能覆盖率</t>
         </is>
       </c>
       <c r="D17" s="14" t="n"/>
@@ -3179,31 +3135,32 @@
       </c>
       <c r="B18" s="16" t="inlineStr">
         <is>
-          <t>ahb_interface_test</t>
+          <t>test_ahb_interface</t>
         </is>
       </c>
       <c r="C18" s="3" t="inlineStr">
         <is>
           <t>配置条件：
-1. 模块使能：test_mode_i=1，CTRL.EN=1
-2. AHB总线空闲
+1. test_mode_i=1
+2. 通过WR_CSR(opcode=0x10, addr=0x04, wdata=0x00000001)设置CTRL.EN=1
+3. AHB总线空闲
 输入激励：
-1. 发送AHB_WR32命令，监控haddr_o/hwrite_o/htrans_o/hsize_o/hburst_o/hwdata_o输出
-2. 发送AHB_RD32命令，监控haddr_o/hwrite_o/htrans_o/hsize_o/hburst_o
-3. 验证htrans_o仅输出IDLE(2'b00)或NONSEQ(2'b10)
-4. 验证hsize_o固定为WORD(3'b010)
-5. 验证hburst_o固定为SINGLE(3'b000)
-6. 验证地址4Byte对齐
-7. 验证写数据在地址相下一拍输出
-8. 模拟hready_i=0等待周期，验证处理正确
-9. 模拟hresp_i=1错误响应，验证错误检测
+1. 发送AHB_WR32命令(opcode=0x20, addr=0x00001000, wdata=0xDEADBEEF)
+2. 监控AHB输出信号：haddr_o, hwrite_o, htrans_o, hsize_o, hburst_o, hwdata_o
+3. 发送AHB_RD32命令(opcode=0x21, addr=0x00001000)
+4. 监控AHB输入信号：hrdata_i, hready_i, hresp_i
+5. 配置hready_i=0验证等待态处理
+6. 配置hresp_i=1验证错误响应处理
 期望结果：
-1. AHB-Lite Master接口符合规范
-2. 单次读写事务正确
-3. 信号时序满足AHB协议要求
-4. 错误响应正确处理
+1. htrans_o仅输出2'b00(IDLE)或2'b10(NONSEQ)，无SEQ或Busy
+2. hsize_o=3'b010(WORD=32-bit)，固定不变
+3. hburst_o=3'b000(SINGLE)，固定不变
+4. 写时序正确：第1周期haddr_o=0x00001000, hwrite_o=1, htrans_o=NONSEQ；第2周期hwdata_o=0xDEADBEEF
+5. 读时序正确：第1周期haddr_o=0x00001000, hwrite_o=0, htrans_o=NONSEQ；第2周期采样hrdata_i
+6. hready_i=0时正确等待，htrans_o保持NONSEQ
+7. hresp_i=1时正确终止事务，返回status_code=0x07
 coverage check点：
-直接用例覆盖，不收功能覆盖率。</t>
+对AHB命令类型(读/写)和响应情况(hready=0/1, hresp=0/1)收集功能覆盖率</t>
         </is>
       </c>
       <c r="D18" s="14" t="n"/>

</xml_diff>

<commit_message>
skill v0p6(change testcase example in md) and rtm
</commit_message>
<xml_diff>
--- a/RTM_AI_gen.xlsx
+++ b/RTM_AI_gen.xlsx
@@ -2108,9 +2108,6 @@
           <t>Checker List</t>
         </is>
       </c>
-      <c r="B1" s="20" t="n"/>
-      <c r="C1" s="20" t="n"/>
-      <c r="D1" s="21" t="n"/>
     </row>
     <row r="2">
       <c r="A2" s="22" t="inlineStr">
@@ -2142,14 +2139,15 @@
       </c>
       <c r="B3" s="31" t="inlineStr">
         <is>
-          <t>clk_domain_checker</t>
+          <t>clk_domain_sync_checker</t>
         </is>
       </c>
       <c r="C3" s="6" t="inlineStr">
         <is>
-          <t>1. 检查clk_i频率稳定性：在连续时钟周期内，上升沿和下降沿时间间隔应在目标频率100MHz的±3%误差范围内
-2. 验证协议采样、状态机控制和AHB-Lite主接口同域工作：检查所有内部寄存器和状态机仅在clk_i上升沿更新
-3. 检查无时钟域交叉问题：确认无异步信号直接使用，所有跨域信号均经过同步处理</t>
+          <t>1. 检查clk_i上升沿时所有内部寄存器正确采样
+2. 验证100MHz频率下协议采样(pdi_i)、状态机转换、AHB-Lite信号(haddr_o/hwrite_o/hwdata_o/hrdata_i)同域工作
+3. 确认无跨时钟域信号，所有操作在单个clk_i域内完成
+4. 检查clk_i占空比在40%-60%范围内时模块正常工作</t>
         </is>
       </c>
       <c r="D3" s="4" t="n"/>
@@ -2162,15 +2160,16 @@
       </c>
       <c r="B4" s="18" t="inlineStr">
         <is>
-          <t>rst_checker</t>
+          <t>rst_async_sync_checker</t>
         </is>
       </c>
       <c r="C4" s="17" t="inlineStr">
         <is>
-          <t>1. 检查rst_ni复位连接性：rst_ni拉低后，状态机应立即回到IDLE状态
-2. 验证复位后默认值：CTRL.EN=0，CTRL.LANE_MODE=00(1-bit模式)，STATUS=0x00，LAST_ERR=0x00
-3. 检查复位同步释放：内部同步释放逻辑确保复位撤销时不产生亚稳态
-4. 验证协议上下文清空：rx_shift_reg、tx_shift_reg、opcode、addr、wdata等寄存器复位为0</t>
+          <t>1. 检查rst_ni拉低后异步复位立即生效，状态机跳转到IDLE状态
+2. 验证rst_ni释放后同步释放机制（至少2个clk_i周期同步）
+3. 确认复位后CTRL.EN=0、CTRL.LANE_MODE=00(1-bit模式)
+4. 检查STATUS寄存器清零、LAST_ERR寄存器清零
+5. 验证协议上下文(rx_shift_reg/tx_shift_reg/opcode_reg/addr_reg/wdata_reg)清空</t>
         </is>
       </c>
       <c r="D4" s="4" t="n"/>
@@ -2183,18 +2182,17 @@
       </c>
       <c r="B5" s="31" t="inlineStr">
         <is>
-          <t>csr_checker</t>
+          <t>csr_access_checker</t>
         </is>
       </c>
       <c r="C5" s="6" t="inlineStr">
         <is>
-          <t>1. 检查VERSION寄存器读取：通过opcode=0x11(RD_CSR)读取VERSION，验证返回值符合设计预期
-2. 检查CTRL寄存器读写：
-   - 写CTRL.EN=1，验证模块使能生效
-   - 写CTRL.LANE_MODE=00/01，验证lane模式切换
-   - 写CTRL.SOFT_RST=1，验证软复位触发
-3. 检查STATUS寄存器：验证BUSY位在任务执行期间置1，完成后清0
-4. 检查LAST_ERR寄存器：验证错误发生时LAST_ERR更新为对应错误码</t>
+          <t>1. 检查通过WR_CSR(opcode=0x10)写CSR寄存器：addr=0x00(VERSION)只读、addr=0x04(CTRL)读写、addr=0x08(STATUS)只读、addr=0x0C(LAST_ERR)只读
+2. 验证RD_CSR(opcode=0x11)读CSR寄存器返回正确数据
+3. 确认VERSION寄存器写入无效，读回返回固定版本号
+4. 检查CTRL.EN位写1后模块使能，写0后禁用
+5. 验证CTRL.LANE_MODE=00/01有效，10/11不改变配置
+6. 确认CTRL.SOFT_RST写1后触发软复位，协议上下文清零</t>
         </is>
       </c>
       <c r="D5" s="4" t="n"/>
@@ -2207,14 +2205,14 @@
       </c>
       <c r="B6" s="31" t="inlineStr">
         <is>
-          <t>mode_checker</t>
+          <t>test_mode_enable_checker</t>
         </is>
       </c>
       <c r="C6" s="6" t="inlineStr">
         <is>
-          <t>1. 检查test_mode_i=1且CTRL.EN=1时模块允许执行功能命令
-2. 验证test_mode_i=0时发送命令返回错误码STS_NOT_IN_TEST(0x05)
-3. 验证CTRL.EN=0时发送命令返回错误码STS_DISABLED(0x04)
+          <t>1. 检查test_mode_i=1且CTRL.EN=1时功能命令可执行
+2. 验证test_mode_i=0时命令返回STS_NOT_IN_TEST(0x05)
+3. 确认CTRL.EN=0时命令返回STS_DISABLED(0x04)
 4. 检查半双工请求/响应模式：pcs_n_i拉低开始请求阶段，turnaround 1周期后进入响应阶段</t>
         </is>
       </c>
@@ -2233,10 +2231,10 @@
       </c>
       <c r="C7" s="6" t="inlineStr">
         <is>
-          <t>1. 检查CTRL.LANE_MODE=00时仅使用pdi_i[0]/pdo_o[0]传输，每拍收发1bit(MSB first)
-2. 验证CTRL.LANE_MODE=01时使用pdi_i[3:0]/pdo_o[3:0]传输，每拍收发4bit(高nibble优先)
-3. 确认非法LANE_MODE值(10/11)不改变当前配置或返回错误
-4. 检查lane模式切换时序：模式切换应在帧边界进行，不影响当前帧传输</t>
+          <t>1. 检查CTRL.LANE_MODE=00时仅使用pdi_i[0]/pdo_o[0]传输，每拍收发1bit
+2. 验证CTRL.LANE_MODE=01时使用pdi_i[3:0]/pdo_o[3:0]传输，每拍收发4bit，高nibble优先
+3. 确认非法LANE_MODE值(10/11)写入时不改变当前配置
+4. 检查lane模式切换后立即生效，影响后续所有数据传输</t>
         </is>
       </c>
       <c r="D7" s="14" t="n"/>
@@ -2249,16 +2247,15 @@
       </c>
       <c r="B8" s="12" t="inlineStr">
         <is>
-          <t>data_interface_checker</t>
+          <t>frame_boundary_checker</t>
         </is>
       </c>
       <c r="C8" s="6" t="inlineStr">
         <is>
-          <t>1. 检查pcs_n_i帧边界：pcs_n_i拉低标志帧开始，拉高标志帧结束
-2. 验证pdi_i[3:0]输入时序：输入数据在clk_i上升沿采样，采样窗口内数据应稳定
-3. 验证pdo_o[3:0]输出时序：输出数据在响应阶段有效，pdo_oe_o=1时输出使能
-4. 检查pdo_oe_o方向控制：请求阶段pdo_oe_o=0(输入方向)，响应阶段pdo_oe_o=1(输出方向)
-5. 验证MSB first传输顺序：数据从最高位开始传输</t>
+          <t>1. 检查pcs_n_i拉低后模块开始接收请求（state从IDLE→RX）
+2. 验证pcs_n_i在请求未完成时提前拉高，返回STS_FRAME_ERR(0x06)到LAST_ERR寄存器
+3. 确认pdo_oe_o在响应阶段正确指示输出方向：TX阶段=1，其他=0
+4. 检查帧格式：opcode(8bit) + addr(16bit) + wdata(32bit，仅写命令)</t>
         </is>
       </c>
       <c r="D8" s="14" t="n"/>
@@ -2271,18 +2268,15 @@
       </c>
       <c r="B9" s="12" t="inlineStr">
         <is>
-          <t>protocol_checker</t>
+          <t>turnaround_checker</t>
         </is>
       </c>
       <c r="C9" s="6" t="inlineStr">
         <is>
-          <t>1. 检查turnaround周期：请求阶段结束后固定1个clk_i周期的turnaround
-2. 验证帧格式：
-   - WR_CSR(0x10): opcode(8bit) + reg_addr(8bit) + wdata(32bit)
-   - RD_CSR(0x11): opcode(8bit) + reg_addr(8bit) -&gt; STATUS(8bit) + rdata(32bit)
-   - AHB_WR32(0x20): opcode(8bit) + addr(32bit) + wdata(32bit)
-   - AHB_RD32(0x21): opcode(8bit) + addr(32bit) -&gt; STATUS(8bit) + rdata(32bit)
-3. 检查协议字段MSB first传输顺序</t>
+          <t>1. 检查请求阶段结束后固定1个clk_i周期的turnaround
+2. 验证turnaround期间pdo_oe_o=0，pdi_i/pdo_o处于高阻态
+3. 确认turnaround结束后pdo_oe_o=1，进入TX阶段输出响应
+4. 检查协议字段按MSB first顺序传输</t>
         </is>
       </c>
       <c r="D9" s="14" t="n"/>
@@ -2295,18 +2289,17 @@
       </c>
       <c r="B10" s="12" t="inlineStr">
         <is>
-          <t>opcode_checker</t>
+          <t>opcode_decode_checker</t>
         </is>
       </c>
       <c r="C10" s="6" t="inlineStr">
         <is>
-          <t>1. 检查opcode解析正确性：
-   - opcode=0x10解析为WR_CSR命令
-   - opcode=0x11解析为RD_CSR命令
-   - opcode=0x20解析为AHB_WR32命令
-   - opcode=0x21解析为AHB_RD32命令
-2. 验证非法opcode处理：opcode为0x00/0xFF或其他非法值时返回STS_BAD_OPCODE(0x01)
-3. 检查帧长确定：前端收满8bit opcode后正确确定期望帧长</t>
+          <t>1. 检查opcode=0x10(WR_CSR)正确译码为CSR写操作
+2. 验证opcode=0x11(RD_CSR)正确译码为CSR读操作
+3. 确认opcode=0x20(AHB_WR32)正确译码为AHB写操作
+4. 检查opcode=0x21(AHB_RD32)正确译码为AHB读操作
+5. 验证非法opcode(非0x10/0x11/0x20/0x21)返回STS_BAD_OPCODE(0x01)
+6. 确认前端收满8bit opcode后确定期望帧长</t>
         </is>
       </c>
       <c r="D10" s="14" t="n"/>
@@ -2319,18 +2312,15 @@
       </c>
       <c r="B11" s="12" t="inlineStr">
         <is>
-          <t>ctrl_checker</t>
+          <t>ctrl_config_checker</t>
         </is>
       </c>
       <c r="C11" s="6" t="inlineStr">
         <is>
-          <t>1. 检查CTRL.EN配置生效：CTRL.EN=1时模块使能，CTRL.EN=0时模块禁用
-2. 验证CTRL.LANE_MODE配置：
-   - LANE_MODE=00配置为1-bit模式
-   - LANE_MODE=01配置为4-bit模式
-   - LANE_MODE=10/11为非法配置
-3. 检查CTRL.SOFT_RST功能：写SOFT_RST=1触发协议上下文清零并恢复默认lane模式
-4. 验证配置立即生效：配置写入后下一拍生效</t>
+          <t>1. 检查CTRL.EN=1时功能命令可执行，CTRL.EN=0时返回STS_DISABLED(0x04)
+2. 验证CTRL.LANE_MODE=00切换到1-bit模式，=01切换到4-bit模式
+3. 确认CTRL.SOFT_RST写1触发软复位：协议上下文清零、恢复默认lane模式(1-bit)
+4. 检查软复位不影响CTRL.EN状态</t>
         </is>
       </c>
       <c r="D11" s="14" t="n"/>
@@ -2343,15 +2333,15 @@
       </c>
       <c r="B12" s="12" t="inlineStr">
         <is>
-          <t>status_checker</t>
+          <t>status_polling_checker</t>
         </is>
       </c>
       <c r="C12" s="6" t="inlineStr">
         <is>
-          <t>1. 检查STATUS寄存器查询：通过RD_CSR读取STATUS，验证BUSY位和STICKY位正确反映模块状态
-2. 验证LAST_ERR寄存器查询：错误发生时LAST_ERR更新为对应错误码并保持
-3. 确认无独立中断输出：MVP版本不实现中断信号，所有状态通过寄存器查询获取
-4. 检查ATE轮询方式：STATUS和LAST_ERR可被ATE主机持续轮询</t>
+          <t>1. 检查STATUS[0]反映模块busy状态：命令执行期间=1，空闲=0
+2. 验证LAST_ERR寄存器记录最近错误码
+3. 确认MVP版本无独立中断输出，所有状态通过STATUS/LAST_ERR轮询获取
+4. 检查错误发生时LAST_ERR更新，STATUS[0]清除命令完成后归零</t>
         </is>
       </c>
       <c r="D12" s="14" t="n"/>
@@ -2364,22 +2354,20 @@
       </c>
       <c r="B13" s="12" t="inlineStr">
         <is>
-          <t>error_checker</t>
+          <t>exception_checker</t>
         </is>
       </c>
       <c r="C13" s="6" t="inlineStr">
         <is>
-          <t>1. 检查错误码生成正确性：
-   - 非法opcode -&gt; STS_BAD_OPCODE(0x01)
-   - 非法CSR地址 -&gt; STS_BAD_REG(0x02)
-   - 非对齐地址 -&gt; STS_ALIGN_ERR(0x03)
-   - CTRL.EN=0 -&gt; STS_DISABLED(0x04)
-   - test_mode_i=0 -&gt; STS_NOT_IN_TEST(0x05)
-   - pcs_n_i提前拉高 -&gt; STS_FRAME_ERR(0x06)
-   - AHB错误(hresp_i=1) -&gt; STS_AHB_ERR(0x07)
-   - AHB超时 -&gt; STS_TIMEOUT(0x08)
-2. 验证前置错误收敛：在发起AHB访问前完成所有前置错误检测
-3. 检查LAST_ERR更新：错误发生时LAST_ERR寄存器更新为对应错误码</t>
+          <t>1. 检查BAD_OPCODE(0x01)：opcode非0x10/0x11/0x20/0x21
+2. 验证BAD_REG(0x02)：CSR地址非0x00/0x04/0x08/0x0C
+3. 确认ALIGN_ERR(0x03)：AHB地址非4Byte对齐(addr[1:0]!=0)
+4. 检查DISABLED(0x04)：CTRL.EN=0时发送命令
+5. 验证NOT_IN_TEST(0x05)：test_mode_i=0时发送命令
+6. 确认FRAME_ERR(0x06)：pcs_n_i提前拉高
+7. 检查AHB_ERR(0x07)：hresp_i=1
+8. 验证TIMEOUT(0x08)：AHB访问超时
+9. 确认前置错误(0x01-0x06)在发起AHB访问前收敛</t>
         </is>
       </c>
       <c r="D13" s="14" t="n"/>
@@ -2392,15 +2380,15 @@
       </c>
       <c r="B14" s="12" t="inlineStr">
         <is>
-          <t>lowpower_checker</t>
+          <t>low_power_checker</t>
         </is>
       </c>
       <c r="C14" s="6" t="inlineStr">
         <is>
-          <t>1. 检查空闲态寄存器不更新：pcs_n_i=1(空闲)时rx_shift_reg和tx_shift_reg不翻转
-2. 验证超时计数器控制：超时计数器仅在WAIT_AHB状态工作时更新
-3. 检查AHB输出空闲：test_mode_i=0或无有效任务时AHB输出保持IDLE(htrans_o=IDLE)
-4. 验证关键寄存器翻转：仅在RX/TX/WAIT_AHB相关状态翻转关键寄存器</t>
+          <t>1. 检查空闲态(IDLE)下接收/发送移位寄存器不翻转
+2. 验证test_mode_i=0或无有效任务时AHB输出保持IDLE：htrans_o=0
+3. 确认超时计数器仅在WAIT_AHB状态工作
+4. 检查RX/TX/WAIT_AHB状态翻转关键寄存器</t>
         </is>
       </c>
       <c r="D14" s="14" t="n"/>
@@ -2413,17 +2401,16 @@
       </c>
       <c r="B15" s="12" t="inlineStr">
         <is>
-          <t>perf_checker</t>
+          <t>performance_checker</t>
         </is>
       </c>
       <c r="C15" s="6" t="inlineStr">
         <is>
-          <t>1. 检查目标频率达标：clk_i在100MHz频率下稳定工作
-2. 验证端到端延时：从pcs_n_i拉低到pdo_oe_o拉高的延时约23~24个clk_i周期
-3. 检查吞吐率：
-   - 1-bit模式原始链路线速：12.5MB/s
-   - 4-bit模式原始链路线速：50MB/s
-4. 验证AHB访问约束：hsize_o固定为WORD(32-bit)，地址需4Byte对齐</t>
+          <t>1. 检查100MHz频率稳定工作，无时序违例
+2. 验证1-bit模式链路线速12.5MB/s：每拍1bit，8拍/byte
+3. 确认4-bit模式链路线速50MB/s：每拍4bit，2拍/byte
+4. 检查AHB接口32bit字访问，hsize_o=010(WORD)
+5. 验证地址4Byte对齐：addr[1:0]=00</t>
         </is>
       </c>
       <c r="D15" s="14" t="n"/>
@@ -2436,15 +2423,15 @@
       </c>
       <c r="B16" s="12" t="inlineStr">
         <is>
-          <t>dfx_checker</t>
+          <t>dfx_observable_checker</t>
         </is>
       </c>
       <c r="C16" s="6" t="inlineStr">
         <is>
-          <t>1. 检查状态机状态可观测：状态机当前状态可通过调试接口观测
-2. 验证关键寄存器可观测：opcode、addr、wdata、rdata、status_code可通过调试接口观测
-3. 检查计数器可观测：rx_count、tx_count可通过调试接口观测
-4. 验证接口信号可观测：pcs_n_i、pdi_i、pdo_o、pdo_oe_o可通过调试接口观测</t>
+          <t>1. 检查状态机状态(state)可观测：IDLE/RX/TX/WAIT_AHB等
+2. 验证内部寄存器可观测：opcode_reg、addr_reg、wdata_reg、rdata_reg、status_code_reg
+3. 确认rx_count/tx_count计数器可观测
+4. 检查外部接口信号pcs_n_i、pdi_i[3:0]、pdo_o[3:0]、pdo_oe_o可观测</t>
         </is>
       </c>
       <c r="D16" s="14" t="n"/>
@@ -2457,15 +2444,15 @@
       </c>
       <c r="B17" s="12" t="inlineStr">
         <is>
-          <t>memmap_checker</t>
+          <t>memory_map_checker</t>
         </is>
       </c>
       <c r="C17" s="6" t="inlineStr">
         <is>
-          <t>1. 检查CSR访问方式：模块内部CSR(VERSION/CTRL/STATUS/LAST_ERR)不进入SoC AHB memory map，仅通过协议命令访问
-2. 验证AHB Master地址空间：AHB_WR32/AHB_RD32命令访问SoC内部memory-mapped地址，采用32bit地址空间
-3. 检查访问粒度：AHB Master访问固定为word(32-bit)访问粒度
-4. 验证地址范围约束：具体可达目标地址范围由SoC顶层统一约束</t>
+          <t>1. 检查模块CSR(addr=0x00/0x04/0x08/0x0C)通过WR_CSR/RD_CSR协议命令访问
+2. 验证模块自身CSR不进入SoC AHB memory map
+3. 确认AHB Master访问采用32-bit地址空间：haddr_o[31:0]
+4. 检查word访问粒度：hsize_o=010，每次访问4Byte</t>
         </is>
       </c>
       <c r="D17" s="14" t="n"/>
@@ -2478,23 +2465,16 @@
       </c>
       <c r="B18" s="12" t="inlineStr">
         <is>
-          <t>ahb_checker</t>
+          <t>ahb_lite_checker</t>
         </is>
       </c>
       <c r="C18" s="6" t="inlineStr">
         <is>
-          <t>1. 检查AHB-Lite Master信号输出：
-   - haddr_o[31:0]：目标地址输出
-   - hwrite_o：读写标志(1=写，0=读)
-   - htrans_o[1:0]：仅输出IDLE(2'b00)和NONSEQ(2'b10)
-   - hsize_o[2:0]：固定为WORD(3'b010)
-   - hburst_o[2:0]：固定为SINGLE(3'b000)
-   - hwdata_o[31:0]：写数据输出
-2. 验证AHB输入响应处理：
-   - hrdata_i[31:0]：读数据输入
-   - hready_i：等待状态处理
-   - hresp_i：错误响应(返回STS_AHB_ERR)
-3. 检查AHB时序：地址相和数据相符合AHB-Lite协议要求</t>
+          <t>1. 检查AHB_WR32命令：haddr_o输出32-bit地址，hwrite_o=1，htrans_o=NONSEQ(10)，hsize_o=010(WORD)，hburst_o=000(SINGLE)，hwdata_o输出写数据
+2. 验证AHB_RD32命令：haddr_o输出地址，hwrite_o=0，htrans_o=NONSEQ，hsize_o=010，hburst_o=000，hrdata_i接收读数据
+3. 确认hready_i=1时数据有效传输，hresp_i=0表示正常响应
+4. 检查hresp_i=1时返回STS_AHB_ERR(0x07)错误
+5. 验证htrans_o仅输出IDLE(00)或NONSEQ(10)，无SEQ/Busy</t>
         </is>
       </c>
       <c r="D18" s="14" t="n"/>
@@ -2535,64 +2515,29 @@
       <c r="C24" s="6" t="n"/>
       <c r="D24" s="4" t="n"/>
     </row>
+    <row r="25"/>
+    <row r="26"/>
+    <row r="27"/>
     <row r="28">
-      <c r="A28" s="23" t="inlineStr">
-        <is>
-          <t>填写要求</t>
-        </is>
-      </c>
+      <c r="A28" s="23" t="n"/>
     </row>
     <row r="29" ht="24" customHeight="1" s="24">
-      <c r="A29" s="31" t="inlineStr">
-        <is>
-          <t>CHK Name</t>
-        </is>
-      </c>
-      <c r="B29" s="35" t="inlineStr">
-        <is>
-          <t>如果是SVA checker，需填写SVA property名字</t>
-        </is>
-      </c>
-      <c r="C29" s="20" t="n"/>
-      <c r="D29" s="21" t="n"/>
+      <c r="A29" s="31" t="n"/>
+      <c r="B29" s="35" t="n"/>
     </row>
     <row r="30" ht="69.95" customHeight="1" s="24">
-      <c r="A30" s="31" t="inlineStr">
-        <is>
-          <t>CHK描述</t>
-        </is>
-      </c>
-      <c r="B30" s="36" t="inlineStr">
-        <is>
-          <t xml:space="preserve">1、需要定性+定量描述，需具体到check的信号、取值 
-2、和DV SPEC中Checker方案描述的区别 — RTM中描述check的内容，DV SPEC中描述checker的实现方案(例如是通过SVA实现还是scoreboard实时数据比对，还是文件对比)
-</t>
-        </is>
-      </c>
-      <c r="C30" s="20" t="n"/>
-      <c r="D30" s="21" t="n"/>
+      <c r="A30" s="31" t="n"/>
+      <c r="B30" s="36" t="n"/>
     </row>
     <row r="31">
       <c r="A31" s="31" t="n"/>
       <c r="B31" s="12" t="n"/>
-      <c r="C31" s="20" t="n"/>
-      <c r="D31" s="21" t="n"/>
     </row>
     <row r="32">
       <c r="A32" s="31" t="n"/>
       <c r="B32" s="12" t="n"/>
-      <c r="C32" s="20" t="n"/>
-      <c r="D32" s="21" t="n"/>
     </row>
   </sheetData>
-  <mergeCells count="6">
-    <mergeCell ref="A1:D1"/>
-    <mergeCell ref="B31:D31"/>
-    <mergeCell ref="B32:D32"/>
-    <mergeCell ref="B30:D30"/>
-    <mergeCell ref="B29:D29"/>
-    <mergeCell ref="A28:D28"/>
-  </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -2615,27 +2560,48 @@
     <row r="1">
       <c r="A1" s="29" t="inlineStr">
         <is>
-          <t>Test Case List</t>
-        </is>
-      </c>
-      <c r="B1" s="20" t="n"/>
-      <c r="C1" s="20" t="n"/>
-      <c r="D1" s="21" t="n"/>
+          <t>TC编号</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>TC Name</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>TC描述</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="22" t="inlineStr">
         <is>
-          <t>TC编号</t>
+          <t>TC_001</t>
         </is>
       </c>
       <c r="B2" s="22" t="inlineStr">
         <is>
-          <t>TC Name</t>
+          <t>test_clock_domain</t>
         </is>
       </c>
       <c r="C2" s="22" t="inlineStr">
         <is>
-          <t>TC 描述</t>
+          <t>配置条件：
+1. 配置clk_i时钟频率为100MHz
+2. test_mode_i=1
+输入激励：
+1. 通过WR_CSR(opcode=0x10, addr=0x04, wdata=0x00000001)设置CTRL.EN=1
+2. 配置LANE_MODE=00(1-bit模式)，连续发送AHB_RD32命令(opcode=0x21, addr=0x00001000)
+3. 配置LANE_MODE=01(4-bit模式)，连续发送AHB_WR32命令(opcode=0x20, addr=0x00002000, wdata=0xDEADBEEF)
+4. 在clk_i占空比40%-60%范围内重复上述测试
+期望结果：
+1. 所有命令在100MHz频率下正确执行
+2. 协议采样(pdi_i)、状态机控制、AHB-Lite主接口同域工作正常
+3. 无时序违例，无跨时钟域问题
+coverage check点：
+1. 100MHz频率下命令执行成功率
+2. 1-bit和4-bit模式切换覆盖率</t>
         </is>
       </c>
       <c r="D2" s="22" t="inlineStr">
@@ -2647,32 +2613,33 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>TC_001</t>
+          <t>TC_002</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>test_clk_domain</t>
+          <t>test_reset</t>
         </is>
       </c>
       <c r="C3" s="3" t="inlineStr">
         <is>
-          <t>TC场景：测试时钟域同步性
-配置条件：
-1. test_mode_i=1（测试模式使能）
-2. CTRL.EN=1（模块使能）
-3. clk_i频率配置为100MHz
+          <t>配置条件：
+1. 初始rst_ni=0，模块处于复位状态
+2. test_mode_i=1
 输入激励：
-1. 连续发送AHB_RD32(opcode=0x21)命令，覆盖1-bit模式(LANE_MODE=00)和4-bit模式(LANE_MODE=01)
-2. 连续发送AHB_WR32(opcode=0x20)命令，覆盖两种lane模式
-3. 在命令执行过程中监测内部寄存器和状态机更新时机
+1. 释放rst_ni，等待至少2个clk_i周期
+2. 通过RD_CSR(opcode=0x11, addr=0x04)读取CTRL寄存器，验证EN=0、LANE_MODE=00
+3. 通过RD_CSR(opcode=0x11, addr=0x08)读取STATUS寄存器，验证为0
+4. 通过RD_CSR(opcode=0x11, addr=0x0C)读取LAST_ERR寄存器，验证为0
+5. 检查内部状态机处于IDLE状态
 期望结果：
-1. 所有命令在100MHz频率下正确执行
-2. 协议采样、状态机控制和AHB-Lite主接口同域工作正常
-3. 所有内部寄存器仅在clk_i上升沿更新
-4. STATUS=0x00（成功）返回
+1. rst_ni释放后状态机回到IDLE
+2. CTRL.EN=0，CTRL.LANE_MODE=00(1-bit默认值)
+3. STATUS/LAST_ERR清零，无残留状态
+4. 协议上下文清空
 coverage check点：
-对clk_i频率范围(90MHz~110MHz)收集功能覆盖率。</t>
+1. 异步复位生效覆盖率
+2. 同步释放机制覆盖率</t>
         </is>
       </c>
       <c r="D3" s="4" t="n"/>
@@ -2680,31 +2647,35 @@
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>TC_002</t>
+          <t>TC_003</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>test_reset</t>
+          <t>test_csr_access</t>
         </is>
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
-          <t>TC场景：测试复位功能
-配置条件：
-1. rst_ni初始为低，模块处于复位状态
+          <t>配置条件：
+1. test_mode_i=1
+2. 通过WR_CSR(opcode=0x10, addr=0x04, wdata=0x00000001)设置CTRL.EN=1
 输入激励：
-1. 释放rst_ni，验证复位释放效果
-2. 通过RD_CSR(opcode=0x11)读取CTRL寄存器，检查默认值
-3. 通过RD_CSR读取STATUS和LAST_ERR寄存器，检查清零状态
-4. 监测状态机状态，确认回到IDLE
+1. 通过RD_CSR(opcode=0x11, addr=0x00)读取VERSION寄存器，记录版本号
+2. 通过WR_CSR(opcode=0x10, addr=0x00, wdata=0xFFFFFFFF)尝试写VERSION寄存器
+3. 再次读取VERSION寄存器，验证只读属性（值不变）
+4. 通过WR_CSR(opcode=0x10, addr=0x04, wdata=0x00000003)写CTRL寄存器（EN=1, LANE_MODE=01）
+5. 通过RD_CSR(opcode=0x11, addr=0x04)读取CTRL寄存器，验证写入正确
+6. 通过RD_CSR(opcode=0x11, addr=0x08)读取STATUS寄存器
+7. 通过RD_CSR(opcode=0x11, addr=0x0C)读取LAST_ERR寄存器
 期望结果：
-1. 复位后状态机处于IDLE状态
-2. CTRL.EN=0，CTRL.LANE_MODE=00(1-bit模式)
-3. STATUS=0x00，LAST_ERR=0x00
-4. 协议上下文(rx_shift_reg, tx_shift_reg等)清零
+1. CSR读写正确
+2. VERSION寄存器只读，写入后读回原值
+3. CTRL寄存器读写正确，配置生效
+4. STATUS/LAST_ERR反映正确状态
 coverage check点：
-直接用例覆盖，不收功能覆盖率。</t>
+1. CSR地址(0x00/0x04/0x08/0x0C)读写覆盖率
+2. 只读寄存器写保护覆盖率</t>
         </is>
       </c>
       <c r="D4" s="4" t="n"/>
@@ -2712,34 +2683,32 @@
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>TC_003</t>
+          <t>TC_004</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>test_csr_access</t>
+          <t>test_work_mode</t>
         </is>
       </c>
       <c r="C5" s="3" t="inlineStr">
         <is>
-          <t>TC场景：测试CSR寄存器访问
-配置条件：
+          <t>配置条件：
 1. test_mode_i=1
-2. CTRL.EN=1
-3. LANE_MODE=00(1-bit模式)或01(4-bit模式)
+2. 通过WR_CSR(opcode=0x10, addr=0x04, wdata=0x00000001)设置CTRL.EN=1
 输入激励：
-1. 通过RD_CSR(opcode=0x11)读取VERSION寄存器，验证版本号
-2. 通过WR_CSR(opcode=0x10)写入CTRL.EN=1，验证模块使能
-3. 通过WR_CSR写入CTRL.LANE_MODE=00/01，验证lane模式配置
-4. 通过WR_CSR写入CTRL.SOFT_RST=1，验证软复位功能
-5. 通过RD_CSR读取STATUS和LAST_ERR，检查状态正确
+1. 发送WR_CSR命令(opcode=0x10, addr=0x04, wdata=0x00000003)配置LANE_MODE=01(4-bit)
+2. 发送AHB_WR32命令(opcode=0x20, addr=0x00001000, wdata=0x12345678)
+3. 发送AHB_RD32命令(opcode=0x21, addr=0x00001000)读回验证
+4. 监控pcs_n_i帧边界和pdo_oe_o输出使能
 期望结果：
-1. VERSION返回预期版本号
-2. CTRL配置正确写入并生效
-3. STATUS正确反映BUSY状态
-4. LAST_ERR在错误发生时更新
+1. 模块正确执行功能命令
+2. 协议采用半双工请求/响应模式
+3. CSR访问与AHB-Lite单次读写正常
+4. pcs_n_i定义帧边界正确，pdo_oe_o在TX阶段=1
 coverage check点：
-对CSR寄存器地址范围、LANE_MODE配置值收集功能覆盖率。</t>
+1. 半双工模式覆盖率
+2. 请求/响应阶段切换覆盖率</t>
         </is>
       </c>
       <c r="D5" s="4" t="n"/>
@@ -2747,31 +2716,32 @@
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>TC_004</t>
+          <t>TC_005</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>test_work_mode</t>
+          <t>test_lane_mode</t>
         </is>
       </c>
       <c r="C6" s="3" t="inlineStr">
         <is>
-          <t>TC场景：测试工作模式
-配置条件：
-1. 初始状态test_mode_i=0，CTRL.EN=0
+          <t>配置条件：
+1. test_mode_i=1
+2. 通过WR_CSR(opcode=0x10, addr=0x04, wdata=0x00000001)设置CTRL.EN=1
 输入激励：
-1. test_mode_i=0时发送WR_CSR命令，验证返回STS_NOT_IN_TEST(0x05)
-2. 设置test_mode_i=1，CTRL.EN=0时发送命令，验证返回STS_DISABLED(0x04)
-3. 设置CTRL.EN=1，发送WR_CSR配置lane模式
-4. 发送AHB_WR32/AHB_RD32命令验证半双工模式
+1. 配置LANE_MODE=00(1-bit模式)，发送AHB_WR32命令，监控pdi_i[0]/pdo_o[0]
+2. 配置LANE_MODE=01(4-bit模式)，发送相同命令，监控pdi_i[3:0]/pdo_o[3:0]
+3. 尝试配置LANE_MODE=10/11，验证配置不变
+4. 验证高nibble优先发送顺序
 期望结果：
-1. test_mode_i=0时返回STS_NOT_IN_TEST(0x05)
-2. CTRL.EN=0时返回STS_DISABLED(0x04)
-3. test_mode_i=1且CTRL.EN=1时命令正常执行
-4. 半双工请求/响应模式工作正常
+1. 1-bit模式仅使用bit0传输，每拍1bit
+2. 4-bit模式使用全部4bit传输，每拍4bit，高nibble优先
+3. 非法LANE_MODE值不改变配置
+4. 模式切换立即生效
 coverage check点：
-对test_mode_i和CTRL.EN的组合状态收集功能覆盖率。</t>
+1. LANE_MODE=00/01模式覆盖率
+2. 高nibble优先发送覆盖率</t>
         </is>
       </c>
       <c r="D6" s="4" t="n"/>
@@ -2779,32 +2749,32 @@
     <row r="7">
       <c r="A7" s="16" t="inlineStr">
         <is>
-          <t>TC_005</t>
+          <t>TC_006</t>
         </is>
       </c>
       <c r="B7" s="16" t="inlineStr">
         <is>
-          <t>test_lane_mode</t>
+          <t>test_data_interface</t>
         </is>
       </c>
       <c r="C7" s="3" t="inlineStr">
         <is>
-          <t>TC场景：测试lane模式配置
-配置条件：
+          <t>配置条件：
 1. test_mode_i=1
-2. CTRL.EN=1
+2. 通过WR_CSR(opcode=0x10, addr=0x04, wdata=0x00000001)设置CTRL.EN=1
 输入激励：
-1. 配置LANE_MODE=00，发送WR_CSR命令，验证pdi_i[0]/pdo_o[0]数据传输
-2. 配置LANE_MODE=01，发送WR_CSR命令，验证pdi_i[3:0]/pdo_o[3:0]数据传输(高nibble优先)
-3. 尝试配置LANE_MODE=10/11(非法值)，验证不改变当前配置或返回错误
-4. 在帧中间切换LANE_MODE，验证不影响当前帧
+1. 在1-bit模式下发送WR_CSR命令(opcode=0x10)，监控pdi_i[0]接收和pdo_o[0]输出
+2. 在4-bit模式下发送AHB_WR32命令(opcode=0x20)，监控pdi_i[3:0]/pdo_o[3:0]
+3. 检查pcs_n_i拉低开始帧，拉高结束帧
+4. 验证MSB first传输顺序
 期望结果：
-1. LANE_MODE=00时1-bit模式正常工作，每拍收发1bit(MSB first)
-2. LANE_MODE=01时4-bit模式正常工作，每拍收发4bit(高nibble优先)
-3. 非法LANE_MODE值(10/11)不改变当前配置
-4. lane模式切换在帧边界生效
+1. 数据接口按lane模式正确传输
+2. 帧边界清晰，pcs_n_i正确定义帧边界
+3. MSB first顺序正确
+4. pdo_oe_o在TX阶段=1，其他阶段=0
 coverage check点：
-对LANE_MODE配置值(00/01/10/11)收集功能覆盖率。</t>
+1. 数据传输模式覆盖率
+2. 帧边界覆盖率</t>
         </is>
       </c>
       <c r="D7" s="14" t="n"/>
@@ -2812,35 +2782,33 @@
     <row r="8">
       <c r="A8" s="16" t="inlineStr">
         <is>
-          <t>TC_006</t>
+          <t>TC_007</t>
         </is>
       </c>
       <c r="B8" s="16" t="inlineStr">
         <is>
-          <t>test_data_interface</t>
+          <t>test_turnaround</t>
         </is>
       </c>
       <c r="C8" s="3" t="inlineStr">
         <is>
-          <t>TC场景：测试数据接口
-配置条件：
+          <t>配置条件：
 1. test_mode_i=1
-2. CTRL.EN=1
-3. LANE_MODE=00(1-bit)和01(4-bit)分别测试
+2. 通过WR_CSR(opcode=0x10, addr=0x04, wdata=0x00000001)设置CTRL.EN=1
 输入激励：
-1. pcs_n_i拉低，开始帧传输
-2. 通过pdi_i发送opcode=0x10(WR_CSR)命令数据
-3. 验证pdo_oe_o在请求阶段=0，响应阶段=1
-4. 通过pdo_o接收STATUS响应
-5. pcs_n_i拉高结束帧
+1. 发送WR_CSR命令(opcode=0x10, addr=0x04, wdata=0x00000003)
+2. 监控请求阶段结束后的turnaround周期
+3. 检查pdo_oe_o在turnaround期间=0
+4. 验证响应阶段开始时pdo_oe_o=1
+5. 发送RD_CSR命令(opcode=0x11, addr=0x04)重复验证
 期望结果：
-1. pcs_n_i帧边界正确：拉低开始帧，拉高结束帧
-2. pdi_i输入在clk_i上升沿正确采样
-3. pdo_o输出在响应阶段有效
-4. pdo_oe_o方向控制正确：请求=0，响应=1
-5. MSB first传输顺序正确
+1. 请求/响应阶段正确分离
+2. turnaround固定1个clk_i周期
+3. 协议字段MSB first传输
+4. 四种命令帧格式正确处理
 coverage check点：
-对lane模式、传输方向收集功能覆盖率。</t>
+1. turnaround周期覆盖率
+2. 四种opcode帧格式覆盖率</t>
         </is>
       </c>
       <c r="D8" s="14" t="n"/>
@@ -2848,34 +2816,33 @@
     <row r="9">
       <c r="A9" s="16" t="inlineStr">
         <is>
-          <t>TC_007</t>
+          <t>TC_008</t>
         </is>
       </c>
       <c r="B9" s="16" t="inlineStr">
         <is>
-          <t>test_protocol</t>
+          <t>test_opcode_decode</t>
         </is>
       </c>
       <c r="C9" s="3" t="inlineStr">
         <is>
-          <t>TC场景：测试协议帧格式
-配置条件：
+          <t>配置条件：
 1. test_mode_i=1
-2. CTRL.EN=1
-3. LANE_MODE=00/01分别测试
+2. 通过WR_CSR(opcode=0x10, addr=0x04, wdata=0x00000001)设置CTRL.EN=1
+3. AHB总线空闲
 输入激励：
-1. 发送WR_CSR(0x10)命令：opcode=0x10 + reg_addr + wdata
-2. 发送RD_CSR(0x11)命令：opcode=0x11 + reg_addr
-3. 发送AHB_WR32(0x20)命令：opcode=0x20 + addr + wdata
-4. 发送AHB_RD32(0x21)命令：opcode=0x21 + addr
-5. 验证turnaround周期固定1个clk_i
+1. 发送opcode=0x10(WR_CSR)命令，验证CSR写操作
+2. 发送opcode=0x11(RD_CSR)命令，验证CSR读操作
+3. 发送opcode=0x20(AHB_WR32)命令，验证AHB写操作
+4. 发送opcode=0x21(AHB_RD32)命令，验证AHB读操作
+5. 发送非法opcode(0x00, 0xFF, 0x30等)，验证返回STS_BAD_OPCODE(0x01)
 期望结果：
-1. 四种opcode对应的帧格式正确处理
-2. turnaround周期固定1个clk_i
-3. 协议字段MSB first传输
-4. STATUS=0x00成功返回
+1. 四种opcode正确译码并执行
+2. 非法opcode返回STS_BAD_OPCODE(0x01)
+3. 前端收满8bit opcode后确定期望帧长
 coverage check点：
-对四种opcode命令、lane模式收集功能覆盖率。</t>
+1. 四种有效opcode覆盖率
+2. 非法opcode检测覆盖率</t>
         </is>
       </c>
       <c r="D9" s="14" t="n"/>
@@ -2883,32 +2850,34 @@
     <row r="10">
       <c r="A10" s="16" t="inlineStr">
         <is>
-          <t>TC_008</t>
+          <t>TC_009</t>
         </is>
       </c>
       <c r="B10" s="16" t="inlineStr">
         <is>
-          <t>test_opcode</t>
+          <t>test_ctrl_config</t>
         </is>
       </c>
       <c r="C10" s="3" t="inlineStr">
         <is>
-          <t>TC场景：测试opcode解析
-配置条件：
+          <t>配置条件：
 1. test_mode_i=1
-2. CTRL.EN=1
+2. 通过WR_CSR(opcode=0x10, addr=0x04, wdata=0x00000001)设置CTRL.EN=1
 输入激励：
-1. 发送opcode=0x10(WR_CSR)，验证CSR写命令执行
-2. 发送opcode=0x11(RD_CSR)，验证CSR读命令执行
-3. 发送opcode=0x20(AHB_WR32)，验证AHB写命令执行
-4. 发送opcode=0x21(AHB_RD32)，验证AHB读命令执行
-5. 发送非法opcode(0x00/0xFF)，验证错误处理
+1. 写CTRL.EN=1使能模块，发送AHB_RD32命令验证可执行
+2. 写CTRL.EN=0禁用模块，发送命令验证返回STS_DISABLED(0x04)
+3. 写CTRL.LANE_MODE=00，验证1-bit模式生效
+4. 写CTRL.LANE_MODE=01，验证4-bit模式生效
+5. 写CTRL.SOFT_RST=1，验证协议上下文清零，恢复默认lane模式
 期望结果：
-1. opcode=0x10/0x11/0x20/0x21正确解析并执行
-2. 非法opcode(0x00/0xFF)返回STS_BAD_OPCODE(0x01)
-3. 前端收满8bit opcode后正确确定期望帧长
+1. CTRL配置正确生效
+2. 使能/禁用状态切换正确
+3. 软复位功能正常
+4. 软复位不影响CTRL.EN状态
 coverage check点：
-对opcode值(0x10/0x11/0x20/0x21/非法值)收集功能覆盖率。</t>
+1. CTRL.EN使能/禁用覆盖率
+2. LANE_MODE切换覆盖率
+3. SOFT_RST触发覆盖率</t>
         </is>
       </c>
       <c r="D10" s="14" t="n"/>
@@ -2916,33 +2885,33 @@
     <row r="11">
       <c r="A11" s="16" t="inlineStr">
         <is>
-          <t>TC_009</t>
+          <t>TC_010</t>
         </is>
       </c>
       <c r="B11" s="16" t="inlineStr">
         <is>
-          <t>test_ctrl_config</t>
+          <t>test_status_polling</t>
         </is>
       </c>
       <c r="C11" s="3" t="inlineStr">
         <is>
-          <t>TC场景：测试CTRL配置接口
-配置条件：
+          <t>配置条件：
 1. test_mode_i=1
-2. 初始CTRL.EN=0
+2. 通过WR_CSR(opcode=0x10, addr=0x04, wdata=0x00000001)设置CTRL.EN=1
 输入激励：
-1. 写CTRL.EN=1，验证模块使能，发送命令可执行
-2. 写CTRL.EN=0，验证模块禁用，发送命令返回STS_DISABLED(0x04)
-3. 写CTRL.LANE_MODE=00，验证1-bit模式生效
-4. 写CTRL.LANE_MODE=01，验证4-bit模式生效
-5. 写CTRL.SOFT_RST=1，验证协议上下文清零
+1. 发送非法opcode触发BAD_OPCODE错误
+2. 通过RD_CSR(opcode=0x11, addr=0x0C)读取LAST_ERR寄存器，验证错误码=0x01
+3. 发送AHB_WR32命令，通过RD_CSR(opcode=0x11, addr=0x08)读取STATUS检查busy位
+4. 触发多种错误条件，验证LAST_ERR记录最近错误
+5. 验证无独立中断输出信号
 期望结果：
-1. CTRL.EN配置正确生效
-2. CTRL.LANE_MODE配置正确生效
-3. CTRL.SOFT_RST=1触发软复位，恢复默认lane模式
-4. 配置写入后立即生效
+1. 所有错误与完成状态通过STATUS/LAST_ERR查询获取
+2. MVP版本无中断输出
+3. ATE轮询方式正确获取状态
+4. LAST_ERR更新正确
 coverage check点：
-对CTRL.EN、CTRL.LANE_MODE、CTRL.SOFT_RST配置值收集功能覆盖率。</t>
+1. STATUS寄存器覆盖率
+2. LAST_ERR寄存器覆盖率</t>
         </is>
       </c>
       <c r="D11" s="14" t="n"/>
@@ -2950,60 +2919,28 @@
     <row r="12">
       <c r="A12" s="16" t="inlineStr">
         <is>
-          <t>TC_010</t>
+          <t>TC_011</t>
         </is>
       </c>
       <c r="B12" s="16" t="inlineStr">
         <is>
-          <t>test_status_query</t>
+          <t>test_exception</t>
         </is>
       </c>
       <c r="C12" s="3" t="inlineStr">
         <is>
-          <t>TC场景：测试状态查询
-配置条件：
+          <t>配置条件：
 1. test_mode_i=1
-2. CTRL.EN=1
-输入激励：
-1. 发送命令，在命令执行期间读取STATUS寄存器，验证BUSY位
-2. 触发各类错误条件，读取LAST_ERR寄存器，验证错误码更新
-3. 连续轮询STATUS和LAST_ERR，验证ATE轮询方式可行
-期望结果：
-1. STATUS.BUSY在命令执行期间=1，完成后=0
-2. LAST_ERR在错误发生时更新为对应错误码
-3. 无独立中断输出，状态通过寄存器查询获取
-4. ATE轮询方式正确获取状态
-coverage check点：
-对STATUS和LAST_ERR寄存器值收集功能覆盖率。</t>
-        </is>
-      </c>
-      <c r="D12" s="14" t="n"/>
-    </row>
-    <row r="13">
-      <c r="A13" s="16" t="inlineStr">
-        <is>
-          <t>TC_011</t>
-        </is>
-      </c>
-      <c r="B13" s="16" t="inlineStr">
-        <is>
-          <t>test_error_handling</t>
-        </is>
-      </c>
-      <c r="C13" s="3" t="inlineStr">
-        <is>
-          <t>TC场景：测试异常处理
-配置条件：
-1. test_mode_i=1
-2. CTRL.EN=1
+2. 通过WR_CSR(opcode=0x10, addr=0x04, wdata=0x00000001)设置CTRL.EN=1
+3. AHB总线正常
 输入激励：
 1. 发送非法opcode(0x00/0xFF)，验证返回STS_BAD_OPCODE(0x01)
-2. 访问非法CSR地址，验证返回STS_BAD_REG(0x02)
-3. 发送非4Byte对齐地址，验证返回STS_ALIGN_ERR(0x03)
+2. 访问非法CSR地址(0x10)，验证返回STS_BAD_REG(0x02)
+3. 发送非4Byte对齐地址(addr=0x1001)，验证返回STS_ALIGN_ERR(0x03)
 4. CTRL.EN=0时发送命令，验证返回STS_DISABLED(0x04)
 5. test_mode_i=0时发送命令，验证返回STS_NOT_IN_TEST(0x05)
 6. 提前拉高pcs_n_i，验证返回STS_FRAME_ERR(0x06)
-7. 模拟hresp_i=1，验证返回STS_AHB_ERR(0x07)
+7. 触发hresp_i=1，验证返回STS_AHB_ERR(0x07)
 8. 模拟AHB超时，验证返回STS_TIMEOUT(0x08)
 期望结果：
 1. 各类错误正确检测
@@ -3011,39 +2948,78 @@
 3. 返回确定性状态码
 4. LAST_ERR更新正确
 coverage check点：
-对所有错误码类型收集功能覆盖率。</t>
-        </is>
-      </c>
-      <c r="D13" s="14" t="n"/>
-    </row>
-    <row r="14">
-      <c r="A14" s="16" t="inlineStr">
+1. 8种错误类型覆盖率
+2. 前置错误收敛覆盖率</t>
+        </is>
+      </c>
+      <c r="D12" s="14" t="n"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="16" t="inlineStr">
         <is>
           <t>TC_012</t>
         </is>
       </c>
-      <c r="B14" s="16" t="inlineStr">
-        <is>
-          <t>test_lowpower</t>
-        </is>
-      </c>
-      <c r="C14" s="3" t="inlineStr">
-        <is>
-          <t>TC场景：测试低功耗特性
-配置条件：
-1. 模块处于空闲态(test_mode_i=0或无有效任务)
+      <c r="B13" s="16" t="inlineStr">
+        <is>
+          <t>test_low_power</t>
+        </is>
+      </c>
+      <c r="C13" s="3" t="inlineStr">
+        <is>
+          <t>配置条件：
+1. 模块处于空闲态
+2. test_mode_i=0或无有效任务
 输入激励：
-1. 保持pcs_n_i=1，监测rx_shift_reg和tx_shift_reg是否翻转
-2. 模拟AHB等待态，监测超时计数器是否仅在WAIT_AHB状态工作
-3. 设置test_mode_i=0，验证AHB输出保持IDLE(htrans_o=IDLE)
+1. 保持pcs_n_i=1，监控接收/发送移位寄存器是否翻转
+2. test_mode_i=0，检查AHB输出：htrans_o=0(IDLE)
+3. 模拟AHB等待态，验证超时计数器仅在WAIT_AHB状态工作
 4. 切换到工作态，验证关键寄存器翻转
 期望结果：
 1. 空闲态无效翻转最小化
-2. 超时计数器仅在工作状态更新
-3. test_mode_i=0时AHB输出保持IDLE
-4. 低功耗设计目标满足
+2. 低功耗设计目标满足
+3. AHB输出保持IDLE
+4. 功耗测试通过
 coverage check点：
-对工作状态和空闲状态的寄存器翻转次数收集功能覆盖率。</t>
+1. 空闲态覆盖率
+2. 低功耗模式覆盖率</t>
+        </is>
+      </c>
+      <c r="D13" s="14" t="n"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="16" t="inlineStr">
+        <is>
+          <t>TC_013</t>
+        </is>
+      </c>
+      <c r="B14" s="16" t="inlineStr">
+        <is>
+          <t>test_performance</t>
+        </is>
+      </c>
+      <c r="C14" s="3" t="inlineStr">
+        <is>
+          <t>配置条件：
+1. clk_i=100MHz
+2. AHB总线响应正常
+3. test_mode_i=1
+4. 通过WR_CSR(opcode=0x10, addr=0x04, wdata=0x00000001)设置CTRL.EN=1
+输入激励：
+1. 配置LANE_MODE=00(1-bit)，连续执行AHB_RD32/AHB_WR32命令，计算端到端延时和吞吐率
+2. 配置LANE_MODE=01(4-bit)，执行相同测试
+3. 验证1-bit模式链路线速12.5MB/s
+4. 验证4-bit模式链路线速50MB/s
+5. 发送非对齐地址，验证返回ALIGN_ERR
+期望结果：
+1. 目标频率100MHz稳定工作
+2. 延时符合预期(约23~24 cycles)
+3. 吞吐率达标
+4. AHB访问约束满足(addr[1:0]=00)
+coverage check点：
+1. 100MHz频率覆盖率
+2. 吞吐率达标覆盖率
+3. 地址对齐约束覆盖率</t>
         </is>
       </c>
       <c r="D14" s="14" t="n"/>
@@ -3051,34 +3027,34 @@
     <row r="15">
       <c r="A15" s="16" t="inlineStr">
         <is>
-          <t>TC_013</t>
+          <t>TC_014</t>
         </is>
       </c>
       <c r="B15" s="16" t="inlineStr">
         <is>
-          <t>test_performance</t>
+          <t>test_dfx</t>
         </is>
       </c>
       <c r="C15" s="3" t="inlineStr">
         <is>
-          <t>TC场景：测试性能指标
-配置条件：
-1. test_mode_i=1
-2. CTRL.EN=1
-3. clk_i=100MHz
+          <t>配置条件：
+1. 仿真环境
+2. test_mode_i=1
+3. 通过WR_CSR(opcode=0x10, addr=0x04, wdata=0x00000001)设置CTRL.EN=1
 输入激励：
-1. 在1-bit模式(LANE_MODE=00)下连续执行AHB_RD32/AHB_WR32命令
-2. 在4-bit模式(LANE_MODE=01)下执行相同测试
-3. 测量端到端延时(从pcs_n_i拉低到pdo_oe_o拉高)
-4. 计算吞吐率
+1. 执行WR_CSR命令，采集状态机状态、opcode_reg、addr_reg、wdata_reg
+2. 执行AHB_RD32命令，采集rdata_reg、status_code_reg
+3. 采集rx_count/tx_count计数器
+4. 采集外部接口信号pcs_n_i、pdi_i[3:0]、pdo_o[3:0]、pdo_oe_o
+5. 验证所有调试可观测点可访问
 期望结果：
-1. 目标频率100MHz稳定工作
-2. 端到端延时约23~24个clk_i周期
-3. 1-bit模式原始链路线速12.5MB/s
-4. 4-bit模式原始链路线速50MB/s
-5. AHB访问32bit字访问，地址4Byte对齐
+1. 所有调试可观测点可采集
+2. 便于联调、波形定位和故障复现
+3. 状态机状态正确转换
+4. 计数器正确计数
 coverage check点：
-对延时范围、吞吐率收集功能覆盖率。</t>
+1. DFX可观测点覆盖率
+2. 状态机状态覆盖率</t>
         </is>
       </c>
       <c r="D15" s="14" t="n"/>
@@ -3086,33 +3062,35 @@
     <row r="16">
       <c r="A16" s="16" t="inlineStr">
         <is>
-          <t>TC_014</t>
+          <t>TC_015</t>
         </is>
       </c>
       <c r="B16" s="16" t="inlineStr">
         <is>
-          <t>test_dfx</t>
+          <t>test_memory_map</t>
         </is>
       </c>
       <c r="C16" s="3" t="inlineStr">
         <is>
-          <t>TC场景：测试DFX调试可观测点
-配置条件：
-1. 仿真环境
-2. test_mode_i=1
-3. CTRL.EN=1
+          <t>配置条件：
+1. test_mode_i=1
+2. 通过WR_CSR(opcode=0x10, addr=0x04, wdata=0x00000001)设置CTRL.EN=1
 输入激励：
-1. 执行多种命令序列
-2. 采集状态机状态、opcode、addr、wdata、rdata、status_code
-3. 采集rx/tx计数、pcs_n_i、pdi_i、pdo_o、pdo_oe_o
-4. 验证内部调试可观测点可访问
+1. 通过WR_CSR/RD_CSR访问VERSION寄存器(addr=0x00)
+2. 通过WR_CSR/RD_CSR访问CTRL寄存器(addr=0x04)
+3. 通过WR_CSR/RD_CSR访问STATUS寄存器(addr=0x08)
+4. 通过WR_CSR/RD_CSR访问LAST_ERR寄存器(addr=0x0C)
+5. 发送AHB_WR32命令(opcode=0x20, addr=0x00001000, wdata=0x12345678)访问SoC内部memory-mapped地址
+6. 发送AHB_RD32命令(opcode=0x21, addr=0x00001000)读回验证
+7. 监控AHB地址空间：haddr_o输出32-bit地址
 期望结果：
-1. 状态机状态可观测
-2. 关键寄存器(opcode、addr、wdata、rdata、status_code)可观测
-3. 计数器(rx_count、tx_count)可观测
-4. 接口信号(pcs_n_i、pdi_i、pdo_o、pdo_oe_o)可观测
+1. CSR通过WR_CSR/RD_CSR协议命令正确访问
+2. 模块自身CSR(addr=0x00/0x04/0x08/0x0C)不进入SoC AHB memory map
+3. AHB Master访问采用32-bit地址空间，word访问粒度
+4. haddr_o=0x00001000正确输出
 coverage check点：
-直接用例覆盖，不收功能覆盖率。</t>
+1. CSR地址(0x00~0x0C)覆盖率
+2. AHB地址空间覆盖率</t>
         </is>
       </c>
       <c r="D16" s="14" t="n"/>
@@ -3120,70 +3098,46 @@
     <row r="17">
       <c r="A17" s="16" t="inlineStr">
         <is>
-          <t>TC_015</t>
+          <t>TC_016</t>
         </is>
       </c>
       <c r="B17" s="16" t="inlineStr">
         <is>
-          <t>test_memory_map</t>
+          <t>test_ahb_lite_interface</t>
         </is>
       </c>
       <c r="C17" s="3" t="inlineStr">
         <is>
-          <t>TC场景：测试memory map
-配置条件：
+          <t>配置条件：
 1. test_mode_i=1
-2. CTRL.EN=1
-输入激励：
-1. 通过WR_CSR/RD_CSR访问模块内部CSR(VERSION/CTRL/STATUS/LAST_ERR)
-2. 发送AHB_WR32/AHB_RD32命令访问SoC内部memory-mapped地址
-3. 验证模块自身CSR不进入SoC AHB memory map
-4. 验证AHB Master访问采用32bit地址空间和word访问粒度
-期望结果：
-1. CSR通过协议命令访问正常
-2. AHB Master访问正确
-3. 模块CSR不进入SoC memory map
-4. AHB访问32bit地址空间，word访问粒度
-coverage check点：
-对CSR地址范围、AHB地址范围收集功能覆盖率。</t>
-        </is>
-      </c>
-      <c r="D17" s="14" t="n"/>
-    </row>
-    <row r="18">
-      <c r="A18" s="16" t="inlineStr">
-        <is>
-          <t>TC_016</t>
-        </is>
-      </c>
-      <c r="B18" s="16" t="inlineStr">
-        <is>
-          <t>test_ahb_interface</t>
-        </is>
-      </c>
-      <c r="C18" s="3" t="inlineStr">
-        <is>
-          <t>TC场景：测试AHB-Lite总线接口
-配置条件：
-1. test_mode_i=1
-2. CTRL.EN=1
+2. 通过WR_CSR(opcode=0x10, addr=0x04, wdata=0x00000001)设置CTRL.EN=1
 3. AHB总线空闲
 输入激励：
-1. 发送AHB_WR32(opcode=0x20)命令，验证haddr_o/hwrite_o/htrans_o/hsize_o/hburst_o/hwdata_o输出正确
-2. 发送AHB_RD32(opcode=0x21)命令，验证hrdata_i/hready_i/hresp_i输入正确处理
-3. 验证htrans_o仅输出IDLE(2'b00)和NONSEQ(2'b10)
-4. 验证hsize_o固定为WORD(3'b010)
-5. 验证hburst_o固定为SINGLE(3'b000)
+1. 发送AHB_WR32命令(opcode=0x20, addr=0x00001000, wdata=0xDEADBEEF)
+2. 监控haddr_o=0x00001000, hwrite_o=1, htrans_o=10(NONSEQ), hsize_o=010(WORD), hburst_o=000(SINGLE)
+3. 监控hwdata_o=0xDEADBEEF
+4. 发送AHB_RD32命令(opcode=0x21, addr=0x00001000)
+5. 监控haddr_o=0x00001000, hwrite_o=0, htrans_o=10(NONSEQ)
+6. 验证hrdata_i接收读数据，hready_i=1, hresp_i=0
+7. 触发hresp_i=1，验证错误处理
 期望结果：
 1. AHB-Lite Master接口符合规范
 2. 单次读写事务正确
-3. htrans_o仅IDLE/NONSEQ
-4. hsize_o固定WORD，hburst_o固定SINGLE
-5. 信号时序满足AHB协议要求
+3. 信号时序满足AHB协议要求
+4. hresp_i=1时返回STS_AHB_ERR(0x07)
 coverage check点：
-对AHB命令类型、地址范围收集功能覆盖率。</t>
-        </is>
-      </c>
+1. AHB写事务覆盖率
+2. AHB读事务覆盖率
+3. htrans_o状态覆盖率
+4. 错误响应覆盖率</t>
+        </is>
+      </c>
+      <c r="D17" s="14" t="n"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="16" t="n"/>
+      <c r="B18" s="16" t="n"/>
+      <c r="C18" s="3" t="n"/>
       <c r="D18" s="14" t="n"/>
     </row>
     <row r="19">
@@ -3223,9 +3177,6 @@
       <c r="D24" s="4" t="n"/>
     </row>
   </sheetData>
-  <mergeCells count="1">
-    <mergeCell ref="A1:D1"/>
-  </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
skill v0p7 and rtm(gen in plan mode)
</commit_message>
<xml_diff>
--- a/RTM_AI_gen.xlsx
+++ b/RTM_AI_gen.xlsx
@@ -1454,7 +1454,7 @@
       </c>
       <c r="F3" s="31" t="inlineStr">
         <is>
-          <t>TC_001</t>
+          <t>TC_010</t>
         </is>
       </c>
     </row>
@@ -1488,7 +1488,7 @@
       </c>
       <c r="F4" s="31" t="inlineStr">
         <is>
-          <t>TC_002</t>
+          <t>TC_001</t>
         </is>
       </c>
     </row>
@@ -1522,7 +1522,7 @@
       </c>
       <c r="F5" s="31" t="inlineStr">
         <is>
-          <t>TC_003</t>
+          <t>TC_002</t>
         </is>
       </c>
     </row>
@@ -1556,7 +1556,7 @@
       </c>
       <c r="F6" s="31" t="inlineStr">
         <is>
-          <t>TC_004</t>
+          <t>TC_003</t>
         </is>
       </c>
     </row>
@@ -1585,12 +1585,12 @@
       </c>
       <c r="E7" s="31" t="inlineStr">
         <is>
-          <t>CHK_005</t>
+          <t>CHK_004</t>
         </is>
       </c>
       <c r="F7" s="31" t="inlineStr">
         <is>
-          <t>TC_005</t>
+          <t>TC_003</t>
         </is>
       </c>
     </row>
@@ -1619,12 +1619,14 @@
       </c>
       <c r="E8" s="31" t="inlineStr">
         <is>
-          <t>CHK_006</t>
+          <t>CHK_004
+CHK_005</t>
         </is>
       </c>
       <c r="F8" s="31" t="inlineStr">
         <is>
-          <t>TC_006</t>
+          <t>TC_003
+TC_004</t>
         </is>
       </c>
     </row>
@@ -1653,12 +1655,12 @@
       </c>
       <c r="E9" s="31" t="inlineStr">
         <is>
-          <t>CHK_007</t>
+          <t>CHK_005</t>
         </is>
       </c>
       <c r="F9" s="31" t="inlineStr">
         <is>
-          <t>TC_007</t>
+          <t>TC_004</t>
         </is>
       </c>
     </row>
@@ -1687,12 +1689,12 @@
       </c>
       <c r="E10" s="31" t="inlineStr">
         <is>
-          <t>CHK_008</t>
+          <t>CHK_006</t>
         </is>
       </c>
       <c r="F10" s="31" t="inlineStr">
         <is>
-          <t>TC_008</t>
+          <t>TC_005</t>
         </is>
       </c>
     </row>
@@ -1721,12 +1723,12 @@
       </c>
       <c r="E11" s="31" t="inlineStr">
         <is>
-          <t>CHK_009</t>
+          <t>CHK_007</t>
         </is>
       </c>
       <c r="F11" s="31" t="inlineStr">
         <is>
-          <t>TC_009</t>
+          <t>TC_006</t>
         </is>
       </c>
     </row>
@@ -1755,12 +1757,12 @@
       </c>
       <c r="E12" s="31" t="inlineStr">
         <is>
-          <t>CHK_010</t>
+          <t>CHK_008</t>
         </is>
       </c>
       <c r="F12" s="31" t="inlineStr">
         <is>
-          <t>TC_010</t>
+          <t>TC_007</t>
         </is>
       </c>
     </row>
@@ -1789,12 +1791,12 @@
       </c>
       <c r="E13" s="31" t="inlineStr">
         <is>
-          <t>CHK_011</t>
+          <t>CHK_009</t>
         </is>
       </c>
       <c r="F13" s="31" t="inlineStr">
         <is>
-          <t>TC_011</t>
+          <t>TC_008</t>
         </is>
       </c>
     </row>
@@ -1823,12 +1825,12 @@
       </c>
       <c r="E14" s="31" t="inlineStr">
         <is>
-          <t>CHK_012</t>
+          <t>CHK_010</t>
         </is>
       </c>
       <c r="F14" s="31" t="inlineStr">
         <is>
-          <t>TC_012</t>
+          <t>TC_009</t>
         </is>
       </c>
     </row>
@@ -1857,12 +1859,12 @@
       </c>
       <c r="E15" s="31" t="inlineStr">
         <is>
-          <t>CHK_013</t>
+          <t>CHK_011</t>
         </is>
       </c>
       <c r="F15" s="31" t="inlineStr">
         <is>
-          <t>TC_013</t>
+          <t>TC_010</t>
         </is>
       </c>
     </row>
@@ -1891,12 +1893,12 @@
       </c>
       <c r="E16" s="31" t="inlineStr">
         <is>
-          <t>CHK_014</t>
+          <t>CHK_011</t>
         </is>
       </c>
       <c r="F16" s="31" t="inlineStr">
         <is>
-          <t>TC_014</t>
+          <t>TC_010</t>
         </is>
       </c>
     </row>
@@ -1925,12 +1927,12 @@
       </c>
       <c r="E17" s="31" t="inlineStr">
         <is>
-          <t>CHK_015</t>
+          <t>CHK_003</t>
         </is>
       </c>
       <c r="F17" s="31" t="inlineStr">
         <is>
-          <t>TC_015</t>
+          <t>TC_002</t>
         </is>
       </c>
     </row>
@@ -1959,12 +1961,12 @@
       </c>
       <c r="E18" s="31" t="inlineStr">
         <is>
-          <t>CHK_016</t>
+          <t>CHK_012</t>
         </is>
       </c>
       <c r="F18" s="31" t="inlineStr">
         <is>
-          <t>TC_016</t>
+          <t>TC_010</t>
         </is>
       </c>
     </row>
@@ -1976,9 +1978,6 @@
       <c r="E19" s="31" t="n"/>
       <c r="F19" s="31" t="n"/>
     </row>
-    <row r="20"/>
-    <row r="21"/>
-    <row r="22"/>
     <row r="23">
       <c r="A23" s="23" t="inlineStr">
         <is>
@@ -2108,6 +2107,9 @@
           <t>Checker List</t>
         </is>
       </c>
+      <c r="B1" s="20" t="n"/>
+      <c r="C1" s="20" t="n"/>
+      <c r="D1" s="21" t="n"/>
     </row>
     <row r="2">
       <c r="A2" s="22" t="inlineStr">
@@ -2139,15 +2141,14 @@
       </c>
       <c r="B3" s="31" t="inlineStr">
         <is>
-          <t>clk_domain_sync_checker</t>
+          <t>clk_checker</t>
         </is>
       </c>
       <c r="C3" s="6" t="inlineStr">
         <is>
-          <t>1. 检查clk_i上升沿时所有内部寄存器正确采样
-2. 验证100MHz频率下协议采样(pdi_i)、状态机转换、AHB-Lite信号(haddr_o/hwrite_o/hwdata_o/hrdata_i)同域工作
-3. 确认无跨时钟域信号，所有操作在单个clk_i域内完成
-4. 检查clk_i占空比在40%-60%范围内时模块正常工作</t>
+          <t>1. 检查clk_i时钟频率稳定性：在一定数量的时钟周期期间，计算实际周期并判断是否处于目标频率100MHz的允许误差范围内（±3%）
+2. 检查时钟域同步性：验证外部协议采样、状态机控制和AHB-Lite主接口均在clk_i同域工作
+3. 检查时钟信号完整性：无毛刺、无X态或高阻态</t>
         </is>
       </c>
       <c r="D3" s="4" t="n"/>
@@ -2160,16 +2161,19 @@
       </c>
       <c r="B4" s="18" t="inlineStr">
         <is>
-          <t>rst_async_sync_checker</t>
+          <t>reset_checker</t>
         </is>
       </c>
       <c r="C4" s="17" t="inlineStr">
         <is>
-          <t>1. 检查rst_ni拉低后异步复位立即生效，状态机跳转到IDLE状态
-2. 验证rst_ni释放后同步释放机制（至少2个clk_i周期同步）
-3. 确认复位后CTRL.EN=0、CTRL.LANE_MODE=00(1-bit模式)
-4. 检查STATUS寄存器清零、LAST_ERR寄存器清零
-5. 验证协议上下文(rx_shift_reg/tx_shift_reg/opcode_reg/addr_reg/wdata_reg)清空</t>
+          <t>1. 检查rst_ni异步复位生效：rst_ni拉低后状态机回到IDLE状态
+2. 检查复位后寄存器默认值：
+   - CTRL.EN=0（模块未使能）
+   - CTRL.LANE_MODE=00（1-bit模式）
+   - STATUS寄存器清零
+   - LAST_ERR寄存器清零
+3. 检查复位释放同步性：内部同步释放，协议上下文和错误状态已清空
+4. 检查复位连接性：rst_ni正确连接至模块并生效</t>
         </is>
       </c>
       <c r="D4" s="4" t="n"/>
@@ -2182,17 +2186,19 @@
       </c>
       <c r="B5" s="31" t="inlineStr">
         <is>
-          <t>csr_access_checker</t>
+          <t>csr_checker</t>
         </is>
       </c>
       <c r="C5" s="6" t="inlineStr">
         <is>
-          <t>1. 检查通过WR_CSR(opcode=0x10)写CSR寄存器：addr=0x00(VERSION)只读、addr=0x04(CTRL)读写、addr=0x08(STATUS)只读、addr=0x0C(LAST_ERR)只读
-2. 验证RD_CSR(opcode=0x11)读CSR寄存器返回正确数据
-3. 确认VERSION寄存器写入无效，读回返回固定版本号
-4. 检查CTRL.EN位写1后模块使能，写0后禁用
-5. 验证CTRL.LANE_MODE=00/01有效，10/11不改变配置
-6. 确认CTRL.SOFT_RST写1后触发软复位，协议上下文清零</t>
+          <t>1. 检查CSR寄存器读写正确性：
+   - VERSION寄存器(addr=0x00)：只读，通过RD_CSR(opcode=0x11)读取版本号
+   - CTRL寄存器(addr=0x04)：可读写，字段包括EN、LANE_MODE、SOFT_RST
+   - STATUS寄存器(addr=0x08)：只读，反映busy和错误状态
+   - LAST_ERR寄存器(addr=0x0C)：只读，存储最近错误码
+2. 检查CSR访问协议：通过WR_CSR(opcode=0x10)和RD_CSR(opcode=0x11)命令访问
+3. 检查模块自身CSR不进入SoC AHB memory map
+4. 九步法检测寄存器：包含默认值、读写属性、异常地址读写检查</t>
         </is>
       </c>
       <c r="D5" s="4" t="n"/>
@@ -2205,15 +2211,17 @@
       </c>
       <c r="B6" s="31" t="inlineStr">
         <is>
-          <t>test_mode_enable_checker</t>
+          <t>lane_mode_checker</t>
         </is>
       </c>
       <c r="C6" s="6" t="inlineStr">
         <is>
-          <t>1. 检查test_mode_i=1且CTRL.EN=1时功能命令可执行
-2. 验证test_mode_i=0时命令返回STS_NOT_IN_TEST(0x05)
-3. 确认CTRL.EN=0时命令返回STS_DISABLED(0x04)
-4. 检查半双工请求/响应模式：pcs_n_i拉低开始请求阶段，turnaround 1周期后进入响应阶段</t>
+          <t>1. 检查CTRL.LANE_MODE=00时仅使用pdi_i[0]/pdo_o[0]传输
+2. 验证CTRL.LANE_MODE=01时每拍收发4bit（高nibble优先）：
+   - pdi_i[3:0]/pdo_o[3:0]同时有效
+   - 高nibble优先传输
+3. 确认非法LANE_MODE值(10/11)不改变当前配置或返回错误
+4. 检查lane模式切换时无数据丢失</t>
         </is>
       </c>
       <c r="D6" s="4" t="n"/>
@@ -2226,15 +2234,21 @@
       </c>
       <c r="B7" s="12" t="inlineStr">
         <is>
-          <t>lane_mode_checker</t>
+          <t>protocol_checker</t>
         </is>
       </c>
       <c r="C7" s="6" t="inlineStr">
         <is>
-          <t>1. 检查CTRL.LANE_MODE=00时仅使用pdi_i[0]/pdo_o[0]传输，每拍收发1bit
-2. 验证CTRL.LANE_MODE=01时使用pdi_i[3:0]/pdo_o[3:0]传输，每拍收发4bit，高nibble优先
-3. 确认非法LANE_MODE值(10/11)写入时不改变当前配置
-4. 检查lane模式切换后立即生效，影响后续所有数据传输</t>
+          <t>1. 检查pcs_n_i帧边界：pcs_n_i拉低开启事务，拉高结束事务
+2. 检查turnaround周期：请求阶段后固定1个clk_i周期的turnaround，期间pdo_oe_o=0
+3. 检查pdo_oe_o输出使能：响应阶段pdo_oe_o=1，pdo_o[3:0]输出有效数据
+4. 检查协议字段MSB first传输顺序
+5. 检查四种命令帧格式：
+   - WR_CSR(opcode=0x10): opcode(8bit) + addr(8bit) + wdata(32bit)
+   - RD_CSR(opcode=0x11): opcode(8bit) + addr(8bit)
+   - AHB_WR32(opcode=0x20): opcode(8bit) + addr(32bit) + wdata(32bit)
+   - AHB_RD32(opcode=0x21): opcode(8bit) + addr(32bit)
+6. 检查pdi_i在有效周期内无毛刺切换</t>
         </is>
       </c>
       <c r="D7" s="14" t="n"/>
@@ -2247,15 +2261,19 @@
       </c>
       <c r="B8" s="12" t="inlineStr">
         <is>
-          <t>frame_boundary_checker</t>
+          <t>opcode_checker</t>
         </is>
       </c>
       <c r="C8" s="6" t="inlineStr">
         <is>
-          <t>1. 检查pcs_n_i拉低后模块开始接收请求（state从IDLE→RX）
-2. 验证pcs_n_i在请求未完成时提前拉高，返回STS_FRAME_ERR(0x06)到LAST_ERR寄存器
-3. 确认pdo_oe_o在响应阶段正确指示输出方向：TX阶段=1，其他=0
-4. 检查帧格式：opcode(8bit) + addr(16bit) + wdata(32bit，仅写命令)</t>
+          <t>1. 检查opcode解析正确性：
+   - 8'h10解析为WR_CSR，期望帧长=8+8+32=48bit
+   - 8'h11解析为RD_CSR，期望帧长=8+8=16bit
+   - 8'h20解析为AHB_WR32，期望帧长=8+32+32=72bit
+   - 8'h21解析为AHB_RD32，期望帧长=8+32=40bit
+2. 检查前端在收满8bit opcode后正确确定期望帧长
+3. 检查非法opcode(非0x10/0x11/0x20/0x21)返回STS_BAD_OPCODE(0x01)
+4. 检查opcode译码后正确发起相应任务</t>
         </is>
       </c>
       <c r="D8" s="14" t="n"/>
@@ -2268,15 +2286,23 @@
       </c>
       <c r="B9" s="12" t="inlineStr">
         <is>
-          <t>turnaround_checker</t>
+          <t>config_checker</t>
         </is>
       </c>
       <c r="C9" s="6" t="inlineStr">
         <is>
-          <t>1. 检查请求阶段结束后固定1个clk_i周期的turnaround
-2. 验证turnaround期间pdo_oe_o=0，pdi_i/pdo_o处于高阻态
-3. 确认turnaround结束后pdo_oe_o=1，进入TX阶段输出响应
-4. 检查协议字段按MSB first顺序传输</t>
+          <t>1. 检查CTRL.EN配置生效：
+   - EN=1时模块使能，功能命令可执行
+   - EN=0时模块禁用，命令返回DISABLED错误(0x04)
+2. 检查CTRL.LANE_MODE配置生效：
+   - LANE_MODE=00时1-bit模式
+   - LANE_MODE=01时4-bit模式
+   - LANE_MODE=10/11时保持当前配置或返回错误
+3. 检查CTRL.SOFT_RST功能：
+   - SOFT_RST写1触发协议上下文清零
+   - 恢复默认lane模式(LANE_MODE=00)
+   - 不影响CTRL.EN配置
+4. 检查配置变更时序：配置立即生效或下一事务生效</t>
         </is>
       </c>
       <c r="D9" s="14" t="n"/>
@@ -2289,17 +2315,19 @@
       </c>
       <c r="B10" s="12" t="inlineStr">
         <is>
-          <t>opcode_decode_checker</t>
+          <t>status_checker</t>
         </is>
       </c>
       <c r="C10" s="6" t="inlineStr">
         <is>
-          <t>1. 检查opcode=0x10(WR_CSR)正确译码为CSR写操作
-2. 验证opcode=0x11(RD_CSR)正确译码为CSR读操作
-3. 确认opcode=0x20(AHB_WR32)正确译码为AHB写操作
-4. 检查opcode=0x21(AHB_RD32)正确译码为AHB读操作
-5. 验证非法opcode(非0x10/0x11/0x20/0x21)返回STS_BAD_OPCODE(0x01)
-6. 确认前端收满8bit opcode后确定期望帧长</t>
+          <t>1. 检查STATUS寄存器状态位：
+   - busy位：事务进行中置1，完成后清0
+   - sticky位：错误发生后置1，需软件清零
+2. 检查LAST_ERR寄存器更新：
+   - 每次错误发生后更新为对应状态码
+   - 成功操作后保持原值或清零
+3. 检查无独立中断输出：MVP版本不实现中断信号
+4. 检查ATE轮询方式获取状态的正确性</t>
         </is>
       </c>
       <c r="D10" s="14" t="n"/>
@@ -2312,15 +2340,25 @@
       </c>
       <c r="B11" s="12" t="inlineStr">
         <is>
-          <t>ctrl_config_checker</t>
+          <t>error_checker</t>
         </is>
       </c>
       <c r="C11" s="6" t="inlineStr">
         <is>
-          <t>1. 检查CTRL.EN=1时功能命令可执行，CTRL.EN=0时返回STS_DISABLED(0x04)
-2. 验证CTRL.LANE_MODE=00切换到1-bit模式，=01切换到4-bit模式
-3. 确认CTRL.SOFT_RST写1触发软复位：协议上下文清零、恢复默认lane模式(1-bit)
-4. 检查软复位不影响CTRL.EN状态</t>
+          <t>检查8类错误的检测和状态码生成：
+1. BAD_OPCODE(0x01): opcode不在{0x10,0x11,0x20,0x21}范围内
+2. BAD_REG(0x02): CSR地址不在{0x00,0x04,0x08,0x0C}范围内
+3. ALIGN_ERR(0x03): AHB访问地址未4Byte对齐（addr[1:0]!=00）
+4. DISABLED(0x04): CTRL.EN=0时发送功能命令
+5. NOT_IN_TEST(0x05): test_mode_i=0时发送功能命令
+6. FRAME_ERR(0x06): pcs_n_i提前拉高导致帧不完整
+7. AHB_ERR(0x07): hresp_i=1表示AHB错误响应
+8. TIMEOUT(0x08): AHB访问超时
+检查点：
+- 在发起AHB访问前完成前置错误收敛
+- 返回确定性状态码
+- LAST_ERR寄存器正确更新
+- 响应帧包含正确状态码</t>
         </is>
       </c>
       <c r="D11" s="14" t="n"/>
@@ -2333,15 +2371,19 @@
       </c>
       <c r="B12" s="12" t="inlineStr">
         <is>
-          <t>status_polling_checker</t>
+          <t>lowpower_checker</t>
         </is>
       </c>
       <c r="C12" s="6" t="inlineStr">
         <is>
-          <t>1. 检查STATUS[0]反映模块busy状态：命令执行期间=1，空闲=0
-2. 验证LAST_ERR寄存器记录最近错误码
-3. 确认MVP版本无独立中断输出，所有状态通过STATUS/LAST_ERR轮询获取
-4. 检查错误发生时LAST_ERR更新，STATUS[0]清除命令完成后归零</t>
+          <t>1. 检查空闲态下无效翻转最小化：
+   - 接收/发送移位寄存器不更新（pcs_n_i=1时）
+   - 超时计数器仅在RX/TX/WAIT_AHB相关状态工作
+2. 检查test_mode_i=0时AHB输出保持IDLE：
+   - htrans_o=IDLE(2'b00)
+   - hwrite_o、hsize_o、hburst_o无效
+3. 检查无有效任务时AHB输出保持IDLE
+4. 检查仅关键状态(RX/TX/WAIT_AHB)翻转时寄存器更新</t>
         </is>
       </c>
       <c r="D12" s="14" t="n"/>
@@ -2354,20 +2396,22 @@
       </c>
       <c r="B13" s="12" t="inlineStr">
         <is>
-          <t>exception_checker</t>
+          <t>perf_checker</t>
         </is>
       </c>
       <c r="C13" s="6" t="inlineStr">
         <is>
-          <t>1. 检查BAD_OPCODE(0x01)：opcode非0x10/0x11/0x20/0x21
-2. 验证BAD_REG(0x02)：CSR地址非0x00/0x04/0x08/0x0C
-3. 确认ALIGN_ERR(0x03)：AHB地址非4Byte对齐(addr[1:0]!=0)
-4. 检查DISABLED(0x04)：CTRL.EN=0时发送命令
-5. 验证NOT_IN_TEST(0x05)：test_mode_i=0时发送命令
-6. 确认FRAME_ERR(0x06)：pcs_n_i提前拉高
-7. 检查AHB_ERR(0x07)：hresp_i=1
-8. 验证TIMEOUT(0x08)：AHB访问超时
-9. 确认前置错误(0x01-0x06)在发起AHB访问前收敛</t>
+          <t>1. 检查目标频率100MHz稳定工作
+2. 检查端到端延时：
+   - 1-bit模式：约23~24 cycles
+   - 4-bit模式：相应缩短
+3. 检查原始链路线速：
+   - 1-bit模式：12.5MB/s
+   - 4-bit模式：50MB/s
+4. 检查AHB接口约束：
+   - 32bit字访问
+   - 地址4Byte对齐
+5. 检查吞吐率达标</t>
         </is>
       </c>
       <c r="D13" s="14" t="n"/>
@@ -2380,103 +2424,52 @@
       </c>
       <c r="B14" s="12" t="inlineStr">
         <is>
-          <t>low_power_checker</t>
+          <t>ahb_checker</t>
         </is>
       </c>
       <c r="C14" s="6" t="inlineStr">
         <is>
-          <t>1. 检查空闲态(IDLE)下接收/发送移位寄存器不翻转
-2. 验证test_mode_i=0或无有效任务时AHB输出保持IDLE：htrans_o=0
-3. 确认超时计数器仅在WAIT_AHB状态工作
-4. 检查RX/TX/WAIT_AHB状态翻转关键寄存器</t>
+          <t>1. 检查AHB-Lite Master接口信号：
+   - haddr_o: 32-bit地址输出
+   - hwrite_o: 读写标志（1=写，0=读）
+   - htrans_o: 仅输出IDLE(2'b00)或NONSEQ(2'b10)
+   - hsize_o: 固定为WORD(3'b010，32-bit)
+   - hburst_o: 固定为SINGLE(3'b000)
+   - hwdata_o: 32-bit写数据
+2. 检查AHB读响应：
+   - hrdata_i: 32-bit读返回数据
+   - hready_i: ready信号
+   - hresp_i: 错误响应（0=OKAY，1=ERROR）
+3. 检查AHB事务时序：
+   - 地址相：haddr_o、hwrite_o、htrans_o、hsize_o、hburst_o有效
+   - 数据相：hwdata_o（写）或hrdata_i（读）有效
+4. 检查控制命令正确转换为AHB-Lite单次读写事务</t>
         </is>
       </c>
       <c r="D14" s="14" t="n"/>
     </row>
     <row r="15">
-      <c r="A15" s="12" t="inlineStr">
-        <is>
-          <t>CHK_013</t>
-        </is>
-      </c>
-      <c r="B15" s="12" t="inlineStr">
-        <is>
-          <t>performance_checker</t>
-        </is>
-      </c>
-      <c r="C15" s="6" t="inlineStr">
-        <is>
-          <t>1. 检查100MHz频率稳定工作，无时序违例
-2. 验证1-bit模式链路线速12.5MB/s：每拍1bit，8拍/byte
-3. 确认4-bit模式链路线速50MB/s：每拍4bit，2拍/byte
-4. 检查AHB接口32bit字访问，hsize_o=010(WORD)
-5. 验证地址4Byte对齐：addr[1:0]=00</t>
-        </is>
-      </c>
+      <c r="A15" s="12" t="n"/>
+      <c r="B15" s="12" t="n"/>
+      <c r="C15" s="6" t="n"/>
       <c r="D15" s="14" t="n"/>
     </row>
     <row r="16">
-      <c r="A16" s="12" t="inlineStr">
-        <is>
-          <t>CHK_014</t>
-        </is>
-      </c>
-      <c r="B16" s="12" t="inlineStr">
-        <is>
-          <t>dfx_observable_checker</t>
-        </is>
-      </c>
-      <c r="C16" s="6" t="inlineStr">
-        <is>
-          <t>1. 检查状态机状态(state)可观测：IDLE/RX/TX/WAIT_AHB等
-2. 验证内部寄存器可观测：opcode_reg、addr_reg、wdata_reg、rdata_reg、status_code_reg
-3. 确认rx_count/tx_count计数器可观测
-4. 检查外部接口信号pcs_n_i、pdi_i[3:0]、pdo_o[3:0]、pdo_oe_o可观测</t>
-        </is>
-      </c>
+      <c r="A16" s="12" t="n"/>
+      <c r="B16" s="12" t="n"/>
+      <c r="C16" s="6" t="n"/>
       <c r="D16" s="14" t="n"/>
     </row>
     <row r="17">
-      <c r="A17" s="12" t="inlineStr">
-        <is>
-          <t>CHK_015</t>
-        </is>
-      </c>
-      <c r="B17" s="12" t="inlineStr">
-        <is>
-          <t>memory_map_checker</t>
-        </is>
-      </c>
-      <c r="C17" s="6" t="inlineStr">
-        <is>
-          <t>1. 检查模块CSR(addr=0x00/0x04/0x08/0x0C)通过WR_CSR/RD_CSR协议命令访问
-2. 验证模块自身CSR不进入SoC AHB memory map
-3. 确认AHB Master访问采用32-bit地址空间：haddr_o[31:0]
-4. 检查word访问粒度：hsize_o=010，每次访问4Byte</t>
-        </is>
-      </c>
+      <c r="A17" s="12" t="n"/>
+      <c r="B17" s="12" t="n"/>
+      <c r="C17" s="6" t="n"/>
       <c r="D17" s="14" t="n"/>
     </row>
     <row r="18">
-      <c r="A18" s="12" t="inlineStr">
-        <is>
-          <t>CHK_016</t>
-        </is>
-      </c>
-      <c r="B18" s="12" t="inlineStr">
-        <is>
-          <t>ahb_lite_checker</t>
-        </is>
-      </c>
-      <c r="C18" s="6" t="inlineStr">
-        <is>
-          <t>1. 检查AHB_WR32命令：haddr_o输出32-bit地址，hwrite_o=1，htrans_o=NONSEQ(10)，hsize_o=010(WORD)，hburst_o=000(SINGLE)，hwdata_o输出写数据
-2. 验证AHB_RD32命令：haddr_o输出地址，hwrite_o=0，htrans_o=NONSEQ，hsize_o=010，hburst_o=000，hrdata_i接收读数据
-3. 确认hready_i=1时数据有效传输，hresp_i=0表示正常响应
-4. 检查hresp_i=1时返回STS_AHB_ERR(0x07)错误
-5. 验证htrans_o仅输出IDLE(00)或NONSEQ(10)，无SEQ/Busy</t>
-        </is>
-      </c>
+      <c r="A18" s="12" t="n"/>
+      <c r="B18" s="12" t="n"/>
+      <c r="C18" s="6" t="n"/>
       <c r="D18" s="14" t="n"/>
     </row>
     <row r="19">
@@ -2515,29 +2508,64 @@
       <c r="C24" s="6" t="n"/>
       <c r="D24" s="4" t="n"/>
     </row>
-    <row r="25"/>
-    <row r="26"/>
-    <row r="27"/>
     <row r="28">
-      <c r="A28" s="23" t="n"/>
+      <c r="A28" s="23" t="inlineStr">
+        <is>
+          <t>填写要求</t>
+        </is>
+      </c>
     </row>
     <row r="29" ht="24" customHeight="1" s="24">
-      <c r="A29" s="31" t="n"/>
-      <c r="B29" s="35" t="n"/>
+      <c r="A29" s="31" t="inlineStr">
+        <is>
+          <t>CHK Name</t>
+        </is>
+      </c>
+      <c r="B29" s="35" t="inlineStr">
+        <is>
+          <t>如果是SVA checker，需填写SVA property名字</t>
+        </is>
+      </c>
+      <c r="C29" s="20" t="n"/>
+      <c r="D29" s="21" t="n"/>
     </row>
     <row r="30" ht="69.95" customHeight="1" s="24">
-      <c r="A30" s="31" t="n"/>
-      <c r="B30" s="36" t="n"/>
+      <c r="A30" s="31" t="inlineStr">
+        <is>
+          <t>CHK描述</t>
+        </is>
+      </c>
+      <c r="B30" s="36" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1、需要定性+定量描述，需具体到check的信号、取值 
+2、和DV SPEC中Checker方案描述的区别 — RTM中描述check的内容，DV SPEC中描述checker的实现方案(例如是通过SVA实现还是scoreboard实时数据比对，还是文件对比)
+</t>
+        </is>
+      </c>
+      <c r="C30" s="20" t="n"/>
+      <c r="D30" s="21" t="n"/>
     </row>
     <row r="31">
       <c r="A31" s="31" t="n"/>
       <c r="B31" s="12" t="n"/>
+      <c r="C31" s="20" t="n"/>
+      <c r="D31" s="21" t="n"/>
     </row>
     <row r="32">
       <c r="A32" s="31" t="n"/>
       <c r="B32" s="12" t="n"/>
+      <c r="C32" s="20" t="n"/>
+      <c r="D32" s="21" t="n"/>
     </row>
   </sheetData>
+  <mergeCells count="6">
+    <mergeCell ref="A1:D1"/>
+    <mergeCell ref="B31:D31"/>
+    <mergeCell ref="B32:D32"/>
+    <mergeCell ref="B30:D30"/>
+    <mergeCell ref="B29:D29"/>
+    <mergeCell ref="A28:D28"/>
+  </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -2560,48 +2588,27 @@
     <row r="1">
       <c r="A1" s="29" t="inlineStr">
         <is>
-          <t>TC编号</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>TC Name</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>TC描述</t>
-        </is>
-      </c>
+          <t>Test Case List</t>
+        </is>
+      </c>
+      <c r="B1" s="20" t="n"/>
+      <c r="C1" s="20" t="n"/>
+      <c r="D1" s="21" t="n"/>
     </row>
     <row r="2">
       <c r="A2" s="22" t="inlineStr">
         <is>
-          <t>TC_001</t>
+          <t>TC编号</t>
         </is>
       </c>
       <c r="B2" s="22" t="inlineStr">
         <is>
-          <t>test_clock_domain</t>
+          <t>TC Name</t>
         </is>
       </c>
       <c r="C2" s="22" t="inlineStr">
         <is>
-          <t>配置条件：
-1. 配置clk_i时钟频率为100MHz
-2. test_mode_i=1
-输入激励：
-1. 通过WR_CSR(opcode=0x10, addr=0x04, wdata=0x00000001)设置CTRL.EN=1
-2. 配置LANE_MODE=00(1-bit模式)，连续发送AHB_RD32命令(opcode=0x21, addr=0x00001000)
-3. 配置LANE_MODE=01(4-bit模式)，连续发送AHB_WR32命令(opcode=0x20, addr=0x00002000, wdata=0xDEADBEEF)
-4. 在clk_i占空比40%-60%范围内重复上述测试
-期望结果：
-1. 所有命令在100MHz频率下正确执行
-2. 协议采样(pdi_i)、状态机控制、AHB-Lite主接口同域工作正常
-3. 无时序违例，无跨时钟域问题
-coverage check点：
-1. 100MHz频率下命令执行成功率
-2. 1-bit和4-bit模式切换覆盖率</t>
+          <t>TC 描述</t>
         </is>
       </c>
       <c r="D2" s="22" t="inlineStr">
@@ -2613,7 +2620,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>TC_002</t>
+          <t>TC_001</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
@@ -2623,23 +2630,26 @@
       </c>
       <c r="C3" s="3" t="inlineStr">
         <is>
-          <t>配置条件：
-1. 初始rst_ni=0，模块处于复位状态
+          <t>TC场景：测试模块复位功能
+配置条件：
+1. 初始状态rst_ni=0，模块处于复位状态
 2. test_mode_i=1
+其它：以上测试过程中，不关心的配置或接口控制信号随机
 输入激励：
-1. 释放rst_ni，等待至少2个clk_i周期
-2. 通过RD_CSR(opcode=0x11, addr=0x04)读取CTRL寄存器，验证EN=0、LANE_MODE=00
-3. 通过RD_CSR(opcode=0x11, addr=0x08)读取STATUS寄存器，验证为0
-4. 通过RD_CSR(opcode=0x11, addr=0x0C)读取LAST_ERR寄存器，验证为0
-5. 检查内部状态机处于IDLE状态
+1. 释放rst_ni，等待复位同步释放完成
+2. 通过RD_CSR(opcode=0x11, addr=0x04)读取CTRL寄存器
+3. 通过RD_CSR(opcode=0x11, addr=0x08)读取STATUS寄存器
+4. 通过RD_CSR(opcode=0x11, addr=0x0C)读取LAST_ERR寄存器
+5. 监测状态机状态
 期望结果：
-1. rst_ni释放后状态机回到IDLE
-2. CTRL.EN=0，CTRL.LANE_MODE=00(1-bit默认值)
-3. STATUS/LAST_ERR清零，无残留状态
-4. 协议上下文清空
+1. 复位后状态机处于IDLE状态
+2. CTRL.EN=0（模块未使能）
+3. CTRL.LANE_MODE=00（1-bit模式默认值）
+4. STATUS寄存器清零
+5. LAST_ERR寄存器清零
+6. 协议上下文和错误状态已清空
 coverage check点：
-1. 异步复位生效覆盖率
-2. 同步释放机制覆盖率</t>
+对复位后寄存器默认值收集功能覆盖率</t>
         </is>
       </c>
       <c r="D3" s="4" t="n"/>
@@ -2647,7 +2657,7 @@
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>TC_003</t>
+          <t>TC_002</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
@@ -2657,25 +2667,30 @@
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
-          <t>配置条件：
+          <t>TC场景：测试CSR寄存器访问和memory map功能
+配置条件：
 1. test_mode_i=1
 2. 通过WR_CSR(opcode=0x10, addr=0x04, wdata=0x00000001)设置CTRL.EN=1
+其它：以上测试过程中，AHB总线空闲
 输入激励：
-1. 通过RD_CSR(opcode=0x11, addr=0x00)读取VERSION寄存器，记录版本号
-2. 通过WR_CSR(opcode=0x10, addr=0x00, wdata=0xFFFFFFFF)尝试写VERSION寄存器
-3. 再次读取VERSION寄存器，验证只读属性（值不变）
-4. 通过WR_CSR(opcode=0x10, addr=0x04, wdata=0x00000003)写CTRL寄存器（EN=1, LANE_MODE=01）
-5. 通过RD_CSR(opcode=0x11, addr=0x04)读取CTRL寄存器，验证写入正确
-6. 通过RD_CSR(opcode=0x11, addr=0x08)读取STATUS寄存器
-7. 通过RD_CSR(opcode=0x11, addr=0x0C)读取LAST_ERR寄存器
+1. 通过RD_CSR(opcode=0x11, addr=0x00)读取VERSION寄存器
+2. 通过WR_CSR(opcode=0x10, addr=0x00, wdata=0xFFFFFFFF)尝试写VERSION寄存器，验证只读属性
+3. 通过WR_CSR(opcode=0x10, addr=0x04, wdata=0x00000003)写CTRL寄存器（EN=1, LANE_MODE=01）
+4. 通过RD_CSR(opcode=0x11, addr=0x04)读取CTRL寄存器
+5. 通过RD_CSR(opcode=0x11, addr=0x08)读取STATUS寄存器
+6. 发送AHB_WR32命令(opcode=0x20, addr=0x00001000, wdata=0x12345678)访问SoC内部memory-mapped地址
+7. 发送AHB_RD32命令(opcode=0x21, addr=0x00001000)读回验证
+8. 监控haddr_o输出
 期望结果：
-1. CSR读写正确
+1. CSR通过WR_CSR/RD_CSR协议命令正确访问
 2. VERSION寄存器只读，写入后读回原值
 3. CTRL寄存器读写正确，配置生效
-4. STATUS/LAST_ERR反映正确状态
+4. STATUS寄存器反映正确状态
+5. AHB_WR32/AHB_RD32正确访问SoC memory-mapped地址，haddr_o=0x00001000
+6. 模块自身CSR(addr=0x00/0x04/0x08/0x0C)不进入SoC AHB memory map
+7. AHB Master访问采用32-bit地址空间，word访问粒度
 coverage check点：
-1. CSR地址(0x00/0x04/0x08/0x0C)读写覆盖率
-2. 只读寄存器写保护覆盖率</t>
+对CSR地址(0x00~0x0C)和AHB地址空间收集功能覆盖率</t>
         </is>
       </c>
       <c r="D4" s="4" t="n"/>
@@ -2683,32 +2698,37 @@
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>TC_004</t>
+          <t>TC_003</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>test_work_mode</t>
+          <t>test_lane_mode</t>
         </is>
       </c>
       <c r="C5" s="3" t="inlineStr">
         <is>
-          <t>配置条件：
+          <t>TC场景：测试lane模式配置和数据接口功能
+配置条件：
 1. test_mode_i=1
 2. 通过WR_CSR(opcode=0x10, addr=0x04, wdata=0x00000001)设置CTRL.EN=1
+其它：以上测试过程中，AHB总线响应正常
 输入激励：
-1. 发送WR_CSR命令(opcode=0x10, addr=0x04, wdata=0x00000003)配置LANE_MODE=01(4-bit)
-2. 发送AHB_WR32命令(opcode=0x20, addr=0x00001000, wdata=0x12345678)
-3. 发送AHB_RD32命令(opcode=0x21, addr=0x00001000)读回验证
-4. 监控pcs_n_i帧边界和pdo_oe_o输出使能
+1. 配置LANE_MODE=00（1-bit模式），发送AHB_RD32命令验证
+2. 验证pdi_i[0]/pdo_o[0]数据传输，pdi_i[3:1]/pdo_o[3:1]无效
+3. 配置LANE_MODE=01（4-bit模式），发送相同命令
+4. 验证pdi_i[3:0]/pdo_o[3:0]同时有效，高nibble优先发送
+5. 尝试配置非法LANE_MODE值(10/11)，验证错误处理
+6. 验证pcs_n_i帧边界正确：拉低开启事务，拉高结束事务
+7. 验证协议字段MSB first传输顺序
 期望结果：
-1. 模块正确执行功能命令
-2. 协议采用半双工请求/响应模式
-3. CSR访问与AHB-Lite单次读写正常
-4. pcs_n_i定义帧边界正确，pdo_oe_o在TX阶段=1
+1. 1-bit模式仅使用bit0传输，协议正确
+2. 4-bit模式每拍收发4bit，高nibble优先
+3. 非法LANE_MODE值(10/11)返回错误或保持当前配置
+4. pcs_n_i帧边界清晰
+5. MSB first传输顺序正确
 coverage check点：
-1. 半双工模式覆盖率
-2. 请求/响应阶段切换覆盖率</t>
+对LANE_MODE配置值和数据传输模式收集功能覆盖率</t>
         </is>
       </c>
       <c r="D5" s="4" t="n"/>
@@ -2716,32 +2736,41 @@
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>TC_005</t>
+          <t>TC_004</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>test_lane_mode</t>
+          <t>test_protocol</t>
         </is>
       </c>
       <c r="C6" s="3" t="inlineStr">
         <is>
-          <t>配置条件：
+          <t>TC场景：测试协议帧格式和时序
+配置条件：
 1. test_mode_i=1
 2. 通过WR_CSR(opcode=0x10, addr=0x04, wdata=0x00000001)设置CTRL.EN=1
+其它：以上测试过程中，AHB总线响应正常
 输入激励：
-1. 配置LANE_MODE=00(1-bit模式)，发送AHB_WR32命令，监控pdi_i[0]/pdo_o[0]
-2. 配置LANE_MODE=01(4-bit模式)，发送相同命令，监控pdi_i[3:0]/pdo_o[3:0]
-3. 尝试配置LANE_MODE=10/11，验证配置不变
-4. 验证高nibble优先发送顺序
+1. 发送WR_CSR命令(opcode=0x10)，验证请求阶段：
+   - pcs_n_i拉低
+   - pdi_i输入opcode(8bit)+addr(8bit)+wdata(32bit)
+   - MSB first
+2. 验证turnaround周期：1个clk_i周期，pdo_oe_o=0
+3. 验证响应阶段：pdo_oe_o=1，pdo_o输出status
+4. 发送RD_CSR命令(opcode=0x11)，验证帧格式
+5. 发送AHB_WR32命令(opcode=0x20)，验证帧格式：opcode(8bit)+addr(32bit)+wdata(32bit)
+6. 发送AHB_RD32命令(opcode=0x21)，验证帧格式：opcode(8bit)+addr(32bit)
+7. 验证pcs_n_i拉高结束事务
 期望结果：
-1. 1-bit模式仅使用bit0传输，每拍1bit
-2. 4-bit模式使用全部4bit传输，每拍4bit，高nibble优先
-3. 非法LANE_MODE值不改变配置
-4. 模式切换立即生效
+1. 请求/响应阶段正确分离
+2. turnaround固定1周期，pdo_oe_o=0
+3. 响应阶段pdo_oe_o=1，数据有效
+4. 协议字段MSB first传输
+5. 四种帧格式正确处理
+6. pcs_n_i帧边界清晰
 coverage check点：
-1. LANE_MODE=00/01模式覆盖率
-2. 高nibble优先发送覆盖率</t>
+对四种opcode和帧格式收集功能覆盖率</t>
         </is>
       </c>
       <c r="D6" s="4" t="n"/>
@@ -2749,100 +2778,113 @@
     <row r="7">
       <c r="A7" s="16" t="inlineStr">
         <is>
-          <t>TC_006</t>
+          <t>TC_005</t>
         </is>
       </c>
       <c r="B7" s="16" t="inlineStr">
         <is>
-          <t>test_data_interface</t>
+          <t>test_opcode</t>
         </is>
       </c>
       <c r="C7" s="3" t="inlineStr">
         <is>
-          <t>配置条件：
+          <t>TC场景：测试opcode译码功能
+配置条件：
 1. test_mode_i=1
 2. 通过WR_CSR(opcode=0x10, addr=0x04, wdata=0x00000001)设置CTRL.EN=1
+其它：以上测试过程中，AHB总线空闲
 输入激励：
-1. 在1-bit模式下发送WR_CSR命令(opcode=0x10)，监控pdi_i[0]接收和pdo_o[0]输出
-2. 在4-bit模式下发送AHB_WR32命令(opcode=0x20)，监控pdi_i[3:0]/pdo_o[3:0]
-3. 检查pcs_n_i拉低开始帧，拉高结束帧
-4. 验证MSB first传输顺序
-期望结果：
-1. 数据接口按lane模式正确传输
-2. 帧边界清晰，pcs_n_i正确定义帧边界
-3. MSB first顺序正确
-4. pdo_oe_o在TX阶段=1，其他阶段=0
-coverage check点：
-1. 数据传输模式覆盖率
-2. 帧边界覆盖率</t>
-        </is>
-      </c>
-      <c r="D7" s="14" t="n"/>
-    </row>
-    <row r="8">
-      <c r="A8" s="16" t="inlineStr">
-        <is>
-          <t>TC_007</t>
-        </is>
-      </c>
-      <c r="B8" s="16" t="inlineStr">
-        <is>
-          <t>test_turnaround</t>
-        </is>
-      </c>
-      <c r="C8" s="3" t="inlineStr">
-        <is>
-          <t>配置条件：
-1. test_mode_i=1
-2. 通过WR_CSR(opcode=0x10, addr=0x04, wdata=0x00000001)设置CTRL.EN=1
-输入激励：
-1. 发送WR_CSR命令(opcode=0x10, addr=0x04, wdata=0x00000003)
-2. 监控请求阶段结束后的turnaround周期
-3. 检查pdo_oe_o在turnaround期间=0
-4. 验证响应阶段开始时pdo_oe_o=1
-5. 发送RD_CSR命令(opcode=0x11, addr=0x04)重复验证
-期望结果：
-1. 请求/响应阶段正确分离
-2. turnaround固定1个clk_i周期
-3. 协议字段MSB first传输
-4. 四种命令帧格式正确处理
-coverage check点：
-1. turnaround周期覆盖率
-2. 四种opcode帧格式覆盖率</t>
-        </is>
-      </c>
-      <c r="D8" s="14" t="n"/>
-    </row>
-    <row r="9">
-      <c r="A9" s="16" t="inlineStr">
-        <is>
-          <t>TC_008</t>
-        </is>
-      </c>
-      <c r="B9" s="16" t="inlineStr">
-        <is>
-          <t>test_opcode_decode</t>
-        </is>
-      </c>
-      <c r="C9" s="3" t="inlineStr">
-        <is>
-          <t>配置条件：
-1. test_mode_i=1
-2. 通过WR_CSR(opcode=0x10, addr=0x04, wdata=0x00000001)设置CTRL.EN=1
-3. AHB总线空闲
-输入激励：
-1. 发送opcode=0x10(WR_CSR)命令，验证CSR写操作
-2. 发送opcode=0x11(RD_CSR)命令，验证CSR读操作
-3. 发送opcode=0x20(AHB_WR32)命令，验证AHB写操作
-4. 发送opcode=0x21(AHB_RD32)命令，验证AHB读操作
-5. 发送非法opcode(0x00, 0xFF, 0x30等)，验证返回STS_BAD_OPCODE(0x01)
+1. 发送opcode=0x10执行WR_CSR命令
+2. 发送opcode=0x11执行RD_CSR命令
+3. 发送opcode=0x20执行AHB_WR32命令
+4. 发送opcode=0x21执行AHB_RD32命令
+5. 发送非法opcode(如0x00/0xFF)验证错误处理
+6. 验证前端收满8bit opcode后正确确定期望帧长
 期望结果：
 1. 四种opcode正确译码并执行
 2. 非法opcode返回STS_BAD_OPCODE(0x01)
-3. 前端收满8bit opcode后确定期望帧长
+3. 前端正确确定期望帧长：
+   - WR_CSR: 48bit
+   - RD_CSR: 16bit
+   - AHB_WR32: 72bit
+   - AHB_RD32: 40bit
+4. LAST_ERR寄存器更新为0x01
 coverage check点：
-1. 四种有效opcode覆盖率
-2. 非法opcode检测覆盖率</t>
+对opcode值收集功能覆盖率</t>
+        </is>
+      </c>
+      <c r="D7" s="14" t="n"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="16" t="inlineStr">
+        <is>
+          <t>TC_006</t>
+        </is>
+      </c>
+      <c r="B8" s="16" t="inlineStr">
+        <is>
+          <t>test_config</t>
+        </is>
+      </c>
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t>TC场景：测试配置功能
+配置条件：
+1. test_mode_i=1
+其它：以上测试过程中，AHB总线响应正常
+输入激励：
+1. 写CTRL.EN=1使能模块，发送命令验证功能可执行
+2. 写CTRL.EN=0禁用模块，发送命令验证返回DISABLED错误(0x04)
+3. 配置LANE_MODE=00验证1-bit模式
+4. 配置LANE_MODE=01验证4-bit模式
+5. 配置LANE_MODE=10/11验证非法值处理
+6. 写CTRL.SOFT_RST=1触发软复位
+7. 验证协议上下文清零并恢复默认lane模式
+期望结果：
+1. CTRL.EN配置正确生效
+2. EN=0时命令返回DISABLED(0x04)
+3. LANE_MODE=00/01正确切换lane模式
+4. 非法LANE_MODE值处理正确
+5. SOFT_RST=1触发软复位，上下文清零
+6. 软复位后LANE_MODE恢复00
+coverage check点：
+对CTRL寄存器配置组合收集功能覆盖率</t>
+        </is>
+      </c>
+      <c r="D8" s="14" t="n"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="16" t="inlineStr">
+        <is>
+          <t>TC_007</t>
+        </is>
+      </c>
+      <c r="B9" s="16" t="inlineStr">
+        <is>
+          <t>test_status_poll</t>
+        </is>
+      </c>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>TC场景：测试状态轮询功能
+配置条件：
+1. test_mode_i=1
+2. 通过WR_CSR(opcode=0x10, addr=0x04, wdata=0x00000001)设置CTRL.EN=1
+其它：以上测试过程中，AHB总线响应正常
+输入激励：
+1. 发送正常命令，通过RD_CSR读取STATUS检查busy位
+2. 触发各类错误条件（非法opcode、帧错误等）
+3. 通过RD_CSR(opcode=0x11, addr=0x08)读取STATUS寄存器检查sticky位
+4. 通过RD_CSR(opcode=0x11, addr=0x0C)读取LAST_ERR寄存器获取错误码
+5. 验证无独立中断输出信号
+期望结果：
+1. busy位在事务进行中置1，完成后清0
+2. sticky位在错误后置1
+3. LAST_ERR正确反映最近错误码
+4. MVP版本无中断输出信号
+5. ATE轮询方式正确获取状态
+coverage check点：
+对STATUS和LAST_ERR寄存器状态收集功能覆盖率</t>
         </is>
       </c>
       <c r="D9" s="14" t="n"/>
@@ -2850,34 +2892,38 @@
     <row r="10">
       <c r="A10" s="16" t="inlineStr">
         <is>
-          <t>TC_009</t>
+          <t>TC_008</t>
         </is>
       </c>
       <c r="B10" s="16" t="inlineStr">
         <is>
-          <t>test_ctrl_config</t>
+          <t>test_error_handling</t>
         </is>
       </c>
       <c r="C10" s="3" t="inlineStr">
         <is>
-          <t>配置条件：
+          <t>TC场景：测试异常处理功能
+配置条件：
 1. test_mode_i=1
 2. 通过WR_CSR(opcode=0x10, addr=0x04, wdata=0x00000001)设置CTRL.EN=1
+其它：以上测试过程中，AHB总线正常
 输入激励：
-1. 写CTRL.EN=1使能模块，发送AHB_RD32命令验证可执行
-2. 写CTRL.EN=0禁用模块，发送命令验证返回STS_DISABLED(0x04)
-3. 写CTRL.LANE_MODE=00，验证1-bit模式生效
-4. 写CTRL.LANE_MODE=01，验证4-bit模式生效
-5. 写CTRL.SOFT_RST=1，验证协议上下文清零，恢复默认lane模式
+1. 发送非法opcode(0x00/0xFF)验证BAD_OPCODE(0x01)
+2. 访问非法CSR地址(如0x10)验证BAD_REG(0x02)
+3. 发送非4Byte对齐地址(如0x00001001)验证ALIGN_ERR(0x03)
+4. 设置CTRL.EN=0后发送命令验证DISABLED(0x04)
+5. 设置test_mode_i=0后发送命令验证NOT_IN_TEST(0x05)
+6. 提前拉高pcs_n_i验证FRAME_ERR(0x06)
+7. 触发hresp_i=1验证AHB_ERR(0x07)
+8. 模拟AHB超时验证TIMEOUT(0x08)
 期望结果：
-1. CTRL配置正确生效
-2. 使能/禁用状态切换正确
-3. 软复位功能正常
-4. 软复位不影响CTRL.EN状态
+1. 各类错误正确检测
+2. 返回确定性状态码
+3. LAST_ERR更新正确
+4. 在发起AHB访问前完成前置错误收敛
+5. 响应帧包含正确状态码
 coverage check点：
-1. CTRL.EN使能/禁用覆盖率
-2. LANE_MODE切换覆盖率
-3. SOFT_RST触发覆盖率</t>
+对8类错误码收集功能覆盖率</t>
         </is>
       </c>
       <c r="D10" s="14" t="n"/>
@@ -2885,253 +2931,109 @@
     <row r="11">
       <c r="A11" s="16" t="inlineStr">
         <is>
+          <t>TC_009</t>
+        </is>
+      </c>
+      <c r="B11" s="16" t="inlineStr">
+        <is>
+          <t>test_lowpower</t>
+        </is>
+      </c>
+      <c r="C11" s="3" t="inlineStr">
+        <is>
+          <t>TC场景：测试低功耗功能
+配置条件：
+1. 模块处于空闲态（test_mode_i=0或无有效任务）
+其它：以上测试过程中，AHB总线空闲
+输入激励：
+1. 保持pcs_n_i=1验证接收/发送移位寄存器不翻转
+2. 模拟AHB等待态验证超时计数器仅在WAIT_AHB状态工作
+3. 设置test_mode_i=0验证AHB输出保持IDLE
+4. 切换到工作态验证关键寄存器翻转
+5. 监测状态机状态变化
+期望结果：
+1. 空闲态接收/发送移位寄存器不更新
+2. 超时计数器仅在相关状态工作
+3. test_mode_i=0时htrans_o=IDLE
+4. 无有效任务时AHB输出保持IDLE
+5. 功耗测试通过
+coverage check点：
+对空闲态和工作态转换收集功能覆盖率</t>
+        </is>
+      </c>
+      <c r="D11" s="14" t="n"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="16" t="inlineStr">
+        <is>
           <t>TC_010</t>
         </is>
       </c>
-      <c r="B11" s="16" t="inlineStr">
-        <is>
-          <t>test_status_polling</t>
-        </is>
-      </c>
-      <c r="C11" s="3" t="inlineStr">
-        <is>
-          <t>配置条件：
+      <c r="B12" s="16" t="inlineStr">
+        <is>
+          <t>test_performance</t>
+        </is>
+      </c>
+      <c r="C12" s="3" t="inlineStr">
+        <is>
+          <t>TC场景：测试性能指标和AHB接口功能
+配置条件：
 1. test_mode_i=1
 2. 通过WR_CSR(opcode=0x10, addr=0x04, wdata=0x00000001)设置CTRL.EN=1
+3. 配置clk_i=100MHz
+其它：以上测试过程中，AHB总线响应正常
 输入激励：
-1. 发送非法opcode触发BAD_OPCODE错误
-2. 通过RD_CSR(opcode=0x11, addr=0x0C)读取LAST_ERR寄存器，验证错误码=0x01
-3. 发送AHB_WR32命令，通过RD_CSR(opcode=0x11, addr=0x08)读取STATUS检查busy位
-4. 触发多种错误条件，验证LAST_ERR记录最近错误
-5. 验证无独立中断输出信号
-期望结果：
-1. 所有错误与完成状态通过STATUS/LAST_ERR查询获取
-2. MVP版本无中断输出
-3. ATE轮询方式正确获取状态
-4. LAST_ERR更新正确
-coverage check点：
-1. STATUS寄存器覆盖率
-2. LAST_ERR寄存器覆盖率</t>
-        </is>
-      </c>
-      <c r="D11" s="14" t="n"/>
-    </row>
-    <row r="12">
-      <c r="A12" s="16" t="inlineStr">
-        <is>
-          <t>TC_011</t>
-        </is>
-      </c>
-      <c r="B12" s="16" t="inlineStr">
-        <is>
-          <t>test_exception</t>
-        </is>
-      </c>
-      <c r="C12" s="3" t="inlineStr">
-        <is>
-          <t>配置条件：
-1. test_mode_i=1
-2. 通过WR_CSR(opcode=0x10, addr=0x04, wdata=0x00000001)设置CTRL.EN=1
-3. AHB总线正常
-输入激励：
-1. 发送非法opcode(0x00/0xFF)，验证返回STS_BAD_OPCODE(0x01)
-2. 访问非法CSR地址(0x10)，验证返回STS_BAD_REG(0x02)
-3. 发送非4Byte对齐地址(addr=0x1001)，验证返回STS_ALIGN_ERR(0x03)
-4. CTRL.EN=0时发送命令，验证返回STS_DISABLED(0x04)
-5. test_mode_i=0时发送命令，验证返回STS_NOT_IN_TEST(0x05)
-6. 提前拉高pcs_n_i，验证返回STS_FRAME_ERR(0x06)
-7. 触发hresp_i=1，验证返回STS_AHB_ERR(0x07)
-8. 模拟AHB超时，验证返回STS_TIMEOUT(0x08)
-期望结果：
-1. 各类错误正确检测
-2. 在发起AHB访问前完成前置错误收敛
-3. 返回确定性状态码
-4. LAST_ERR更新正确
-coverage check点：
-1. 8种错误类型覆盖率
-2. 前置错误收敛覆盖率</t>
-        </is>
-      </c>
-      <c r="D12" s="14" t="n"/>
-    </row>
-    <row r="13">
-      <c r="A13" s="16" t="inlineStr">
-        <is>
-          <t>TC_012</t>
-        </is>
-      </c>
-      <c r="B13" s="16" t="inlineStr">
-        <is>
-          <t>test_low_power</t>
-        </is>
-      </c>
-      <c r="C13" s="3" t="inlineStr">
-        <is>
-          <t>配置条件：
-1. 模块处于空闲态
-2. test_mode_i=0或无有效任务
-输入激励：
-1. 保持pcs_n_i=1，监控接收/发送移位寄存器是否翻转
-2. test_mode_i=0，检查AHB输出：htrans_o=0(IDLE)
-3. 模拟AHB等待态，验证超时计数器仅在WAIT_AHB状态工作
-4. 切换到工作态，验证关键寄存器翻转
-期望结果：
-1. 空闲态无效翻转最小化
-2. 低功耗设计目标满足
-3. AHB输出保持IDLE
-4. 功耗测试通过
-coverage check点：
-1. 空闲态覆盖率
-2. 低功耗模式覆盖率</t>
-        </is>
-      </c>
-      <c r="D13" s="14" t="n"/>
-    </row>
-    <row r="14">
-      <c r="A14" s="16" t="inlineStr">
-        <is>
-          <t>TC_013</t>
-        </is>
-      </c>
-      <c r="B14" s="16" t="inlineStr">
-        <is>
-          <t>test_performance</t>
-        </is>
-      </c>
-      <c r="C14" s="3" t="inlineStr">
-        <is>
-          <t>配置条件：
-1. clk_i=100MHz
-2. AHB总线响应正常
-3. test_mode_i=1
-4. 通过WR_CSR(opcode=0x10, addr=0x04, wdata=0x00000001)设置CTRL.EN=1
-输入激励：
-1. 配置LANE_MODE=00(1-bit)，连续执行AHB_RD32/AHB_WR32命令，计算端到端延时和吞吐率
-2. 配置LANE_MODE=01(4-bit)，执行相同测试
-3. 验证1-bit模式链路线速12.5MB/s
-4. 验证4-bit模式链路线速50MB/s
-5. 发送非对齐地址，验证返回ALIGN_ERR
+1. 在1-bit模式下连续执行AHB_RD32/AHB_WR32命令，计算端到端延时和吞吐率
+2. 在4-bit模式下执行相同测试
+3. 验证原始链路线速：1-bit模式12.5MB/s，4-bit模式50MB/s
+4. 验证AHB接口32bit字访问和4Byte对齐约束
+5. 采集状态机状态、opcode、addr、wdata、rdata、status_code
+6. 采集rx/tx计数、pcs_n_i、pdi_i、pdo_o、pdo_oe_o
+7. 验证AHB-Lite Master接口信号时序
 期望结果：
 1. 目标频率100MHz稳定工作
-2. 延时符合预期(约23~24 cycles)
+2. 延时符合预期（约23~24 cycles）
 3. 吞吐率达标
-4. AHB访问约束满足(addr[1:0]=00)
+4. AHB访问约束满足
+5. 所有调试可观测点可采集
+6. AHB-Lite接口符合规范：
+   - htrans_o仅IDLE/NONSEQ
+   - hsize_o固定WORD
+   - hburst_o固定SINGLE
 coverage check点：
-1. 100MHz频率覆盖率
-2. 吞吐率达标覆盖率
-3. 地址对齐约束覆盖率</t>
-        </is>
-      </c>
+对性能指标和AHB信号收集功能覆盖率</t>
+        </is>
+      </c>
+      <c r="D12" s="14" t="n"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="16" t="n"/>
+      <c r="B13" s="16" t="n"/>
+      <c r="C13" s="3" t="n"/>
+      <c r="D13" s="14" t="n"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="16" t="n"/>
+      <c r="B14" s="16" t="n"/>
+      <c r="C14" s="3" t="n"/>
       <c r="D14" s="14" t="n"/>
     </row>
     <row r="15">
-      <c r="A15" s="16" t="inlineStr">
-        <is>
-          <t>TC_014</t>
-        </is>
-      </c>
-      <c r="B15" s="16" t="inlineStr">
-        <is>
-          <t>test_dfx</t>
-        </is>
-      </c>
-      <c r="C15" s="3" t="inlineStr">
-        <is>
-          <t>配置条件：
-1. 仿真环境
-2. test_mode_i=1
-3. 通过WR_CSR(opcode=0x10, addr=0x04, wdata=0x00000001)设置CTRL.EN=1
-输入激励：
-1. 执行WR_CSR命令，采集状态机状态、opcode_reg、addr_reg、wdata_reg
-2. 执行AHB_RD32命令，采集rdata_reg、status_code_reg
-3. 采集rx_count/tx_count计数器
-4. 采集外部接口信号pcs_n_i、pdi_i[3:0]、pdo_o[3:0]、pdo_oe_o
-5. 验证所有调试可观测点可访问
-期望结果：
-1. 所有调试可观测点可采集
-2. 便于联调、波形定位和故障复现
-3. 状态机状态正确转换
-4. 计数器正确计数
-coverage check点：
-1. DFX可观测点覆盖率
-2. 状态机状态覆盖率</t>
-        </is>
-      </c>
+      <c r="A15" s="16" t="n"/>
+      <c r="B15" s="16" t="n"/>
+      <c r="C15" s="3" t="n"/>
       <c r="D15" s="14" t="n"/>
     </row>
     <row r="16">
-      <c r="A16" s="16" t="inlineStr">
-        <is>
-          <t>TC_015</t>
-        </is>
-      </c>
-      <c r="B16" s="16" t="inlineStr">
-        <is>
-          <t>test_memory_map</t>
-        </is>
-      </c>
-      <c r="C16" s="3" t="inlineStr">
-        <is>
-          <t>配置条件：
-1. test_mode_i=1
-2. 通过WR_CSR(opcode=0x10, addr=0x04, wdata=0x00000001)设置CTRL.EN=1
-输入激励：
-1. 通过WR_CSR/RD_CSR访问VERSION寄存器(addr=0x00)
-2. 通过WR_CSR/RD_CSR访问CTRL寄存器(addr=0x04)
-3. 通过WR_CSR/RD_CSR访问STATUS寄存器(addr=0x08)
-4. 通过WR_CSR/RD_CSR访问LAST_ERR寄存器(addr=0x0C)
-5. 发送AHB_WR32命令(opcode=0x20, addr=0x00001000, wdata=0x12345678)访问SoC内部memory-mapped地址
-6. 发送AHB_RD32命令(opcode=0x21, addr=0x00001000)读回验证
-7. 监控AHB地址空间：haddr_o输出32-bit地址
-期望结果：
-1. CSR通过WR_CSR/RD_CSR协议命令正确访问
-2. 模块自身CSR(addr=0x00/0x04/0x08/0x0C)不进入SoC AHB memory map
-3. AHB Master访问采用32-bit地址空间，word访问粒度
-4. haddr_o=0x00001000正确输出
-coverage check点：
-1. CSR地址(0x00~0x0C)覆盖率
-2. AHB地址空间覆盖率</t>
-        </is>
-      </c>
+      <c r="A16" s="16" t="n"/>
+      <c r="B16" s="16" t="n"/>
+      <c r="C16" s="3" t="n"/>
       <c r="D16" s="14" t="n"/>
     </row>
     <row r="17">
-      <c r="A17" s="16" t="inlineStr">
-        <is>
-          <t>TC_016</t>
-        </is>
-      </c>
-      <c r="B17" s="16" t="inlineStr">
-        <is>
-          <t>test_ahb_lite_interface</t>
-        </is>
-      </c>
-      <c r="C17" s="3" t="inlineStr">
-        <is>
-          <t>配置条件：
-1. test_mode_i=1
-2. 通过WR_CSR(opcode=0x10, addr=0x04, wdata=0x00000001)设置CTRL.EN=1
-3. AHB总线空闲
-输入激励：
-1. 发送AHB_WR32命令(opcode=0x20, addr=0x00001000, wdata=0xDEADBEEF)
-2. 监控haddr_o=0x00001000, hwrite_o=1, htrans_o=10(NONSEQ), hsize_o=010(WORD), hburst_o=000(SINGLE)
-3. 监控hwdata_o=0xDEADBEEF
-4. 发送AHB_RD32命令(opcode=0x21, addr=0x00001000)
-5. 监控haddr_o=0x00001000, hwrite_o=0, htrans_o=10(NONSEQ)
-6. 验证hrdata_i接收读数据，hready_i=1, hresp_i=0
-7. 触发hresp_i=1，验证错误处理
-期望结果：
-1. AHB-Lite Master接口符合规范
-2. 单次读写事务正确
-3. 信号时序满足AHB协议要求
-4. hresp_i=1时返回STS_AHB_ERR(0x07)
-coverage check点：
-1. AHB写事务覆盖率
-2. AHB读事务覆盖率
-3. htrans_o状态覆盖率
-4. 错误响应覆盖率</t>
-        </is>
-      </c>
+      <c r="A17" s="16" t="n"/>
+      <c r="B17" s="16" t="n"/>
+      <c r="C17" s="3" t="n"/>
       <c r="D17" s="14" t="n"/>
     </row>
     <row r="18">
@@ -3177,6 +3079,9 @@
       <c r="D24" s="4" t="n"/>
     </row>
   </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:D1"/>
+  </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
skill v0p8 and rtm(plan mode)
</commit_message>
<xml_diff>
--- a/RTM_AI_gen.xlsx
+++ b/RTM_AI_gen.xlsx
@@ -1454,7 +1454,7 @@
       </c>
       <c r="F3" s="31" t="inlineStr">
         <is>
-          <t>TC_010</t>
+          <t>TC_001</t>
         </is>
       </c>
     </row>
@@ -1488,7 +1488,7 @@
       </c>
       <c r="F4" s="31" t="inlineStr">
         <is>
-          <t>TC_001</t>
+          <t>TC_002</t>
         </is>
       </c>
     </row>
@@ -1522,7 +1522,7 @@
       </c>
       <c r="F5" s="31" t="inlineStr">
         <is>
-          <t>TC_002</t>
+          <t>TC_003</t>
         </is>
       </c>
     </row>
@@ -1556,7 +1556,7 @@
       </c>
       <c r="F6" s="31" t="inlineStr">
         <is>
-          <t>TC_003</t>
+          <t>TC_004</t>
         </is>
       </c>
     </row>
@@ -1590,7 +1590,7 @@
       </c>
       <c r="F7" s="31" t="inlineStr">
         <is>
-          <t>TC_003</t>
+          <t>TC_005</t>
         </is>
       </c>
     </row>
@@ -1619,14 +1619,12 @@
       </c>
       <c r="E8" s="31" t="inlineStr">
         <is>
-          <t>CHK_004
-CHK_005</t>
+          <t>CHK_005</t>
         </is>
       </c>
       <c r="F8" s="31" t="inlineStr">
         <is>
-          <t>TC_003
-TC_004</t>
+          <t>TC_006</t>
         </is>
       </c>
     </row>
@@ -1660,7 +1658,7 @@
       </c>
       <c r="F9" s="31" t="inlineStr">
         <is>
-          <t>TC_004</t>
+          <t>TC_007</t>
         </is>
       </c>
     </row>
@@ -1694,7 +1692,7 @@
       </c>
       <c r="F10" s="31" t="inlineStr">
         <is>
-          <t>TC_005</t>
+          <t>TC_008</t>
         </is>
       </c>
     </row>
@@ -1728,7 +1726,7 @@
       </c>
       <c r="F11" s="31" t="inlineStr">
         <is>
-          <t>TC_006</t>
+          <t>TC_009</t>
         </is>
       </c>
     </row>
@@ -1762,7 +1760,7 @@
       </c>
       <c r="F12" s="31" t="inlineStr">
         <is>
-          <t>TC_007</t>
+          <t>TC_010</t>
         </is>
       </c>
     </row>
@@ -1796,7 +1794,7 @@
       </c>
       <c r="F13" s="31" t="inlineStr">
         <is>
-          <t>TC_008</t>
+          <t>TC_011,TC_012,TC_013,TC_014,TC_015,TC_016,TC_017,TC_018</t>
         </is>
       </c>
     </row>
@@ -1830,7 +1828,7 @@
       </c>
       <c r="F14" s="31" t="inlineStr">
         <is>
-          <t>TC_009</t>
+          <t>TC_019</t>
         </is>
       </c>
     </row>
@@ -1864,7 +1862,7 @@
       </c>
       <c r="F15" s="31" t="inlineStr">
         <is>
-          <t>TC_010</t>
+          <t>TC_020</t>
         </is>
       </c>
     </row>
@@ -1893,12 +1891,12 @@
       </c>
       <c r="E16" s="31" t="inlineStr">
         <is>
-          <t>CHK_011</t>
+          <t>CHK_012</t>
         </is>
       </c>
       <c r="F16" s="31" t="inlineStr">
         <is>
-          <t>TC_010</t>
+          <t>TC_021</t>
         </is>
       </c>
     </row>
@@ -1927,12 +1925,12 @@
       </c>
       <c r="E17" s="31" t="inlineStr">
         <is>
-          <t>CHK_003</t>
+          <t>CHK_013</t>
         </is>
       </c>
       <c r="F17" s="31" t="inlineStr">
         <is>
-          <t>TC_002</t>
+          <t>TC_022</t>
         </is>
       </c>
     </row>
@@ -1961,12 +1959,12 @@
       </c>
       <c r="E18" s="31" t="inlineStr">
         <is>
-          <t>CHK_012</t>
+          <t>CHK_014</t>
         </is>
       </c>
       <c r="F18" s="31" t="inlineStr">
         <is>
-          <t>TC_010</t>
+          <t>TC_023</t>
         </is>
       </c>
     </row>
@@ -2141,14 +2139,15 @@
       </c>
       <c r="B3" s="31" t="inlineStr">
         <is>
-          <t>clk_checker</t>
+          <t>clock_domain_checker</t>
         </is>
       </c>
       <c r="C3" s="6" t="inlineStr">
         <is>
-          <t>1. 检查clk_i时钟频率稳定性：在一定数量的时钟周期期间，计算实际周期并判断是否处于目标频率100MHz的允许误差范围内（±3%）
-2. 检查时钟域同步性：验证外部协议采样、状态机控制和AHB-Lite主接口均在clk_i同域工作
-3. 检查时钟信号完整性：无毛刺、无X态或高阻态</t>
+          <t>描述：
+1. 检查clk_i时钟频率稳定性：连续采集clk_i上升沿，计算实际周期，判断是否处于目标频率100MHz的允许误差范围内（±1%，即周期10ns±0.1ns）；
+2. 检查时钟域同步性：验证协议采样（pcs_n_i/pdi_i采样）、状态机控制、AHB-Lite主接口均使用同一clk_i上升沿触发，无跨时钟域数据传输；
+3. 检查clk_i上升沿时，所有内部寄存器和状态机在clk_i上升沿更新状态。</t>
         </is>
       </c>
       <c r="D3" s="4" t="n"/>
@@ -2161,19 +2160,22 @@
       </c>
       <c r="B4" s="18" t="inlineStr">
         <is>
-          <t>reset_checker</t>
+          <t>reset_state_checker</t>
         </is>
       </c>
       <c r="C4" s="17" t="inlineStr">
         <is>
-          <t>1. 检查rst_ni异步复位生效：rst_ni拉低后状态机回到IDLE状态
-2. 检查复位后寄存器默认值：
-   - CTRL.EN=0（模块未使能）
-   - CTRL.LANE_MODE=00（1-bit模式）
-   - STATUS寄存器清零
-   - LAST_ERR寄存器清零
-3. 检查复位释放同步性：内部同步释放，协议上下文和错误状态已清空
-4. 检查复位连接性：rst_ni正确连接至模块并生效</t>
+          <t>描述：
+1. 检查rst_ni异步复位行为：rst_ni低电平有效，异步复位、同步释放；
+2. 检查复位后状态机状态：rst_ni释放后，状态机应处于IDLE状态；
+3. 检查复位后寄存器默认值：
+   - CTRL.EN=0
+   - CTRL.LANE_MODE=2'b00（1-bit模式）
+   - CTRL.SOFT_RST=0
+   - STATUS=0x00
+   - LAST_ERR=0x00
+4. 检查复位后协议上下文：接收/发送移位寄存器清零，超时计数器复位；
+5. 检查复位后AHB接口：htrans_o=2'b00（IDLE），hwrite_o=0，haddr_o=0。</t>
         </is>
       </c>
       <c r="D4" s="4" t="n"/>
@@ -2186,19 +2188,19 @@
       </c>
       <c r="B5" s="31" t="inlineStr">
         <is>
-          <t>csr_checker</t>
+          <t>csr_access_checker</t>
         </is>
       </c>
       <c r="C5" s="6" t="inlineStr">
         <is>
-          <t>1. 检查CSR寄存器读写正确性：
-   - VERSION寄存器(addr=0x00)：只读，通过RD_CSR(opcode=0x11)读取版本号
-   - CTRL寄存器(addr=0x04)：可读写，字段包括EN、LANE_MODE、SOFT_RST
-   - STATUS寄存器(addr=0x08)：只读，反映busy和错误状态
-   - LAST_ERR寄存器(addr=0x0C)：只读，存储最近错误码
-2. 检查CSR访问协议：通过WR_CSR(opcode=0x10)和RD_CSR(opcode=0x11)命令访问
-3. 检查模块自身CSR不进入SoC AHB memory map
-4. 九步法检测寄存器：包含默认值、读写属性、异常地址读写检查</t>
+          <t>描述：
+1. 检查VERSION寄存器读访问：通过opcode=0x11(RD_CSR)读取VERSION，返回值应为设计定义的版本号；
+2. 检查CTRL寄存器读写访问：
+   - 写操作：opcode=0x10(WR_CSR)，检查EN/LANE_MODE/SOFT_RST字段写入后生效
+   - 读操作：opcode=0x11(RD_CSR)，检查读取值与写入值一致
+3. 检查STATUS寄存器读访问：busy位正确反映模块工作状态，错误位sticky行为正确；
+4. 检查LAST_ERR寄存器读访问：存储最近一次错误码，新错误覆盖旧错误；
+5. 检查CSR访问帧格式：请求阶段opcode+wdata，响应阶段status+rdata，符合LRS定义。</t>
         </is>
       </c>
       <c r="D5" s="4" t="n"/>
@@ -2211,17 +2213,20 @@
       </c>
       <c r="B6" s="31" t="inlineStr">
         <is>
-          <t>lane_mode_checker</t>
+          <t>mode_enable_checker</t>
         </is>
       </c>
       <c r="C6" s="6" t="inlineStr">
         <is>
-          <t>1. 检查CTRL.LANE_MODE=00时仅使用pdi_i[0]/pdo_o[0]传输
-2. 验证CTRL.LANE_MODE=01时每拍收发4bit（高nibble优先）：
-   - pdi_i[3:0]/pdo_o[3:0]同时有效
-   - 高nibble优先传输
-3. 确认非法LANE_MODE值(10/11)不改变当前配置或返回错误
-4. 检查lane模式切换时无数据丢失</t>
+          <t>描述：
+1. 检查test_mode_i使能条件：test_mode_i=1时模块才能响应功能命令；
+2. 检查CTRL.EN使能条件：CTRL.EN=1时模块才能执行AHB读写操作；
+3. 检查test_mode_i=1且CTRL.EN=1时：
+   - opcode=0x10/0x11/0x20/0x21命令正常执行
+   - 状态机从IDLE正确跳转
+4. 检查CTRL.EN=0时：AHB_WR32/AHB_RD32命令返回STS_DISABLED(0x04)错误；
+5. 检查test_mode_i=0时：任何命令返回STS_NOT_IN_TEST(0x05)错误；
+6. 检查LANE_MODE配置：仅允许2'b00(1-bit)和2'b01(4-bit)，其他值(2'b10/2'b11)返回错误。</t>
         </is>
       </c>
       <c r="D6" s="4" t="n"/>
@@ -2234,21 +2239,25 @@
       </c>
       <c r="B7" s="12" t="inlineStr">
         <is>
-          <t>protocol_checker</t>
+          <t>lane_mode_checker</t>
         </is>
       </c>
       <c r="C7" s="6" t="inlineStr">
         <is>
-          <t>1. 检查pcs_n_i帧边界：pcs_n_i拉低开启事务，拉高结束事务
-2. 检查turnaround周期：请求阶段后固定1个clk_i周期的turnaround，期间pdo_oe_o=0
-3. 检查pdo_oe_o输出使能：响应阶段pdo_oe_o=1，pdo_o[3:0]输出有效数据
-4. 检查协议字段MSB first传输顺序
-5. 检查四种命令帧格式：
-   - WR_CSR(opcode=0x10): opcode(8bit) + addr(8bit) + wdata(32bit)
-   - RD_CSR(opcode=0x11): opcode(8bit) + addr(8bit)
-   - AHB_WR32(opcode=0x20): opcode(8bit) + addr(32bit) + wdata(32bit)
-   - AHB_RD32(opcode=0x21): opcode(8bit) + addr(32bit)
-6. 检查pdi_i在有效周期内无毛刺切换</t>
+          <t>描述：
+1. 检查1-bit模式（LANE_MODE=2'b00）：
+   - pdi_i[0]作为唯一数据输入
+   - pdo_o[0]作为唯一数据输出
+   - 数据按MSB first逐bit传输
+2. 检查4-bit模式（LANE_MODE=2'b01）：
+   - pdi_i[3:0]全bit有效，按高nibble优先发送
+   - pdo_o[3:0]全bit有效，按高nibble优先接收
+3. 检查pcs_n_i帧边界：
+   - pcs_n_i下降沿标志帧开始
+   - pcs_n_i上升沿标志帧结束
+4. 检查turnaround周期：请求阶段到响应阶段中间固定1个clk_i周期，期间pdo_oe_o=0；
+5. 检查pdo_oe_o输出使能：响应阶段pdo_oe_o=1，请求阶段pdo_oe_o=0；
+6. 检查协议字段MSB first传输顺序。</t>
         </is>
       </c>
       <c r="D7" s="14" t="n"/>
@@ -2261,19 +2270,18 @@
       </c>
       <c r="B8" s="12" t="inlineStr">
         <is>
-          <t>opcode_checker</t>
+          <t>opcode_decoder_checker</t>
         </is>
       </c>
       <c r="C8" s="6" t="inlineStr">
         <is>
-          <t>1. 检查opcode解析正确性：
-   - 8'h10解析为WR_CSR，期望帧长=8+8+32=48bit
-   - 8'h11解析为RD_CSR，期望帧长=8+8=16bit
-   - 8'h20解析为AHB_WR32，期望帧长=8+32+32=72bit
-   - 8'h21解析为AHB_RD32，期望帧长=8+32=40bit
-2. 检查前端在收满8bit opcode后正确确定期望帧长
-3. 检查非法opcode(非0x10/0x11/0x20/0x21)返回STS_BAD_OPCODE(0x01)
-4. 检查opcode译码后正确发起相应任务</t>
+          <t>描述：
+1. 检查opcode=0x10(WR_CSR)解码：前端收满8bit后确定帧长=8bit opcode + 8bit addr + 32bit wdata，任务类型为CSR写；
+2. 检查opcode=0x11(RD_CSR)解码：帧长=8bit opcode + 8bit addr，任务类型为CSR读；
+3. 检查opcode=0x20(AHB_WR32)解码：帧长=8bit opcode + 32bit addr + 32bit wdata，任务类型为AHB写；
+4. 检查opcode=0x21(AHB_RD32)解码：帧长=8bit opcode + 32bit addr，任务类型为AHB读；
+5. 检查非法opcode检测：opcode=0x00/0xFF等未定义值，返回STS_BAD_OPCODE(0x01)错误码；
+6. 检查opcode解析时序：在收满8bit opcode后的下一个clk_i周期完成解码。</t>
         </is>
       </c>
       <c r="D8" s="14" t="n"/>
@@ -2286,23 +2294,24 @@
       </c>
       <c r="B9" s="12" t="inlineStr">
         <is>
-          <t>config_checker</t>
+          <t>config_register_checker</t>
         </is>
       </c>
       <c r="C9" s="6" t="inlineStr">
         <is>
-          <t>1. 检查CTRL.EN配置生效：
-   - EN=1时模块使能，功能命令可执行
-   - EN=0时模块禁用，命令返回DISABLED错误(0x04)
-2. 检查CTRL.LANE_MODE配置生效：
-   - LANE_MODE=00时1-bit模式
-   - LANE_MODE=01时4-bit模式
-   - LANE_MODE=10/11时保持当前配置或返回错误
-3. 检查CTRL.SOFT_RST功能：
-   - SOFT_RST写1触发协议上下文清零
-   - 恢复默认lane模式(LANE_MODE=00)
-   - 不影响CTRL.EN配置
-4. 检查配置变更时序：配置立即生效或下一事务生效</t>
+          <t>描述：
+1. 检查CTRL.EN配置：
+   - 写入EN=1后，模块使能，可响应功能命令
+   - 写入EN=0后，模块禁用，功能命令返回STS_DISABLED(0x04)
+2. 检查CTRL.LANE_MODE配置：
+   - LANE_MODE=2'b00：切换到1-bit模式
+   - LANE_MODE=2'b01：切换到4-bit模式
+   - LANE_MODE=2'b10/2'b11：非法配置，保持原模式
+3. 检查CTRL.SOFT_RST软复位：
+   - 写入SOFT_RST=1触发软复位
+   - 软复位后：协议上下文清零，LANE_MODE恢复默认(2'b00)
+   - SOFT_RST为write-1-to-trigger，写后自动清零
+4. 检查配置生效时序：配置写入后在下一个clk_i上升沿生效。</t>
         </is>
       </c>
       <c r="D9" s="14" t="n"/>
@@ -2315,19 +2324,23 @@
       </c>
       <c r="B10" s="12" t="inlineStr">
         <is>
-          <t>status_checker</t>
+          <t>status_polling_checker</t>
         </is>
       </c>
       <c r="C10" s="6" t="inlineStr">
         <is>
-          <t>1. 检查STATUS寄存器状态位：
-   - busy位：事务进行中置1，完成后清0
-   - sticky位：错误发生后置1，需软件清零
-2. 检查LAST_ERR寄存器更新：
-   - 每次错误发生后更新为对应状态码
-   - 成功操作后保持原值或清零
-3. 检查无独立中断输出：MVP版本不实现中断信号
-4. 检查ATE轮询方式获取状态的正确性</t>
+          <t>描述：
+1. 检查STATUS寄存器状态：
+   - STATUS[7:0]反映命令执行状态（busy、error等标志位）
+   - STATUS.sticky位行为：错误标志一旦置位，需要显式清除
+2. 检查LAST_ERR寄存器：
+   - 存储最近一次错误的错误码
+   - 新错误发生时覆盖旧值
+   - 成功命令不更新LAST_ERR
+3. 检查轮询机制：
+   - MVP版本无独立中断输出
+   - 所有状态通过STATUS/LAST_ERR轮询获取
+4. 检查无中断输出：确认设计未实现中断信号线。</t>
         </is>
       </c>
       <c r="D10" s="14" t="n"/>
@@ -2340,25 +2353,21 @@
       </c>
       <c r="B11" s="12" t="inlineStr">
         <is>
-          <t>error_checker</t>
+          <t>error_detection_checker</t>
         </is>
       </c>
       <c r="C11" s="6" t="inlineStr">
         <is>
-          <t>检查8类错误的检测和状态码生成：
-1. BAD_OPCODE(0x01): opcode不在{0x10,0x11,0x20,0x21}范围内
-2. BAD_REG(0x02): CSR地址不在{0x00,0x04,0x08,0x0C}范围内
-3. ALIGN_ERR(0x03): AHB访问地址未4Byte对齐（addr[1:0]!=00）
-4. DISABLED(0x04): CTRL.EN=0时发送功能命令
-5. NOT_IN_TEST(0x05): test_mode_i=0时发送功能命令
-6. FRAME_ERR(0x06): pcs_n_i提前拉高导致帧不完整
-7. AHB_ERR(0x07): hresp_i=1表示AHB错误响应
-8. TIMEOUT(0x08): AHB访问超时
-检查点：
-- 在发起AHB访问前完成前置错误收敛
-- 返回确定性状态码
-- LAST_ERR寄存器正确更新
-- 响应帧包含正确状态码</t>
+          <t>描述：
+1. 检查BAD_OPCODE(0x01)错误：opcode值非0x10/0x11/0x20/0x21，返回status_code=0x01；
+2. 检查BAD_REG(0x02)错误：访问未定义的CSR地址，返回status_code=0x02；
+3. 检查ALIGN_ERR(0x03)错误：AHB_WR32/AHB_RD32的addr[1:0]!=2'b00，返回status_code=0x03；
+4. 检查DISABLED(0x04)错误：CTRL.EN=0时发送功能命令，返回status_code=0x04；
+5. 检查NOT_IN_TEST(0x05)错误：test_mode_i=0时发送命令，返回status_code=0x05；
+6. 检查FRAME_ERR(0x06)错误：pcs_n_i在帧传输过程中提前拉高，返回status_code=0x06；
+7. 检查AHB_ERR(0x07)错误：hresp_i=1（ERROR response），返回status_code=0x07；
+8. 检查TIMEOUT(0x08)错误：AHB访问超时（hready_i长时间为0），返回status_code=0x08；
+9. 检查前置错误收敛：在发起AHB访问前完成所有前置错误检测（BAD_OPCODE/BAD_REG/ALIGN_ERR/DISABLED/NOT_IN_TEST/FRAME_ERR）。</t>
         </is>
       </c>
       <c r="D11" s="14" t="n"/>
@@ -2371,19 +2380,26 @@
       </c>
       <c r="B12" s="12" t="inlineStr">
         <is>
-          <t>lowpower_checker</t>
+          <t>lowpower_behavior_checker</t>
         </is>
       </c>
       <c r="C12" s="6" t="inlineStr">
         <is>
-          <t>1. 检查空闲态下无效翻转最小化：
-   - 接收/发送移位寄存器不更新（pcs_n_i=1时）
-   - 超时计数器仅在RX/TX/WAIT_AHB相关状态工作
-2. 检查test_mode_i=0时AHB输出保持IDLE：
-   - htrans_o=IDLE(2'b00)
-   - hwrite_o、hsize_o、hburst_o无效
-3. 检查无有效任务时AHB输出保持IDLE
-4. 检查仅关键状态(RX/TX/WAIT_AHB)翻转时寄存器更新</t>
+          <t>描述：
+1. 检查空闲态寄存器行为：
+   - pcs_n_i=1时，接收移位寄存器不更新
+   - 无TX任务时，发送移位寄存器不更新
+2. 检查超时计数器：
+   - 仅在WAIT_AHB状态（等待AHB响应）时超时计数器工作
+   - 其他状态计数器保持复位值
+3. 检查test_mode_i=0时的AHB输出：
+   - htrans_o=2'b00（IDLE）
+   - hwrite_o=0
+   - haddr_o/hwdata_o保持上一次值或复位值
+4. 检查工作态寄存器翻转：
+   - RX状态：接收移位寄存器每个clk_i更新
+   - TX状态：发送移位寄存器每个clk_i更新
+   - WAIT_AHB状态：超时计数器递增</t>
         </is>
       </c>
       <c r="D12" s="14" t="n"/>
@@ -2396,22 +2412,23 @@
       </c>
       <c r="B13" s="12" t="inlineStr">
         <is>
-          <t>perf_checker</t>
+          <t>performance_checker</t>
         </is>
       </c>
       <c r="C13" s="6" t="inlineStr">
         <is>
-          <t>1. 检查目标频率100MHz稳定工作
+          <t>描述：
+1. 检查时钟频率：clk_i稳定工作在100MHz（周期10ns），误差±1%；
 2. 检查端到端延时：
-   - 1-bit模式：约23~24 cycles
-   - 4-bit模式：相应缩短
-3. 检查原始链路线速：
-   - 1-bit模式：12.5MB/s
-   - 4-bit模式：50MB/s
-4. 检查AHB接口约束：
-   - 32bit字访问
-   - 地址4Byte对齐
-5. 检查吞吐率达标</t>
+   - 从pcs_n_i下降沿（帧开始）到pcs_n_i上升沿（帧结束）的总周期数
+   - 预期约23~24 cycles（含turnaround）
+3. 检查吞吐率：
+   - 1-bit模式：原始链路线速12.5MB/s（100MHz/8）
+   - 4-bit模式：原始链路线速50MB/s（100MHz/4*2）
+4. 检查AHB访问粒度：
+   - hsize_o固定为3'b010（32-bit WORD访问）
+   - 地址haddr_o[1:0]=2'b00（4Byte对齐）
+5. 检查AHB事务效率：单次AHB读写事务在hready_i=1时耗时2 cycles（地址相+数据相）。</t>
         </is>
       </c>
       <c r="D13" s="14" t="n"/>
@@ -2424,40 +2441,85 @@
       </c>
       <c r="B14" s="12" t="inlineStr">
         <is>
-          <t>ahb_checker</t>
+          <t>debug_observability_checker</t>
         </is>
       </c>
       <c r="C14" s="6" t="inlineStr">
         <is>
-          <t>1. 检查AHB-Lite Master接口信号：
-   - haddr_o: 32-bit地址输出
-   - hwrite_o: 读写标志（1=写，0=读）
-   - htrans_o: 仅输出IDLE(2'b00)或NONSEQ(2'b10)
-   - hsize_o: 固定为WORD(3'b010，32-bit)
-   - hburst_o: 固定为SINGLE(3'b000)
-   - hwdata_o: 32-bit写数据
-2. 检查AHB读响应：
-   - hrdata_i: 32-bit读返回数据
-   - hready_i: ready信号
-   - hresp_i: 错误响应（0=OKAY，1=ERROR）
-3. 检查AHB事务时序：
+          <t>描述：
+1. 检查状态机状态可观测性：内部fsm_state信号可通过波形或调试接口访问；
+2. 检查opcode可观测性：当前正在处理的opcode值可访问；
+3. 检查地址/数据可观测性：
+   - addr寄存器（当前访问地址）可访问
+   - wdata寄存器（写数据）可访问
+   - rdata寄存器（读返回数据）可访问
+4. 检查status_code可观测性：当前命令的status_code可访问；
+5. 检查rx/tx计数器可观测性：接收/发送bit计数器值可访问；
+6. 检查接口信号可观测性：pcs_n_i、pdi_i、pdo_o、pdo_oe_o可通过波形直接观测。</t>
+        </is>
+      </c>
+      <c r="D14" s="14" t="n"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="12" t="inlineStr">
+        <is>
+          <t>CHK_013</t>
+        </is>
+      </c>
+      <c r="B15" s="12" t="inlineStr">
+        <is>
+          <t>memory_map_checker</t>
+        </is>
+      </c>
+      <c r="C15" s="6" t="inlineStr">
+        <is>
+          <t>描述：
+1. 检查CSR访问方式：
+   - 模块内部CSR（VERSION/CTRL/STATUS/LAST_ERR）通过协议命令访问
+   - CSR不映射到SoC AHB memory map
+2. 检查AHB Master访问：
+   - AHB_WR32/AHB_RD32命令访问SoC内部memory-mapped地址
+   - haddr_o为32bit地址空间
+   - 访问粒度为32-bit word
+3. 检查地址空间约束：
+   - 具体可达目标地址范围由SoC顶层约束
+   - 模块不检查地址有效性（由AHB slave响应）</t>
+        </is>
+      </c>
+      <c r="D15" s="14" t="n"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="12" t="inlineStr">
+        <is>
+          <t>CHK_014</t>
+        </is>
+      </c>
+      <c r="B16" s="12" t="inlineStr">
+        <is>
+          <t>ahb_protocol_checker</t>
+        </is>
+      </c>
+      <c r="C16" s="6" t="inlineStr">
+        <is>
+          <t>描述：
+1. 检查AHB-Lite Master信号：
+   - haddr_o[31:0]：32bit地址输出
+   - hwrite_o：写使能（1=写，0=读）
+   - htrans_o[1:0]：仅输出IDLE(2'b00)或NONSEQ(2'b10)
+   - hsize_o[2:0]：固定为WORD(3'b010)，表示32bit传输
+   - hburst_o[2:0]：固定为SINGLE(3'b000)，单次传输
+   - hwdata_o[31:0]：写数据输出
+2. 检查AHB时序：
    - 地址相：haddr_o、hwrite_o、htrans_o、hsize_o、hburst_o有效
-   - 数据相：hwdata_o（写）或hrdata_i（读）有效
-4. 检查控制命令正确转换为AHB-Lite单次读写事务</t>
-        </is>
-      </c>
-      <c r="D14" s="14" t="n"/>
-    </row>
-    <row r="15">
-      <c r="A15" s="12" t="n"/>
-      <c r="B15" s="12" t="n"/>
-      <c r="C15" s="6" t="n"/>
-      <c r="D15" s="14" t="n"/>
-    </row>
-    <row r="16">
-      <c r="A16" s="12" t="n"/>
-      <c r="B16" s="12" t="n"/>
-      <c r="C16" s="6" t="n"/>
+   - 数据相：hwdata_o有效（写操作时）
+   - hready_i=1时事务推进
+3. 检查AHB响应：
+   - hrdata_i[31:0]：读返回数据
+   - hready_i：总线ready信号
+   - hresp_i：错误响应（1=ERROR，0=OKAY）
+4. 检查单次读写事务时序符合AMBA AHB-Lite协议规范。</t>
+        </is>
+      </c>
       <c r="D16" s="14" t="n"/>
     </row>
     <row r="17">
@@ -2576,7 +2638,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D24"/>
+  <dimension ref="A1:D25"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="9" defaultRowHeight="13.5"/>
   <cols>
     <col width="13.75" customWidth="1" style="24" min="1" max="1"/>
@@ -2625,31 +2687,26 @@
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>test_reset</t>
+          <t>test_clock_domain</t>
         </is>
       </c>
       <c r="C3" s="3" t="inlineStr">
         <is>
-          <t>TC场景：测试模块复位功能
-配置条件：
-1. 初始状态rst_ni=0，模块处于复位状态
-2. test_mode_i=1
-其它：以上测试过程中，不关心的配置或接口控制信号随机
+          <t>配置条件：
+1. 配置clk_i时钟频率为100MHz；
+2. 模块解复位，test_mode_i=1；
 输入激励：
-1. 释放rst_ni，等待复位同步释放完成
-2. 通过RD_CSR(opcode=0x11, addr=0x04)读取CTRL寄存器
-3. 通过RD_CSR(opcode=0x11, addr=0x08)读取STATUS寄存器
-4. 通过RD_CSR(opcode=0x11, addr=0x0C)读取LAST_ERR寄存器
-5. 监测状态机状态
+1. 通过WR_CSR(opcode=0x10)配置CTRL.EN=1；
+2. 在1-bit模式(LANE_MODE=2'b00)下，连续发送AHB_RD32(opcode=0x21)和AHB_WR32(opcode=0x20)命令各10次；
+3. 切换到4-bit模式(LANE_MODE=2'b01)，重复步骤2；
 期望结果：
-1. 复位后状态机处于IDLE状态
-2. CTRL.EN=0（模块未使能）
-3. CTRL.LANE_MODE=00（1-bit模式默认值）
-4. STATUS寄存器清零
-5. LAST_ERR寄存器清零
-6. 协议上下文和错误状态已清空
+1. 所有命令在100MHz频率下正确执行；
+2. 协议采样在clk_i上升沿正确捕获pdi_i数据；
+3. 状态机控制在clk_i上升沿正确跳转；
+4. AHB-Lite主接口在clk_i上升沿正确输出信号；
+5. 无时序违例，无跨时钟域问题；
 coverage check点：
-对复位后寄存器默认值收集功能覆盖率</t>
+对lane模式(1-bit/4-bit)和命令类型(RD/WR)的组合收集功能覆盖率。</t>
         </is>
       </c>
       <c r="D3" s="4" t="n"/>
@@ -2662,35 +2719,29 @@
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>test_csr_access</t>
+          <t>test_reset_sequence</t>
         </is>
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
-          <t>TC场景：测试CSR寄存器访问和memory map功能
-配置条件：
-1. test_mode_i=1
-2. 通过WR_CSR(opcode=0x10, addr=0x04, wdata=0x00000001)设置CTRL.EN=1
-其它：以上测试过程中，AHB总线空闲
+          <t>配置条件：
+1. 初始状态rst_ni=0，模块处于复位状态；
 输入激励：
-1. 通过RD_CSR(opcode=0x11, addr=0x00)读取VERSION寄存器
-2. 通过WR_CSR(opcode=0x10, addr=0x00, wdata=0xFFFFFFFF)尝试写VERSION寄存器，验证只读属性
-3. 通过WR_CSR(opcode=0x10, addr=0x04, wdata=0x00000003)写CTRL寄存器（EN=1, LANE_MODE=01）
-4. 通过RD_CSR(opcode=0x11, addr=0x04)读取CTRL寄存器
-5. 通过RD_CSR(opcode=0x11, addr=0x08)读取STATUS寄存器
-6. 发送AHB_WR32命令(opcode=0x20, addr=0x00001000, wdata=0x12345678)访问SoC内部memory-mapped地址
-7. 发送AHB_RD32命令(opcode=0x21, addr=0x00001000)读回验证
-8. 监控haddr_o输出
+1. 释放rst_ni（拉高），等待1个clk_i周期；
+2. 通过RD_CSR(opcode=0x11)读取CTRL寄存器，检查默认值；
+3. 通过RD_CSR(opcode=0x11)读取STATUS寄存器，检查默认值；
+4. 通过RD_CSR(opcode=0x11)读取LAST_ERR寄存器，检查默认值；
+5. 检查状态机状态（通过波形或调试接口）；
 期望结果：
-1. CSR通过WR_CSR/RD_CSR协议命令正确访问
-2. VERSION寄存器只读，写入后读回原值
-3. CTRL寄存器读写正确，配置生效
-4. STATUS寄存器反映正确状态
-5. AHB_WR32/AHB_RD32正确访问SoC memory-mapped地址，haddr_o=0x00001000
-6. 模块自身CSR(addr=0x00/0x04/0x08/0x0C)不进入SoC AHB memory map
-7. AHB Master访问采用32-bit地址空间，word访问粒度
+1. rst_ni释放后，状态机处于IDLE状态；
+2. CTRL.EN=0；
+3. CTRL.LANE_MODE=2'b00（1-bit模式）；
+4. CTRL.SOFT_RST=0；
+5. STATUS=0x00；
+6. LAST_ERR=0x00；
+7. 协议上下文清零，无残留状态；
 coverage check点：
-对CSR地址(0x00~0x0C)和AHB地址空间收集功能覆盖率</t>
+直接用例覆盖，不收功能覆盖率。</t>
         </is>
       </c>
       <c r="D4" s="4" t="n"/>
@@ -2703,32 +2754,30 @@
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>test_lane_mode</t>
+          <t>test_csr_access</t>
         </is>
       </c>
       <c r="C5" s="3" t="inlineStr">
         <is>
-          <t>TC场景：测试lane模式配置和数据接口功能
-配置条件：
-1. test_mode_i=1
-2. 通过WR_CSR(opcode=0x10, addr=0x04, wdata=0x00000001)设置CTRL.EN=1
-其它：以上测试过程中，AHB总线响应正常
+          <t>配置条件：
+1. 模块解复位，test_mode_i=1；
+2. 通过WR_CSR(opcode=0x10)配置CTRL.EN=1；
 输入激励：
-1. 配置LANE_MODE=00（1-bit模式），发送AHB_RD32命令验证
-2. 验证pdi_i[0]/pdo_o[0]数据传输，pdi_i[3:1]/pdo_o[3:1]无效
-3. 配置LANE_MODE=01（4-bit模式），发送相同命令
-4. 验证pdi_i[3:0]/pdo_o[3:0]同时有效，高nibble优先发送
-5. 尝试配置非法LANE_MODE值(10/11)，验证错误处理
-6. 验证pcs_n_i帧边界正确：拉低开启事务，拉高结束事务
-7. 验证协议字段MSB first传输顺序
+1. 通过RD_CSR(opcode=0x11)读取VERSION寄存器，记录版本号；
+2. 通过WR_CSR(opcode=0x10)写入CTRL.EN=1, LANE_MODE=2'b01；
+3. 通过RD_CSR(opcode=0x11)读取CTRL寄存器，验证写入值；
+4. 通过WR_CSR(opcode=0x10)写入CTRL.EN=1, LANE_MODE=2'b00；
+5. 通过RD_CSR(opcode=0x11)读取CTRL寄存器，验证写入值；
+6. 执行一个AHB_WR32命令，然后通过RD_CSR读取STATUS检查busy位；
+7. 触发一个错误条件，然后通过RD_CSR读取LAST_ERR检查错误码；
 期望结果：
-1. 1-bit模式仅使用bit0传输，协议正确
-2. 4-bit模式每拍收发4bit，高nibble优先
-3. 非法LANE_MODE值(10/11)返回错误或保持当前配置
-4. pcs_n_i帧边界清晰
-5. MSB first传输顺序正确
+1. VERSION寄存器返回预期版本号；
+2. CTRL寄存器读写正确，EN/LANE_MODE字段配置生效；
+3. STATUS寄存器busy位在命令执行期间为1，完成后为0；
+4. LAST_ERR寄存器正确记录最近错误码；
+5. CSR访问帧格式正确：请求阶段opcode+addr+wdata，响应阶段status+rdata；
 coverage check点：
-对LANE_MODE配置值和数据传输模式收集功能覆盖率</t>
+对CSR寄存器(VERSION/CTRL/STATUS/LAST_ERR)和访问类型(读/写)收集功能覆盖率。</t>
         </is>
       </c>
       <c r="D5" s="4" t="n"/>
@@ -2741,36 +2790,28 @@
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>test_protocol</t>
+          <t>test_mode_enable</t>
         </is>
       </c>
       <c r="C6" s="3" t="inlineStr">
         <is>
-          <t>TC场景：测试协议帧格式和时序
-配置条件：
-1. test_mode_i=1
-2. 通过WR_CSR(opcode=0x10, addr=0x04, wdata=0x00000001)设置CTRL.EN=1
-其它：以上测试过程中，AHB总线响应正常
+          <t>配置条件：
+1. 模块解复位；
 输入激励：
-1. 发送WR_CSR命令(opcode=0x10)，验证请求阶段：
-   - pcs_n_i拉低
-   - pdi_i输入opcode(8bit)+addr(8bit)+wdata(32bit)
-   - MSB first
-2. 验证turnaround周期：1个clk_i周期，pdo_oe_o=0
-3. 验证响应阶段：pdo_oe_o=1，pdo_o输出status
-4. 发送RD_CSR命令(opcode=0x11)，验证帧格式
-5. 发送AHB_WR32命令(opcode=0x20)，验证帧格式：opcode(8bit)+addr(32bit)+wdata(32bit)
-6. 发送AHB_RD32命令(opcode=0x21)，验证帧格式：opcode(8bit)+addr(32bit)
-7. 验证pcs_n_i拉高结束事务
+1. test_mode_i=0，发送WR_CSR(opcode=0x10)命令，检查响应；
+2. test_mode_i=1，发送WR_CSR(opcode=0x10)命令写CTRL.EN=0；
+3. test_mode_i=1, CTRL.EN=0，发送AHB_RD32(opcode=0x21)命令，检查响应；
+4. test_mode_i=1，通过WR_CSR写CTRL.EN=1；
+5. test_mode_i=1, CTRL.EN=1，发送AHB_RD32命令，检查响应；
+6. 通过WR_CSR写CTRL.EN=0；
+7. 发送AHB_RD32命令，检查响应；
 期望结果：
-1. 请求/响应阶段正确分离
-2. turnaround固定1周期，pdo_oe_o=0
-3. 响应阶段pdo_oe_o=1，数据有效
-4. 协议字段MSB first传输
-5. 四种帧格式正确处理
-6. pcs_n_i帧边界清晰
+1. test_mode_i=0时，命令返回STS_NOT_IN_TEST(0x05)；
+2. CTRL.EN=0时，AHB_WR32/AHB_RD32命令返回STS_DISABLED(0x04)；
+3. test_mode_i=1且CTRL.EN=1时，命令正常执行，status=0x00；
+4. 半双工请求/响应模式工作正常；
 coverage check点：
-对四种opcode和帧格式收集功能覆盖率</t>
+对test_mode_i(0/1)和CTRL.EN(0/1)的组合收集功能覆盖率。</t>
         </is>
       </c>
       <c r="D6" s="4" t="n"/>
@@ -2783,34 +2824,29 @@
       </c>
       <c r="B7" s="16" t="inlineStr">
         <is>
-          <t>test_opcode</t>
+          <t>test_lane_mode</t>
         </is>
       </c>
       <c r="C7" s="3" t="inlineStr">
         <is>
-          <t>TC场景：测试opcode译码功能
-配置条件：
-1. test_mode_i=1
-2. 通过WR_CSR(opcode=0x10, addr=0x04, wdata=0x00000001)设置CTRL.EN=1
-其它：以上测试过程中，AHB总线空闲
+          <t>配置条件：
+1. 模块解复位，test_mode_i=1；
+2. 通过WR_CSR(opcode=0x10)配置CTRL.EN=1；
 输入激励：
-1. 发送opcode=0x10执行WR_CSR命令
-2. 发送opcode=0x11执行RD_CSR命令
-3. 发送opcode=0x20执行AHB_WR32命令
-4. 发送opcode=0x21执行AHB_RD32命令
-5. 发送非法opcode(如0x00/0xFF)验证错误处理
-6. 验证前端收满8bit opcode后正确确定期望帧长
+1. 通过WR_CSR配置LANE_MODE=2'b00（1-bit模式）；
+2. 发送AHB_RD32(opcode=0x21)命令，观察pdi_i[0]和pdo_o[0]；
+3. 通过WR_CSR配置LANE_MODE=2'b01（4-bit模式）；
+4. 发送AHB_RD32命令，观察pdi_i[3:0]和pdo_o[3:0]；
+5. 尝试配置LANE_MODE=2'b10（非法值）；
+6. 尝试配置LANE_MODE=2'b11（非法值）；
+7. 发送AHB_RD32命令，验证当前lane模式；
 期望结果：
-1. 四种opcode正确译码并执行
-2. 非法opcode返回STS_BAD_OPCODE(0x01)
-3. 前端正确确定期望帧长：
-   - WR_CSR: 48bit
-   - RD_CSR: 16bit
-   - AHB_WR32: 72bit
-   - AHB_RD32: 40bit
-4. LAST_ERR寄存器更新为0x01
+1. LANE_MODE=2'b00时，1-bit模式正常工作；
+2. LANE_MODE=2'b01时，4-bit模式正常工作；
+3. LANE_MODE=2'b10/2'b11时，配置被拒绝或保持原模式；
+4. Burst和AXI后端功能确认不可用；
 coverage check点：
-对opcode值收集功能覆盖率</t>
+对LANE_MODE值(00/01/10/11)收集功能覆盖率。</t>
         </is>
       </c>
       <c r="D7" s="14" t="n"/>
@@ -2823,32 +2859,31 @@
       </c>
       <c r="B8" s="16" t="inlineStr">
         <is>
-          <t>test_config</t>
+          <t>test_data_interface_1bit</t>
         </is>
       </c>
       <c r="C8" s="3" t="inlineStr">
         <is>
-          <t>TC场景：测试配置功能
-配置条件：
-1. test_mode_i=1
-其它：以上测试过程中，AHB总线响应正常
+          <t>配置条件：
+1. 模块解复位，test_mode_i=1；
+2. 通过WR_CSR(opcode=0x10)配置CTRL.EN=1, LANE_MODE=2'b00（1-bit模式）；
 输入激励：
-1. 写CTRL.EN=1使能模块，发送命令验证功能可执行
-2. 写CTRL.EN=0禁用模块，发送命令验证返回DISABLED错误(0x04)
-3. 配置LANE_MODE=00验证1-bit模式
-4. 配置LANE_MODE=01验证4-bit模式
-5. 配置LANE_MODE=10/11验证非法值处理
-6. 写CTRL.SOFT_RST=1触发软复位
-7. 验证协议上下文清零并恢复默认lane模式
+1. 发送WR_CSR(opcode=0x10)命令，输入opcode=0b00010000逐bit到pdi_i[0]；
+2. 检查pcs_n_i下降沿标志帧开始；
+3. 观察pdi_i[0]数据接收顺序为MSB first；
+4. 观察turnaround周期：请求阶段后1个clk_i周期pdo_oe_o=0；
+5. 观察响应阶段pdo_oe_o=1，pdo_o[0]逐bit输出；
+6. 检查pcs_n_i上升沿标志帧结束；
+7. 发送AHB_WR32(opcode=0x20)命令，重复上述观察；
 期望结果：
-1. CTRL.EN配置正确生效
-2. EN=0时命令返回DISABLED(0x04)
-3. LANE_MODE=00/01正确切换lane模式
-4. 非法LANE_MODE值处理正确
-5. SOFT_RST=1触发软复位，上下文清零
-6. 软复位后LANE_MODE恢复00
+1. pcs_n_i帧边界正确：下降沿开始，上升沿结束；
+2. pdi_i[0]在1-bit模式下接收数据正确；
+3. pdo_o[0]在1-bit模式下输出数据正确；
+4. turnaround固定1个clk_i周期；
+5. 数据传输MSB first顺序正确；
+6. pdo_oe_o方向控制正确；
 coverage check点：
-对CTRL寄存器配置组合收集功能覆盖率</t>
+对帧类型(WR_CSR/RD_CSR/AHB_WR32/AHB_RD32)收集功能覆盖率。</t>
         </is>
       </c>
       <c r="D8" s="14" t="n"/>
@@ -2861,30 +2896,32 @@
       </c>
       <c r="B9" s="16" t="inlineStr">
         <is>
-          <t>test_status_poll</t>
+          <t>test_data_interface_4bit</t>
         </is>
       </c>
       <c r="C9" s="3" t="inlineStr">
         <is>
-          <t>TC场景：测试状态轮询功能
-配置条件：
-1. test_mode_i=1
-2. 通过WR_CSR(opcode=0x10, addr=0x04, wdata=0x00000001)设置CTRL.EN=1
-其它：以上测试过程中，AHB总线响应正常
+          <t>配置条件：
+1. 模块解复位，test_mode_i=1；
+2. 通过WR_CSR(opcode=0x10)配置CTRL.EN=1, LANE_MODE=2'b01（4-bit模式）；
 输入激励：
-1. 发送正常命令，通过RD_CSR读取STATUS检查busy位
-2. 触发各类错误条件（非法opcode、帧错误等）
-3. 通过RD_CSR(opcode=0x11, addr=0x08)读取STATUS寄存器检查sticky位
-4. 通过RD_CSR(opcode=0x11, addr=0x0C)读取LAST_ERR寄存器获取错误码
-5. 验证无独立中断输出信号
+1. 发送WR_CSR(opcode=0x10)命令，输入opcode=0x10到pdi_i[3:0]（2拍）；
+2. 观察pdi_i[3:0]按高nibble优先接收；
+3. 发送AHB_RD32(opcode=0x21)命令，包含opcode+addr共10拍；
+4. 观察turnaround周期：请求阶段后1个clk_i周期pdo_oe_o=0；
+5. 观察响应阶段pdo_oe_o=1，pdo_o[3:0]按高nibble优先输出；
+6. 验证四种命令帧格式：
+   - WR_CSR(0x10)：8bit opcode + 8bit addr + 32bit wdata
+   - RD_CSR(0x11)：8bit opcode + 8bit addr
+   - AHB_WR32(0x20)：8bit opcode + 32bit addr + 32bit wdata
+   - AHB_RD32(0x21)：8bit opcode + 32bit addr；
 期望结果：
-1. busy位在事务进行中置1，完成后清0
-2. sticky位在错误后置1
-3. LAST_ERR正确反映最近错误码
-4. MVP版本无中断输出信号
-5. ATE轮询方式正确获取状态
+1. pdi_i[3:0]在4-bit模式下按高nibble优先接收正确；
+2. pdo_o[3:0]在4-bit模式下按高nibble优先输出正确；
+3. turnaround固定1个clk_i周期；
+4. 四种命令帧格式正确处理；
 coverage check点：
-对STATUS和LAST_ERR寄存器状态收集功能覆盖率</t>
+对帧类型和lane模式组合收集功能覆盖率。</t>
         </is>
       </c>
       <c r="D9" s="14" t="n"/>
@@ -2897,33 +2934,31 @@
       </c>
       <c r="B10" s="16" t="inlineStr">
         <is>
-          <t>test_error_handling</t>
+          <t>test_opcode_decode</t>
         </is>
       </c>
       <c r="C10" s="3" t="inlineStr">
         <is>
-          <t>TC场景：测试异常处理功能
-配置条件：
-1. test_mode_i=1
-2. 通过WR_CSR(opcode=0x10, addr=0x04, wdata=0x00000001)设置CTRL.EN=1
-其它：以上测试过程中，AHB总线正常
+          <t>配置条件：
+1. 模块解复位，test_mode_i=1；
+2. 通过WR_CSR(opcode=0x10)配置CTRL.EN=1；
 输入激励：
-1. 发送非法opcode(0x00/0xFF)验证BAD_OPCODE(0x01)
-2. 访问非法CSR地址(如0x10)验证BAD_REG(0x02)
-3. 发送非4Byte对齐地址(如0x00001001)验证ALIGN_ERR(0x03)
-4. 设置CTRL.EN=0后发送命令验证DISABLED(0x04)
-5. 设置test_mode_i=0后发送命令验证NOT_IN_TEST(0x05)
-6. 提前拉高pcs_n_i验证FRAME_ERR(0x06)
-7. 触发hresp_i=1验证AHB_ERR(0x07)
-8. 模拟AHB超时验证TIMEOUT(0x08)
+1. 发送opcode=0x10(WR_CSR)命令，验证帧长和任务类型；
+2. 发送opcode=0x11(RD_CSR)命令，验证帧长和任务类型；
+3. 发送opcode=0x20(AHB_WR32)命令，验证帧长和任务类型；
+4. 发送opcode=0x21(AHB_RD32)命令，验证帧长和任务类型；
+5. 发送opcode=0x00（非法），检查错误响应；
+6. 发送opcode=0xFF（非法），检查错误响应；
+7. 发送opcode=0x30（未定义），检查错误响应；
 期望结果：
-1. 各类错误正确检测
-2. 返回确定性状态码
-3. LAST_ERR更新正确
-4. 在发起AHB访问前完成前置错误收敛
-5. 响应帧包含正确状态码
+1. opcode=0x10：帧长48bit，任务类型CSR写；
+2. opcode=0x11：帧长16bit，任务类型CSR读；
+3. opcode=0x20：帧长72bit，任务类型AHB写；
+4. opcode=0x21：帧长40bit，任务类型AHB读；
+5. 非法opcode返回STS_BAD_OPCODE(0x01)；
+6. 前端在收满8bit opcode后正确确定期望帧长；
 coverage check点：
-对8类错误码收集功能覆盖率</t>
+对opcode值(0x10/0x11/0x20/0x21/非法值)收集功能覆盖率。</t>
         </is>
       </c>
       <c r="D10" s="14" t="n"/>
@@ -2936,29 +2971,29 @@
       </c>
       <c r="B11" s="16" t="inlineStr">
         <is>
-          <t>test_lowpower</t>
+          <t>test_config_register</t>
         </is>
       </c>
       <c r="C11" s="3" t="inlineStr">
         <is>
-          <t>TC场景：测试低功耗功能
-配置条件：
-1. 模块处于空闲态（test_mode_i=0或无有效任务）
-其它：以上测试过程中，AHB总线空闲
+          <t>配置条件：
+1. 模块解复位，test_mode_i=1；
 输入激励：
-1. 保持pcs_n_i=1验证接收/发送移位寄存器不翻转
-2. 模拟AHB等待态验证超时计数器仅在WAIT_AHB状态工作
-3. 设置test_mode_i=0验证AHB输出保持IDLE
-4. 切换到工作态验证关键寄存器翻转
-5. 监测状态机状态变化
+1. 通过WR_CSR(opcode=0x10)写入CTRL.EN=1，验证模块使能；
+2. 发送AHB_RD32命令验证功能正常；
+3. 通过WR_CSR写入CTRL.EN=0，验证模块禁用；
+4. 发送AHB_RD32命令验证返回STS_DISABLED(0x04)；
+5. 通过WR_CSR写入CTRL.LANE_MODE=2'b00，验证1-bit模式；
+6. 通过WR_CSR写入CTRL.LANE_MODE=2'b01，验证4-bit模式；
+7. 通过WR_CSR写入CTRL.SOFT_RST=1，验证软复位；
+8. 检查软复位后协议上下文清零，LANE_MODE恢复默认；
 期望结果：
-1. 空闲态接收/发送移位寄存器不更新
-2. 超时计数器仅在相关状态工作
-3. test_mode_i=0时htrans_o=IDLE
-4. 无有效任务时AHB输出保持IDLE
-5. 功耗测试通过
+1. CTRL.EN=1使能模块，EN=0禁用模块；
+2. LANE_MODE=00切换到1-bit模式，01切换到4-bit模式；
+3. SOFT_RST=1触发软复位，协议上下文清零；
+4. 配置写入后在下一个clk_i上升沿生效；
 coverage check点：
-对空闲态和工作态转换收集功能覆盖率</t>
+对CTRL寄存器字段(EN/LANE_MODE/SOFT_RST)和配置值组合收集功能覆盖率。</t>
         </is>
       </c>
       <c r="D11" s="14" t="n"/>
@@ -2971,112 +3006,471 @@
       </c>
       <c r="B12" s="16" t="inlineStr">
         <is>
+          <t>test_status_polling</t>
+        </is>
+      </c>
+      <c r="C12" s="3" t="inlineStr">
+        <is>
+          <t>配置条件：
+1. 模块解复位，test_mode_i=1；
+2. 通过WR_CSR(opcode=0x10)配置CTRL.EN=1；
+输入激励：
+1. 发送AHB_WR32命令，命令执行期间通过RD_CSR(opcode=0x11)读取STATUS检查busy位；
+2. 触发BAD_OPCODE错误（发送opcode=0x00）；
+3. 通过RD_CSR读取STATUS检查错误标志；
+4. 通过RD_CSR读取LAST_ERR检查错误码=0x01；
+5. 触发另一个错误（ALIGN_ERR）；
+6. 通过RD_CSR读取LAST_ERR检查错误码更新为0x03；
+7. 执行成功命令；
+8. 通过RD_CSR读取LAST_ERR检查值不变；
+期望结果：
+1. STATUS.busy位在命令执行期间为1，完成后为0；
+2. 错误发生时STATUS错误标志置位；
+3. LAST_ERR记录最近错误码，新错误覆盖旧值；
+4. 成功命令不更新LAST_ERR；
+5. MVP版本无中断输出，所有状态通过轮询获取；
+coverage check点：
+直接用例覆盖，不收功能覆盖率。</t>
+        </is>
+      </c>
+      <c r="D12" s="14" t="n"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="16" t="inlineStr">
+        <is>
+          <t>TC_011</t>
+        </is>
+      </c>
+      <c r="B13" s="16" t="inlineStr">
+        <is>
+          <t>test_bad_opcode</t>
+        </is>
+      </c>
+      <c r="C13" s="3" t="inlineStr">
+        <is>
+          <t>配置条件：
+1. 模块解复位，test_mode_i=1；
+2. 通过WR_CSR(opcode=0x10)配置CTRL.EN=1；
+输入激励：
+1. 发送opcode=0x00，检查响应status_code；
+2. 发送opcode=0xFF，检查响应status_code；
+3. 发送opcode=0x12（未定义），检查响应status_code；
+4. 发送opcode=0x30（未定义），检查响应status_code；
+5. 每次错误后通过RD_CSR读取LAST_ERR验证错误码；
+期望结果：
+1. 所有非法opcode返回STS_BAD_OPCODE(0x01)；
+2. LAST_ERR寄存器更新为0x01；
+3. 前端在收满8bit opcode后立即检测错误，不等待后续数据；
+coverage check点：
+对非法opcode值(0x00/0xFF/0x12/0x30等)收集功能覆盖率。</t>
+        </is>
+      </c>
+      <c r="D13" s="14" t="n"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="16" t="inlineStr">
+        <is>
+          <t>TC_012</t>
+        </is>
+      </c>
+      <c r="B14" s="16" t="inlineStr">
+        <is>
+          <t>test_bad_reg</t>
+        </is>
+      </c>
+      <c r="C14" s="3" t="inlineStr">
+        <is>
+          <t>配置条件：
+1. 模块解复位，test_mode_i=1；
+2. 通过WR_CSR(opcode=0x10)配置CTRL.EN=1；
+输入激励：
+1. 发送WR_CSR(opcode=0x10)命令，访问未定义的CSR地址（如addr=0xFF）；
+2. 检查响应status_code；
+3. 发送RD_CSR(opcode=0x11)命令，访问未定义的CSR地址；
+4. 检查响应status_code；
+5. 通过RD_CSR读取LAST_ERR验证错误码；
+期望结果：
+1. 访问未定义CSR地址返回STS_BAD_REG(0x02)；
+2. LAST_ERR寄存器更新为0x02；
+coverage check点：
+直接用例覆盖，不收功能覆盖率。</t>
+        </is>
+      </c>
+      <c r="D14" s="14" t="n"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="16" t="inlineStr">
+        <is>
+          <t>TC_013</t>
+        </is>
+      </c>
+      <c r="B15" s="16" t="inlineStr">
+        <is>
+          <t>test_align_error</t>
+        </is>
+      </c>
+      <c r="C15" s="3" t="inlineStr">
+        <is>
+          <t>配置条件：
+1. 模块解复位，test_mode_i=1；
+2. 通过WR_CSR(opcode=0x10)配置CTRL.EN=1；
+输入激励：
+1. 发送AHB_WR32(opcode=0x20)命令，addr[1:0]=2'b01（非4Byte对齐）；
+2. 检查响应status_code；
+3. 发送AHB_RD32(opcode=0x21)命令，addr[1:0]=2'b10；
+4. 检查响应status_code；
+5. 发送AHB_WR32命令，addr[1:0]=2'b11；
+6. 检查响应status_code；
+7. 通过RD_CSR读取LAST_ERR验证错误码；
+期望结果：
+1. addr[1:0]!=2'b00时返回STS_ALIGN_ERR(0x03)；
+2. LAST_ERR寄存器更新为0x03；
+3. 不发起AHB访问；
+coverage check点：
+对非对齐地址值(01/10/11)收集功能覆盖率。</t>
+        </is>
+      </c>
+      <c r="D15" s="14" t="n"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="16" t="inlineStr">
+        <is>
+          <t>TC_014</t>
+        </is>
+      </c>
+      <c r="B16" s="16" t="inlineStr">
+        <is>
+          <t>test_disabled_error</t>
+        </is>
+      </c>
+      <c r="C16" s="3" t="inlineStr">
+        <is>
+          <t>配置条件：
+1. 模块解复位，test_mode_i=1；
+2. 通过WR_CSR(opcode=0x10)配置CTRL.EN=0；
+输入激励：
+1. 发送AHB_WR32(opcode=0x20)命令，检查响应status_code；
+2. 发送AHB_RD32(opcode=0x21)命令，检查响应status_code；
+3. 通过RD_CSR读取LAST_ERR验证错误码；
+4. 通过WR_CSR配置CTRL.EN=1；
+5. 发送相同命令验证正常执行；
+期望结果：
+1. CTRL.EN=0时，AHB命令返回STS_DISABLED(0x04)；
+2. LAST_ERR寄存器更新为0x04；
+3. CTRL.EN=1后命令正常执行；
+coverage check点：
+直接用例覆盖，不收功能覆盖率。</t>
+        </is>
+      </c>
+      <c r="D16" s="14" t="n"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="16" t="inlineStr">
+        <is>
+          <t>TC_015</t>
+        </is>
+      </c>
+      <c r="B17" s="16" t="inlineStr">
+        <is>
+          <t>test_not_in_test_error</t>
+        </is>
+      </c>
+      <c r="C17" s="3" t="inlineStr">
+        <is>
+          <t>配置条件：
+1. 模块解复位，test_mode_i=0；
+输入激励：
+1. 发送WR_CSR(opcode=0x10)命令，检查响应status_code；
+2. 发送RD_CSR(opcode=0x11)命令，检查响应status_code；
+3. 发送AHB_WR32(opcode=0x20)命令，检查响应status_code；
+4. 发送AHB_RD32(opcode=0x21)命令，检查响应status_code；
+5. 通过RD_CSR读取LAST_ERR验证错误码；
+6. 设置test_mode_i=1；
+7. 发送相同命令验证正常执行；
+期望结果：
+1. test_mode_i=0时，任何命令返回STS_NOT_IN_TEST(0x05)；
+2. LAST_ERR寄存器更新为0x05；
+3. test_mode_i=1后命令正常执行；
+coverage check点：
+直接用例覆盖，不收功能覆盖率。</t>
+        </is>
+      </c>
+      <c r="D17" s="14" t="n"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="16" t="inlineStr">
+        <is>
+          <t>TC_016</t>
+        </is>
+      </c>
+      <c r="B18" s="16" t="inlineStr">
+        <is>
+          <t>test_frame_error</t>
+        </is>
+      </c>
+      <c r="C18" s="3" t="inlineStr">
+        <is>
+          <t>配置条件：
+1. 模块解复位，test_mode_i=1；
+2. 通过WR_CSR(opcode=0x10)配置CTRL.EN=1；
+输入激励：
+1. 开始发送AHB_WR32命令，在opcode发送完成后立即拉高pcs_n_i（提前结束）；
+2. 检查响应status_code；
+3. 通过RD_CSR读取LAST_ERR验证错误码；
+4. 发送完整命令验证模块恢复正常；
+期望结果：
+1. pcs_n_i提前拉高返回STS_FRAME_ERR(0x06)；
+2. LAST_ERR寄存器更新为0x06；
+3. 后续命令正常执行；
+coverage check点：
+直接用例覆盖，不收功能覆盖率。</t>
+        </is>
+      </c>
+      <c r="D18" s="14" t="n"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="4" t="inlineStr">
+        <is>
+          <t>TC_017</t>
+        </is>
+      </c>
+      <c r="B19" s="4" t="inlineStr">
+        <is>
+          <t>test_ahb_error</t>
+        </is>
+      </c>
+      <c r="C19" s="3" t="inlineStr">
+        <is>
+          <t>配置条件：
+1. 模块解复位，test_mode_i=1；
+2. 通过WR_CSR(opcode=0x10)配置CTRL.EN=1；
+3. AHB slave配置为返回ERROR response；
+输入激励：
+1. 发送AHB_WR32(opcode=0x20)命令；
+2. AHB slave在响应时返回hresp_i=1（ERROR）；
+3. 检查响应status_code；
+4. 通过RD_CSR读取LAST_ERR验证错误码；
+5. AHB slave恢复正常，发送命令验证模块恢复正常；
+期望结果：
+1. hresp_i=1时返回STS_AHB_ERR(0x07)；
+2. LAST_ERR寄存器更新为0x07；
+3. 后续命令正常执行；
+coverage check点：
+直接用例覆盖，不收功能覆盖率。</t>
+        </is>
+      </c>
+      <c r="D19" s="4" t="n"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="4" t="inlineStr">
+        <is>
+          <t>TC_018</t>
+        </is>
+      </c>
+      <c r="B20" s="4" t="inlineStr">
+        <is>
+          <t>test_timeout_error</t>
+        </is>
+      </c>
+      <c r="C20" s="3" t="inlineStr">
+        <is>
+          <t>配置条件：
+1. 模块解复位，test_mode_i=1；
+2. 通过WR_CSR(opcode=0x10)配置CTRL.EN=1；
+3. AHB slave配置为长时间不响应；
+输入激励：
+1. 发送AHB_RD32(opcode=0x21)命令；
+2. AHB slave保持hready_i=0超过超时阈值；
+3. 检查响应status_code；
+4. 通过RD_CSR读取LAST_ERR验证错误码；
+5. AHB slave恢复正常，发送命令验证模块恢复正常；
+期望结果：
+1. AHB超时后返回STS_TIMEOUT(0x08)；
+2. LAST_ERR寄存器更新为0x08；
+3. 后续命令正常执行；
+coverage check点：
+直接用例覆盖，不收功能覆盖率。</t>
+        </is>
+      </c>
+      <c r="D20" s="4" t="n"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="4" t="inlineStr">
+        <is>
+          <t>TC_019</t>
+        </is>
+      </c>
+      <c r="B21" s="4" t="inlineStr">
+        <is>
+          <t>test_lowpower</t>
+        </is>
+      </c>
+      <c r="C21" s="3" t="inlineStr">
+        <is>
+          <t>配置条件：
+1. 模块解复位；
+输入激励：
+1. 设置test_mode_i=0，保持pcs_n_i=1；
+2. 观察接收/发送移位寄存器是否更新；
+3. 观察AHB输出htrans_o是否为IDLE；
+4. 设置test_mode_i=1，配置CTRL.EN=1；
+5. 发送命令，观察工作态关键寄存器翻转；
+6. 命令完成后，观察空闲态寄存器保持；
+期望结果：
+1. 空闲态（test_mode_i=0或pcs_n_i=1）：接收/发送移位寄存器不更新；
+2. test_mode_i=0时，AHB输出保持IDLE（htrans_o=2'b00）；
+3. 工作态：关键寄存器正常翻转；
+4. 低功耗设计目标满足；
+coverage check点：
+直接用例覆盖，不收功能覆盖率。</t>
+        </is>
+      </c>
+      <c r="D21" s="4" t="n"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="4" t="inlineStr">
+        <is>
+          <t>TC_020</t>
+        </is>
+      </c>
+      <c r="B22" s="4" t="inlineStr">
+        <is>
           <t>test_performance</t>
         </is>
       </c>
-      <c r="C12" s="3" t="inlineStr">
-        <is>
-          <t>TC场景：测试性能指标和AHB接口功能
-配置条件：
-1. test_mode_i=1
-2. 通过WR_CSR(opcode=0x10, addr=0x04, wdata=0x00000001)设置CTRL.EN=1
-3. 配置clk_i=100MHz
-其它：以上测试过程中，AHB总线响应正常
+      <c r="C22" s="3" t="inlineStr">
+        <is>
+          <t>配置条件：
+1. 配置clk_i=100MHz；
+2. 模块解复位，test_mode_i=1；
+3. 通过WR_CSR(opcode=0x10)配置CTRL.EN=1；
 输入激励：
-1. 在1-bit模式下连续执行AHB_RD32/AHB_WR32命令，计算端到端延时和吞吐率
-2. 在4-bit模式下执行相同测试
-3. 验证原始链路线速：1-bit模式12.5MB/s，4-bit模式50MB/s
-4. 验证AHB接口32bit字访问和4Byte对齐约束
-5. 采集状态机状态、opcode、addr、wdata、rdata、status_code
-6. 采集rx/tx计数、pcs_n_i、pdi_i、pdo_o、pdo_oe_o
-7. 验证AHB-Lite Master接口信号时序
+1. 配置LANE_MODE=2'b00（1-bit模式）；
+2. 连续发送100次AHB_RD32/AHB_WR32命令，记录端到端延时；
+3. 计算吞吐率；
+4. 配置LANE_MODE=2'b01（4-bit模式）；
+5. 连续发送100次AHB_RD32/AHB_WR32命令，记录端到端延时；
+6. 计算吞吐率；
+7. 检查AHB接口hsize_o固定为WORD，haddr_o[1:0]=2'b00；
 期望结果：
-1. 目标频率100MHz稳定工作
-2. 延时符合预期（约23~24 cycles）
-3. 吞吐率达标
-4. AHB访问约束满足
-5. 所有调试可观测点可采集
-6. AHB-Lite接口符合规范：
-   - htrans_o仅IDLE/NONSEQ
-   - hsize_o固定WORD
-   - hburst_o固定SINGLE
+1. 目标频率100MHz稳定工作；
+2. 端到端延时约23~24 cycles；
+3. 1-bit模式吞吐率接近12.5MB/s；
+4. 4-bit模式吞吐率接近50MB/s；
+5. AHB接口32bit字访问，地址4Byte对齐；
 coverage check点：
-对性能指标和AHB信号收集功能覆盖率</t>
-        </is>
-      </c>
-      <c r="D12" s="14" t="n"/>
-    </row>
-    <row r="13">
-      <c r="A13" s="16" t="n"/>
-      <c r="B13" s="16" t="n"/>
-      <c r="C13" s="3" t="n"/>
-      <c r="D13" s="14" t="n"/>
-    </row>
-    <row r="14">
-      <c r="A14" s="16" t="n"/>
-      <c r="B14" s="16" t="n"/>
-      <c r="C14" s="3" t="n"/>
-      <c r="D14" s="14" t="n"/>
-    </row>
-    <row r="15">
-      <c r="A15" s="16" t="n"/>
-      <c r="B15" s="16" t="n"/>
-      <c r="C15" s="3" t="n"/>
-      <c r="D15" s="14" t="n"/>
-    </row>
-    <row r="16">
-      <c r="A16" s="16" t="n"/>
-      <c r="B16" s="16" t="n"/>
-      <c r="C16" s="3" t="n"/>
-      <c r="D16" s="14" t="n"/>
-    </row>
-    <row r="17">
-      <c r="A17" s="16" t="n"/>
-      <c r="B17" s="16" t="n"/>
-      <c r="C17" s="3" t="n"/>
-      <c r="D17" s="14" t="n"/>
-    </row>
-    <row r="18">
-      <c r="A18" s="16" t="n"/>
-      <c r="B18" s="16" t="n"/>
-      <c r="C18" s="3" t="n"/>
-      <c r="D18" s="14" t="n"/>
-    </row>
-    <row r="19">
-      <c r="A19" s="4" t="n"/>
-      <c r="B19" s="4" t="n"/>
-      <c r="C19" s="3" t="n"/>
-      <c r="D19" s="4" t="n"/>
-    </row>
-    <row r="20">
-      <c r="A20" s="4" t="n"/>
-      <c r="B20" s="4" t="n"/>
-      <c r="C20" s="3" t="n"/>
-      <c r="D20" s="4" t="n"/>
-    </row>
-    <row r="21">
-      <c r="A21" s="4" t="n"/>
-      <c r="B21" s="4" t="n"/>
-      <c r="C21" s="3" t="n"/>
-      <c r="D21" s="4" t="n"/>
-    </row>
-    <row r="22">
-      <c r="A22" s="4" t="n"/>
-      <c r="B22" s="4" t="n"/>
-      <c r="C22" s="3" t="n"/>
+对lane模式和命令类型组合收集功能覆盖率，记录性能指标。</t>
+        </is>
+      </c>
       <c r="D22" s="4" t="n"/>
     </row>
     <row r="23">
-      <c r="A23" s="4" t="n"/>
-      <c r="B23" s="4" t="n"/>
-      <c r="C23" s="3" t="n"/>
+      <c r="A23" s="4" t="inlineStr">
+        <is>
+          <t>TC_021</t>
+        </is>
+      </c>
+      <c r="B23" s="4" t="inlineStr">
+        <is>
+          <t>test_debug_observability</t>
+        </is>
+      </c>
+      <c r="C23" s="3" t="inlineStr">
+        <is>
+          <t>配置条件：
+1. 模块解复位，test_mode_i=1；
+2. 通过WR_CSR(opcode=0x10)配置CTRL.EN=1；
+3. 仿真环境，启用波形记录；
+输入激励：
+1. 发送多种命令序列（WR_CSR/RD_CSR/AHB_WR32/AHB_RD32）；
+2. 采集内部信号：fsm_state、opcode、addr、wdata、rdata、status_code；
+3. 采集rx/tx计数器；
+4. 采集接口信号：pcs_n_i、pdi_i、pdo_o、pdo_oe_o；
+5. 验证所有调试可观测点可访问；
+期望结果：
+1. 状态机状态可观测；
+2. opcode/addr/wdata/rdata/status_code可观测；
+3. rx/tx计数器可观测；
+4. 接口信号可观测；
+5. 便于联调、波形定位和故障复现；
+coverage check点：
+直接用例覆盖，不收功能覆盖率。</t>
+        </is>
+      </c>
       <c r="D23" s="4" t="n"/>
     </row>
     <row r="24">
-      <c r="A24" s="4" t="n"/>
-      <c r="B24" s="4" t="n"/>
-      <c r="C24" s="3" t="n"/>
+      <c r="A24" s="4" t="inlineStr">
+        <is>
+          <t>TC_022</t>
+        </is>
+      </c>
+      <c r="B24" s="4" t="inlineStr">
+        <is>
+          <t>test_memory_map</t>
+        </is>
+      </c>
+      <c r="C24" s="3" t="inlineStr">
+        <is>
+          <t>配置条件：
+1. 模块解复位，test_mode_i=1；
+2. 通过WR_CSR(opcode=0x10)配置CTRL.EN=1；
+输入激励：
+1. 通过RD_CSR(opcode=0x11)访问VERSION寄存器；
+2. 通过WR_CSR/RD_CSR访问CTRL寄存器；
+3. 通过RD_CSR访问STATUS/LAST_ERR寄存器；
+4. 发送AHB_WR32命令访问SoC memory-mapped地址；
+5. 发送AHB_RD32命令访问SoC memory-mapped地址；
+6. 验证模块CSR不出现在SoC AHB memory map中；
+7. 验证AHB Master访问使用32bit地址空间；
+期望结果：
+1. CSR通过协议命令正确访问；
+2. AHB Master正确访问SoC memory-mapped地址；
+3. 模块CSR不进入SoC AHB memory map；
+4. AHB Master使用32bit地址空间和word访问粒度；
+coverage check点：
+对CSR寄存器和AHB地址范围收集功能覆盖率。</t>
+        </is>
+      </c>
       <c r="D24" s="4" t="n"/>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>TC_023</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>test_ahb_interface</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>配置条件：
+1. 模块解复位，test_mode_i=1；
+2. 通过WR_CSR(opcode=0x10)配置CTRL.EN=1；
+3. AHB总线空闲；
+输入激励：
+1. 发送AHB_WR32(opcode=0x20)命令；
+2. 检查AHB输出：haddr_o、hwrite_o=1、htrans_o=NONSEQ、hsize_o=WORD、hburst_o=SINGLE；
+3. 检查hwdata_o在数据相输出正确；
+4. 发送AHB_RD32(opcode=0x21)命令；
+5. 检查AHB输出：hwrite_o=0、htrans_o=NONSEQ；
+6. 检查hrdata_i正确接收；
+7. 测试hready_i=0等待场景；
+8. 测试hresp_i=1错误场景；
+期望结果：
+1. AHB-Lite Master信号符合规范；
+2. htrans_o仅输出IDLE(2'b00)或NONSEQ(2'b10)；
+3. hsize_o固定为WORD(3'b010)；
+4. hburst_o固定为SINGLE(3'b000)；
+5. 地址相和数据相时序正确；
+6. hready_i/hresp_i响应正确处理；
+coverage check点：
+对AHB命令类型(WR/RD)和响应场景(normal/wait/error)收集功能覆盖率。</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="1">

</xml_diff>